<commit_message>
- implement stat_fun = min & max - add all of the stat_fun possibilities to one question in mapping file - add snapshot test for all these `stat_fun`s
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4360B0C8-1794-4A7E-89D0-76A472F232C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A07552D-5E30-4735-851E-100862A35515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -951,9 +951,6 @@
     <t>3. Wie verteilten sich die Studien prozentual auf die einzelnen Arten?</t>
   </si>
   <si>
-    <t>S1E2</t>
-  </si>
-  <si>
     <t>5. Was lief besonders gut in den Projekten?</t>
   </si>
   <si>
@@ -1024,6 +1021,9 @@
   </si>
   <si>
     <t>kregio</t>
+  </si>
+  <si>
+    <t>S1E2M0P250T0I0A0</t>
   </si>
 </sst>
 </file>
@@ -2165,7 +2165,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E15" s="10"/>
     </row>
@@ -2228,10 +2228,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="B23" s="33" t="s">
         <v>277</v>
-      </c>
-      <c r="B23" s="33" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2881,7 +2881,7 @@
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>149</v>
@@ -2893,7 +2893,7 @@
         <v>151</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F5" s="29" t="str">
         <f>E5</f>
@@ -6515,13 +6515,13 @@
         <v>223</v>
       </c>
       <c r="C1" s="28" t="s">
+        <v>269</v>
+      </c>
+      <c r="D1" s="28" t="s">
         <v>270</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="E1" s="28" t="s">
         <v>271</v>
-      </c>
-      <c r="E1" s="28" t="s">
-        <v>272</v>
       </c>
       <c r="F1" s="28" t="s">
         <v>224</v>
@@ -6551,10 +6551,10 @@
         <v>244</v>
       </c>
       <c r="O1" s="28" t="s">
+        <v>272</v>
+      </c>
+      <c r="P1" s="28" t="s">
         <v>273</v>
-      </c>
-      <c r="P1" s="28" t="s">
-        <v>274</v>
       </c>
       <c r="Q1" s="28" t="s">
         <v>245</v>
@@ -6581,7 +6581,7 @@
         <v>202</v>
       </c>
       <c r="Y1" s="28" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Z1" s="28" t="s">
         <v>232</v>
@@ -6593,7 +6593,7 @@
         <v>234</v>
       </c>
       <c r="AC1" s="28" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="AD1" s="28" t="s">
         <v>248</v>
@@ -6620,13 +6620,13 @@
         <v>236</v>
       </c>
       <c r="AL1" s="28" t="s">
+        <v>260</v>
+      </c>
+      <c r="AM1" s="28" t="s">
         <v>261</v>
       </c>
-      <c r="AM1" s="28" t="s">
+      <c r="AN1" s="28" t="s">
         <v>262</v>
-      </c>
-      <c r="AN1" s="28" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
@@ -6765,7 +6765,7 @@
         <v>237</v>
       </c>
       <c r="G5" s="31" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H5" s="31" t="s">
         <v>251</v>
@@ -6819,10 +6819,10 @@
         <v>253</v>
       </c>
       <c r="G6" s="31" t="s">
+        <v>265</v>
+      </c>
+      <c r="H6" s="31" t="s">
         <v>266</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>267</v>
       </c>
       <c r="I6" s="31"/>
       <c r="J6" s="31"/>
@@ -6873,10 +6873,10 @@
         <v>238</v>
       </c>
       <c r="G7" s="31" t="s">
+        <v>267</v>
+      </c>
+      <c r="H7" s="31" t="s">
         <v>268</v>
-      </c>
-      <c r="H7" s="31" t="s">
-        <v>269</v>
       </c>
       <c r="I7" s="31"/>
       <c r="J7" s="31"/>
@@ -6884,7 +6884,7 @@
       <c r="L7" s="31"/>
       <c r="M7" s="31"/>
       <c r="N7" s="31" t="s">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="O7" s="25"/>
       <c r="P7" s="31"/>
@@ -6920,16 +6920,16 @@
         <v>Q5</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
       <c r="F8" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G8" s="31" t="s">
         <v>257</v>
-      </c>
-      <c r="G8" s="31" t="s">
-        <v>258</v>
       </c>
       <c r="H8" s="31" t="s">
         <v>251</v>
@@ -6943,7 +6943,7 @@
       <c r="O8" s="25"/>
       <c r="P8" s="31"/>
       <c r="Q8" s="31" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="R8" s="31"/>
       <c r="S8" s="31"/>
@@ -32714,14 +32714,12 @@
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A8">
+    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="17"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A9:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A8">
-    <cfRule type="duplicateValues" dxfId="1" priority="16"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A8">
-    <cfRule type="duplicateValues" dxfId="0" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
add test for summary of medians
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A07552D-5E30-4735-851E-100862A35515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D5DA3A-2696-42FA-AA08-8AC796F8721F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -184,7 +184,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="283">
   <si>
     <t>Make script</t>
   </si>
@@ -1024,6 +1024,15 @@
   </si>
   <si>
     <t>S1E2M0P250T0I0A0</t>
+  </si>
+  <si>
+    <t>q3a q3b</t>
+  </si>
+  <si>
+    <t>median</t>
+  </si>
+  <si>
+    <t>Summary of Medians</t>
   </si>
 </sst>
 </file>
@@ -6484,7 +6493,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI668"/>
+  <dimension ref="A1:AMI669"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -6806,7 +6815,7 @@
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="str">
-        <f t="shared" ref="A6:A8" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
+        <f t="shared" ref="A6:A9" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
         <v>Q2</v>
       </c>
       <c r="B6" s="30" t="s">
@@ -6900,7 +6909,9 @@
       <c r="Z7" s="25"/>
       <c r="AA7" s="25"/>
       <c r="AB7" s="25"/>
-      <c r="AC7" s="25"/>
+      <c r="AC7" s="25">
+        <v>0</v>
+      </c>
       <c r="AD7" s="14"/>
       <c r="AE7" s="25"/>
       <c r="AF7" s="25"/>
@@ -6916,23 +6927,23 @@
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5</v>
+        <f t="shared" ref="A8" si="1">"Q"&amp;LEFT(B8,FIND(".",B8)-1)</f>
+        <v>Q3</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
       <c r="F8" s="31" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>257</v>
+        <v>280</v>
       </c>
       <c r="H8" s="31" t="s">
-        <v>251</v>
+        <v>268</v>
       </c>
       <c r="I8" s="31"/>
       <c r="J8" s="31"/>
@@ -6942,14 +6953,14 @@
       <c r="N8" s="31"/>
       <c r="O8" s="25"/>
       <c r="P8" s="31"/>
-      <c r="Q8" s="31" t="s">
-        <v>258</v>
-      </c>
+      <c r="Q8" s="31"/>
       <c r="R8" s="31"/>
       <c r="S8" s="31"/>
       <c r="T8" s="31"/>
       <c r="U8" s="25"/>
-      <c r="V8" s="25"/>
+      <c r="V8" s="25">
+        <v>0</v>
+      </c>
       <c r="W8" s="25"/>
       <c r="X8" s="25"/>
       <c r="Y8" s="25"/>
@@ -6957,11 +6968,15 @@
       <c r="AA8" s="25"/>
       <c r="AB8" s="25"/>
       <c r="AC8" s="25"/>
-      <c r="AD8" s="25"/>
+      <c r="AD8" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="AE8" s="25"/>
       <c r="AF8" s="25"/>
       <c r="AG8" s="25"/>
-      <c r="AH8" s="25"/>
+      <c r="AH8" s="25" t="s">
+        <v>282</v>
+      </c>
       <c r="AI8" s="25"/>
       <c r="AJ8" s="25"/>
       <c r="AK8" s="25"/>
@@ -6971,22 +6986,39 @@
       <c r="AO8" s="26"/>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C9" s="22"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
+      <c r="A9" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>Q5</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="H9" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
       <c r="O9" s="25"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="25"/>
-      <c r="R9" s="25"/>
-      <c r="S9" s="25"/>
-      <c r="T9" s="25"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R9" s="31"/>
+      <c r="S9" s="31"/>
+      <c r="T9" s="31"/>
       <c r="U9" s="25"/>
       <c r="V9" s="25"/>
       <c r="W9" s="25"/>
@@ -32710,15 +32742,54 @@
       <c r="AN668" s="25"/>
       <c r="AO668" s="26"/>
     </row>
+    <row r="669" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C669" s="22"/>
+      <c r="F669" s="25"/>
+      <c r="G669" s="25"/>
+      <c r="H669" s="25"/>
+      <c r="I669" s="25"/>
+      <c r="J669" s="25"/>
+      <c r="K669" s="25"/>
+      <c r="L669" s="25"/>
+      <c r="M669" s="25"/>
+      <c r="N669" s="25"/>
+      <c r="O669" s="25"/>
+      <c r="P669" s="25"/>
+      <c r="Q669" s="25"/>
+      <c r="R669" s="25"/>
+      <c r="S669" s="25"/>
+      <c r="T669" s="25"/>
+      <c r="U669" s="25"/>
+      <c r="V669" s="25"/>
+      <c r="W669" s="25"/>
+      <c r="X669" s="25"/>
+      <c r="Y669" s="25"/>
+      <c r="Z669" s="25"/>
+      <c r="AA669" s="25"/>
+      <c r="AB669" s="25"/>
+      <c r="AC669" s="25"/>
+      <c r="AD669" s="25"/>
+      <c r="AE669" s="25"/>
+      <c r="AF669" s="25"/>
+      <c r="AG669" s="25"/>
+      <c r="AH669" s="25"/>
+      <c r="AI669" s="25"/>
+      <c r="AJ669" s="25"/>
+      <c r="AK669" s="25"/>
+      <c r="AL669" s="25"/>
+      <c r="AM669" s="25"/>
+      <c r="AN669" s="25"/>
+      <c r="AO669" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A8">
+  <conditionalFormatting sqref="A5:A9">
     <cfRule type="duplicateValues" dxfId="2" priority="16"/>
     <cfRule type="duplicateValues" dxfId="1" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A9:A1048576 A2:A4">
+  <conditionalFormatting sqref="A10:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
add possibility to calculate weighted tables: - add test for weighted summary of means
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D5DA3A-2696-42FA-AA08-8AC796F8721F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9A26F4-E944-4330-98B5-886C40579803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -184,7 +184,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="283">
   <si>
     <t>Make script</t>
   </si>
@@ -6493,7 +6493,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI669"/>
+  <dimension ref="A1:AMI670"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -6815,7 +6815,7 @@
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="str">
-        <f t="shared" ref="A6:A9" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
+        <f t="shared" ref="A6:A10" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
         <v>Q2</v>
       </c>
       <c r="B6" s="30" t="s">
@@ -6987,23 +6987,23 @@
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5</v>
+        <f t="shared" ref="A9" si="2">"Q"&amp;LEFT(B9,FIND(".",B9)-1)</f>
+        <v>Q3</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
       <c r="F9" s="31" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>257</v>
+        <v>280</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>251</v>
+        <v>268</v>
       </c>
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
@@ -7013,14 +7013,14 @@
       <c r="N9" s="31"/>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
-      <c r="Q9" s="31" t="s">
-        <v>258</v>
-      </c>
+      <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
       <c r="S9" s="31"/>
       <c r="T9" s="31"/>
       <c r="U9" s="25"/>
-      <c r="V9" s="25"/>
+      <c r="V9" s="25">
+        <v>0</v>
+      </c>
       <c r="W9" s="25"/>
       <c r="X9" s="25"/>
       <c r="Y9" s="25"/>
@@ -7028,11 +7028,15 @@
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
       <c r="AC9" s="25"/>
-      <c r="AD9" s="25"/>
+      <c r="AD9" s="14"/>
       <c r="AE9" s="25"/>
-      <c r="AF9" s="25"/>
+      <c r="AF9" s="25" t="s">
+        <v>249</v>
+      </c>
       <c r="AG9" s="25"/>
-      <c r="AH9" s="25"/>
+      <c r="AH9" s="25" t="s">
+        <v>282</v>
+      </c>
       <c r="AI9" s="25"/>
       <c r="AJ9" s="25"/>
       <c r="AK9" s="25"/>
@@ -7042,22 +7046,39 @@
       <c r="AO9" s="26"/>
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C10" s="22"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="25"/>
-      <c r="L10" s="25"/>
-      <c r="M10" s="25"/>
-      <c r="N10" s="25"/>
+      <c r="A10" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>Q5</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="H10" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
       <c r="O10" s="25"/>
-      <c r="P10" s="25"/>
-      <c r="Q10" s="25"/>
-      <c r="R10" s="25"/>
-      <c r="S10" s="25"/>
-      <c r="T10" s="25"/>
+      <c r="P10" s="31"/>
+      <c r="Q10" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R10" s="31"/>
+      <c r="S10" s="31"/>
+      <c r="T10" s="31"/>
       <c r="U10" s="25"/>
       <c r="V10" s="25"/>
       <c r="W10" s="25"/>
@@ -32781,15 +32802,54 @@
       <c r="AN669" s="25"/>
       <c r="AO669" s="26"/>
     </row>
+    <row r="670" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C670" s="22"/>
+      <c r="F670" s="25"/>
+      <c r="G670" s="25"/>
+      <c r="H670" s="25"/>
+      <c r="I670" s="25"/>
+      <c r="J670" s="25"/>
+      <c r="K670" s="25"/>
+      <c r="L670" s="25"/>
+      <c r="M670" s="25"/>
+      <c r="N670" s="25"/>
+      <c r="O670" s="25"/>
+      <c r="P670" s="25"/>
+      <c r="Q670" s="25"/>
+      <c r="R670" s="25"/>
+      <c r="S670" s="25"/>
+      <c r="T670" s="25"/>
+      <c r="U670" s="25"/>
+      <c r="V670" s="25"/>
+      <c r="W670" s="25"/>
+      <c r="X670" s="25"/>
+      <c r="Y670" s="25"/>
+      <c r="Z670" s="25"/>
+      <c r="AA670" s="25"/>
+      <c r="AB670" s="25"/>
+      <c r="AC670" s="25"/>
+      <c r="AD670" s="25"/>
+      <c r="AE670" s="25"/>
+      <c r="AF670" s="25"/>
+      <c r="AG670" s="25"/>
+      <c r="AH670" s="25"/>
+      <c r="AI670" s="25"/>
+      <c r="AJ670" s="25"/>
+      <c r="AK670" s="25"/>
+      <c r="AL670" s="25"/>
+      <c r="AM670" s="25"/>
+      <c r="AN670" s="25"/>
+      <c r="AO670" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A9">
+  <conditionalFormatting sqref="A5:A10">
     <cfRule type="duplicateValues" dxfId="2" priority="16"/>
     <cfRule type="duplicateValues" dxfId="1" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A10:A1048576 A2:A4">
+  <conditionalFormatting sqref="A11:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
add snapshot test for weighted MetrMac table
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9A26F4-E944-4330-98B5-886C40579803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC07DEA4-ACF1-4ACF-B7D8-9A7FCCFB1883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7010,7 +7010,9 @@
       <c r="K9" s="31"/>
       <c r="L9" s="31"/>
       <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
+      <c r="N9" s="31" t="s">
+        <v>279</v>
+      </c>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
       <c r="Q9" s="31"/>
@@ -7018,9 +7020,7 @@
       <c r="S9" s="31"/>
       <c r="T9" s="31"/>
       <c r="U9" s="25"/>
-      <c r="V9" s="25">
-        <v>0</v>
-      </c>
+      <c r="V9" s="25"/>
       <c r="W9" s="25"/>
       <c r="X9" s="25"/>
       <c r="Y9" s="25"/>
@@ -7034,9 +7034,7 @@
         <v>249</v>
       </c>
       <c r="AG9" s="25"/>
-      <c r="AH9" s="25" t="s">
-        <v>282</v>
-      </c>
+      <c r="AH9" s="25"/>
       <c r="AI9" s="25"/>
       <c r="AJ9" s="25"/>
       <c r="AK9" s="25"/>
@@ -32845,12 +32843,12 @@
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A11:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A5:A10">
-    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="17"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A11:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="0" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="19"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
no idea what changed
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC07DEA4-ACF1-4ACF-B7D8-9A7FCCFB1883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4850C16-1E45-43E7-8515-92147D8E03CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7027,7 +7027,9 @@
       <c r="Z9" s="25"/>
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
-      <c r="AC9" s="25"/>
+      <c r="AC9" s="25">
+        <v>0</v>
+      </c>
       <c r="AD9" s="14"/>
       <c r="AE9" s="25"/>
       <c r="AF9" s="25" t="s">

</xml_diff>

<commit_message>
fix CatRec and add snapshot test for it
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4850C16-1E45-43E7-8515-92147D8E03CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC243E6-6CE9-48B5-A6E8-3647B70C25E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -184,7 +184,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="288">
   <si>
     <t>Make script</t>
   </si>
@@ -1034,6 +1034,21 @@
   <si>
     <t>Summary of Medians</t>
   </si>
+  <si>
+    <t xml:space="preserve">4. Wie häufig haben Sie einen Tabellenband in den letzten 12 Monaten erstellen lassen? </t>
+  </si>
+  <si>
+    <t>q4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1 THRU 2 = 1) (3 THRU 5 = 2) (6 THRU HI = 3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 '1-2mal' 2 '3-5mal' 3 '&gt;5mal' </t>
+  </si>
+  <si>
+    <t>S1E2M0</t>
+  </si>
 </sst>
 </file>
 
@@ -1283,7 +1298,27 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2375,22 +2410,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="7" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="6" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6493,7 +6528,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI670"/>
+  <dimension ref="A1:AMI671"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -6815,7 +6850,7 @@
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="str">
-        <f t="shared" ref="A6:A10" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
+        <f t="shared" ref="A6:A11" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
         <v>Q2</v>
       </c>
       <c r="B6" s="30" t="s">
@@ -6987,7 +7022,7 @@
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="str">
-        <f t="shared" ref="A9" si="2">"Q"&amp;LEFT(B9,FIND(".",B9)-1)</f>
+        <f t="shared" ref="A9:A10" si="2">"Q"&amp;LEFT(B9,FIND(".",B9)-1)</f>
         <v>Q3</v>
       </c>
       <c r="B9" s="30" t="s">
@@ -7047,35 +7082,39 @@
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5</v>
+        <f t="shared" si="2"/>
+        <v>Q4</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="31" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="H10" s="31" t="s">
-        <v>251</v>
+        <v>268</v>
       </c>
       <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
-      <c r="K10" s="31"/>
+      <c r="J10" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="K10" s="31" t="s">
+        <v>286</v>
+      </c>
       <c r="L10" s="31"/>
       <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
+      <c r="N10" s="31" t="s">
+        <v>287</v>
+      </c>
       <c r="O10" s="25"/>
       <c r="P10" s="31"/>
-      <c r="Q10" s="31" t="s">
-        <v>258</v>
-      </c>
+      <c r="Q10" s="31"/>
       <c r="R10" s="31"/>
       <c r="S10" s="31"/>
       <c r="T10" s="31"/>
@@ -7087,8 +7126,10 @@
       <c r="Z10" s="25"/>
       <c r="AA10" s="25"/>
       <c r="AB10" s="25"/>
-      <c r="AC10" s="25"/>
-      <c r="AD10" s="25"/>
+      <c r="AC10" s="25">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="14"/>
       <c r="AE10" s="25"/>
       <c r="AF10" s="25"/>
       <c r="AG10" s="25"/>
@@ -7102,22 +7143,39 @@
       <c r="AO10" s="26"/>
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C11" s="22"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
+      <c r="A11" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>Q5</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G11" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="H11" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
       <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="25"/>
-      <c r="R11" s="25"/>
-      <c r="S11" s="25"/>
-      <c r="T11" s="25"/>
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R11" s="31"/>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
       <c r="U11" s="25"/>
       <c r="V11" s="25"/>
       <c r="W11" s="25"/>
@@ -32841,16 +32899,61 @@
       <c r="AN670" s="25"/>
       <c r="AO670" s="26"/>
     </row>
+    <row r="671" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C671" s="22"/>
+      <c r="F671" s="25"/>
+      <c r="G671" s="25"/>
+      <c r="H671" s="25"/>
+      <c r="I671" s="25"/>
+      <c r="J671" s="25"/>
+      <c r="K671" s="25"/>
+      <c r="L671" s="25"/>
+      <c r="M671" s="25"/>
+      <c r="N671" s="25"/>
+      <c r="O671" s="25"/>
+      <c r="P671" s="25"/>
+      <c r="Q671" s="25"/>
+      <c r="R671" s="25"/>
+      <c r="S671" s="25"/>
+      <c r="T671" s="25"/>
+      <c r="U671" s="25"/>
+      <c r="V671" s="25"/>
+      <c r="W671" s="25"/>
+      <c r="X671" s="25"/>
+      <c r="Y671" s="25"/>
+      <c r="Z671" s="25"/>
+      <c r="AA671" s="25"/>
+      <c r="AB671" s="25"/>
+      <c r="AC671" s="25"/>
+      <c r="AD671" s="25"/>
+      <c r="AE671" s="25"/>
+      <c r="AF671" s="25"/>
+      <c r="AG671" s="25"/>
+      <c r="AH671" s="25"/>
+      <c r="AI671" s="25"/>
+      <c r="AJ671" s="25"/>
+      <c r="AK671" s="25"/>
+      <c r="AL671" s="25"/>
+      <c r="AM671" s="25"/>
+      <c r="AN671" s="25"/>
+      <c r="AO671" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A11:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
+  <conditionalFormatting sqref="A5:A9 A11">
+    <cfRule type="duplicateValues" dxfId="4" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A10">
-    <cfRule type="duplicateValues" dxfId="1" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="19"/>
+  <conditionalFormatting sqref="A12:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="2" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A10">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
implement Sort = "KEY=COUNT" for mcg
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC243E6-6CE9-48B5-A6E8-3647B70C25E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310A5179-3A28-497D-9EB1-DCE8820B1398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -184,7 +184,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="289">
   <si>
     <t>Make script</t>
   </si>
@@ -1048,6 +1048,9 @@
   </si>
   <si>
     <t>S1E2M0</t>
+  </si>
+  <si>
+    <t>ORDER=D KEY=COUNT</t>
   </si>
 </sst>
 </file>
@@ -7173,7 +7176,9 @@
       <c r="Q11" s="31" t="s">
         <v>258</v>
       </c>
-      <c r="R11" s="31"/>
+      <c r="R11" s="31" t="s">
+        <v>288</v>
+      </c>
       <c r="S11" s="31"/>
       <c r="T11" s="31"/>
       <c r="U11" s="25"/>

</xml_diff>

<commit_message>
- add named region R_miss_rec_val to mapping file - and read it with datenanpassr:::extract_named_region_params.excel()
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310A5179-3A28-497D-9EB1-DCE8820B1398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD4753-8658-464E-8079-CB735DFA2BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
+    <definedName name="R_miss_rec_val">Config!$B$35</definedName>
     <definedName name="V_Datum">Config!$B$18</definedName>
     <definedName name="V_ErrCountLog10">#REF!</definedName>
     <definedName name="V_ErrCountLog20">#REF!</definedName>
@@ -64,6 +65,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Wolf Wilke</author>
+    <author>wolf</author>
   </authors>
   <commentList>
     <comment ref="A23" authorId="0" shapeId="0" xr:uid="{55BAE0B3-D31C-4026-AEC7-838494A478E9}">
@@ -76,6 +78,30 @@
             <family val="2"/>
           </rPr>
           <t>Name of XML file with table date, to be appended by '&lt;QuestNo&gt;.xml'</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B35" authorId="1" shapeId="0" xr:uid="{C66B2E7D-D0C0-4A6E-9EDE-30A8B5CC27E2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>wolf:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+set all system missing values to this value, leave empty to keep them</t>
         </r>
       </text>
     </comment>
@@ -184,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="290">
   <si>
     <t>Make script</t>
   </si>
@@ -1052,6 +1078,9 @@
   <si>
     <t>ORDER=D KEY=COUNT</t>
   </si>
+  <si>
+    <t>Set missing value to</t>
+  </si>
 </sst>
 </file>
 
@@ -1136,7 +1165,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1233,6 +1262,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1247,7 +1282,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1296,6 +1331,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1734,7 +1770,6 @@
       <sheetName val="TableDefinition"/>
       <sheetName val="Free Beispiele"/>
       <sheetName val="Limesurvey"/>
-      <sheetName val="Funktionen 202304"/>
     </sheetNames>
     <definedNames>
       <definedName name="V_TemplateFill" refersTo="='Vorgaben Questions'!$A$4:$A$32"/>
@@ -1750,7 +1785,6 @@
       <sheetData sheetId="7"/>
       <sheetData sheetId="8"/>
       <sheetData sheetId="9"/>
-      <sheetData sheetId="10" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2359,6 +2393,14 @@
         <v>0</v>
       </c>
     </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="B35" s="36">
+        <v>-2</v>
+      </c>
+    </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="10" t="s">
         <v>36</v>
@@ -32951,14 +32993,12 @@
     <cfRule type="duplicateValues" dxfId="4" priority="20"/>
     <cfRule type="duplicateValues" dxfId="3" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="10"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A10">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A10">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A12:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
first version to remove invalid values from counts that are: - equal to R_miss_rec_val - or which are not the first in the list of invalid values (per case) - add invalid values to Unguelt in mapping to make the test make more sense
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFD4753-8658-464E-8079-CB735DFA2BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DE463C-64CF-4B2D-88B7-0E3BEB61657F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="291">
   <si>
     <t>Make script</t>
   </si>
@@ -1080,6 +1080,9 @@
   </si>
   <si>
     <t>Set missing value to</t>
+  </si>
+  <si>
+    <t>5, 2, 99,-2</t>
   </si>
 </sst>
 </file>
@@ -7205,7 +7208,7 @@
         <v>257</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>251</v>
+        <v>290</v>
       </c>
       <c r="I11" s="31"/>
       <c r="J11" s="31"/>

</xml_diff>

<commit_message>
implement Exclusive: - write in the same boolean column "val_to_count" as with the flagging of invalid values (see df_rows_long_invalids) - add new snapshot test
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DE463C-64CF-4B2D-88B7-0E3BEB61657F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2C206D-D51D-4517-80A8-5FD0775033EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="292">
   <si>
     <t>Make script</t>
   </si>
@@ -1084,6 +1084,9 @@
   <si>
     <t>5, 2, 99,-2</t>
   </si>
+  <si>
+    <t>5, 2</t>
+  </si>
 </sst>
 </file>
 
@@ -1328,13 +1331,13 @@
     <xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2400,7 +2403,7 @@
       <c r="A35" s="33" t="s">
         <v>289</v>
       </c>
-      <c r="B35" s="36">
+      <c r="B35" s="34">
         <v>-2</v>
       </c>
     </row>
@@ -2662,8 +2665,8 @@
     </row>
     <row r="2" spans="1:56" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="34"/>
-      <c r="B3" s="35"/>
+      <c r="A3" s="35"/>
+      <c r="B3" s="36"/>
       <c r="E3" s="18">
         <v>1</v>
       </c>
@@ -2817,8 +2820,8 @@
       <c r="BD3" s="19"/>
     </row>
     <row r="4" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="34"/>
-      <c r="B4" s="35"/>
+      <c r="A4" s="35"/>
+      <c r="B4" s="36"/>
       <c r="E4" s="18" t="s">
         <v>15</v>
       </c>
@@ -7249,20 +7252,39 @@
       <c r="AO11" s="26"/>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C12" s="22"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="25"/>
-      <c r="N12" s="25"/>
+      <c r="A12" s="30" t="str">
+        <f t="shared" ref="A12" si="3">"Q"&amp;LEFT(B12,FIND(".",B12)-1)</f>
+        <v>Q5</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G12" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="H12" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="31"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
-      <c r="Q12" s="25"/>
-      <c r="R12" s="25"/>
+      <c r="P12" s="31"/>
+      <c r="Q12" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R12" s="31" t="s">
+        <v>288</v>
+      </c>
       <c r="S12" s="25"/>
       <c r="T12" s="25"/>
       <c r="U12" s="25"/>
@@ -7284,7 +7306,9 @@
       <c r="AK12" s="25"/>
       <c r="AL12" s="25"/>
       <c r="AM12" s="25"/>
-      <c r="AN12" s="25"/>
+      <c r="AN12" s="25" t="s">
+        <v>291</v>
+      </c>
       <c r="AO12" s="26"/>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.25">
@@ -32992,7 +33016,7 @@
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="5" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A9 A11">
+  <conditionalFormatting sqref="A5:A9 A11:A12">
     <cfRule type="duplicateValues" dxfId="4" priority="20"/>
     <cfRule type="duplicateValues" dxfId="3" priority="21"/>
   </conditionalFormatting>
@@ -33000,7 +33024,7 @@
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12:A1048576 A2:A4">
+  <conditionalFormatting sqref="A13:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
set Freq = 0 for mw tables and test only one of the individual cat tables in the following row of the Questions sheet
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2C206D-D51D-4517-80A8-5FD0775033EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6DF5433-6DE0-45D0-A1F4-FDA62E4B9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="294">
   <si>
     <t>Make script</t>
   </si>
@@ -1087,6 +1087,12 @@
   <si>
     <t>5, 2</t>
   </si>
+  <si>
+    <t>q3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q3a </t>
+  </si>
 </sst>
 </file>
 
@@ -1776,6 +1782,7 @@
       <sheetName val="TableDefinition"/>
       <sheetName val="Free Beispiele"/>
       <sheetName val="Limesurvey"/>
+      <sheetName val="Funktionen 202304"/>
     </sheetNames>
     <definedNames>
       <definedName name="V_TemplateFill" refersTo="='Vorgaben Questions'!$A$4:$A$32"/>
@@ -1791,6 +1798,7 @@
       <sheetData sheetId="7"/>
       <sheetData sheetId="8"/>
       <sheetData sheetId="9"/>
+      <sheetData sheetId="10" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -6579,7 +6587,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI671"/>
+  <dimension ref="A1:AMI673"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -6901,7 +6909,7 @@
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="str">
-        <f t="shared" ref="A6:A11" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
+        <f t="shared" ref="A6:A13" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
         <v>Q2</v>
       </c>
       <c r="B6" s="30" t="s">
@@ -6988,7 +6996,9 @@
       <c r="S7" s="31"/>
       <c r="T7" s="31"/>
       <c r="U7" s="25"/>
-      <c r="V7" s="25"/>
+      <c r="V7" s="25">
+        <v>0</v>
+      </c>
       <c r="W7" s="25"/>
       <c r="X7" s="25"/>
       <c r="Y7" s="25"/>
@@ -7023,10 +7033,10 @@
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
       <c r="F8" s="31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="H8" s="31" t="s">
         <v>268</v>
@@ -7036,7 +7046,9 @@
       <c r="K8" s="31"/>
       <c r="L8" s="31"/>
       <c r="M8" s="31"/>
-      <c r="N8" s="31"/>
+      <c r="N8" s="31" t="s">
+        <v>279</v>
+      </c>
       <c r="O8" s="25"/>
       <c r="P8" s="31"/>
       <c r="Q8" s="31"/>
@@ -7044,25 +7056,21 @@
       <c r="S8" s="31"/>
       <c r="T8" s="31"/>
       <c r="U8" s="25"/>
-      <c r="V8" s="25">
-        <v>0</v>
-      </c>
+      <c r="V8" s="25"/>
       <c r="W8" s="25"/>
       <c r="X8" s="25"/>
       <c r="Y8" s="25"/>
       <c r="Z8" s="25"/>
       <c r="AA8" s="25"/>
       <c r="AB8" s="25"/>
-      <c r="AC8" s="25"/>
-      <c r="AD8" s="14" t="s">
-        <v>281</v>
-      </c>
+      <c r="AC8" s="25">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="14"/>
       <c r="AE8" s="25"/>
       <c r="AF8" s="25"/>
       <c r="AG8" s="25"/>
-      <c r="AH8" s="25" t="s">
-        <v>282</v>
-      </c>
+      <c r="AH8" s="25"/>
       <c r="AI8" s="25"/>
       <c r="AJ8" s="25"/>
       <c r="AK8" s="25"/>
@@ -7073,7 +7081,7 @@
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A9" s="30" t="str">
-        <f t="shared" ref="A9:A10" si="2">"Q"&amp;LEFT(B9,FIND(".",B9)-1)</f>
+        <f t="shared" ref="A9" si="2">"Q"&amp;LEFT(B9,FIND(".",B9)-1)</f>
         <v>Q3</v>
       </c>
       <c r="B9" s="30" t="s">
@@ -7096,9 +7104,7 @@
       <c r="K9" s="31"/>
       <c r="L9" s="31"/>
       <c r="M9" s="31"/>
-      <c r="N9" s="31" t="s">
-        <v>279</v>
-      </c>
+      <c r="N9" s="31"/>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
       <c r="Q9" s="31"/>
@@ -7106,23 +7112,25 @@
       <c r="S9" s="31"/>
       <c r="T9" s="31"/>
       <c r="U9" s="25"/>
-      <c r="V9" s="25"/>
+      <c r="V9" s="25">
+        <v>0</v>
+      </c>
       <c r="W9" s="25"/>
       <c r="X9" s="25"/>
       <c r="Y9" s="25"/>
       <c r="Z9" s="25"/>
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
-      <c r="AC9" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="14"/>
+      <c r="AC9" s="25"/>
+      <c r="AD9" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="AE9" s="25"/>
-      <c r="AF9" s="25" t="s">
-        <v>249</v>
-      </c>
+      <c r="AF9" s="25"/>
       <c r="AG9" s="25"/>
-      <c r="AH9" s="25"/>
+      <c r="AH9" s="25" t="s">
+        <v>282</v>
+      </c>
       <c r="AI9" s="25"/>
       <c r="AJ9" s="25"/>
       <c r="AK9" s="25"/>
@@ -7133,35 +7141,31 @@
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="str">
-        <f t="shared" si="2"/>
-        <v>Q4</v>
+        <f t="shared" ref="A10:A12" si="3">"Q"&amp;LEFT(B10,FIND(".",B10)-1)</f>
+        <v>Q3</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>283</v>
+        <v>254</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="31" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>268</v>
       </c>
       <c r="I10" s="31"/>
-      <c r="J10" s="31" t="s">
-        <v>285</v>
-      </c>
-      <c r="K10" s="31" t="s">
-        <v>286</v>
-      </c>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
       <c r="L10" s="31"/>
       <c r="M10" s="31"/>
       <c r="N10" s="31" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="O10" s="25"/>
       <c r="P10" s="31"/>
@@ -7170,7 +7174,9 @@
       <c r="S10" s="31"/>
       <c r="T10" s="31"/>
       <c r="U10" s="25"/>
-      <c r="V10" s="25"/>
+      <c r="V10" s="25">
+        <v>0</v>
+      </c>
       <c r="W10" s="25"/>
       <c r="X10" s="25"/>
       <c r="Y10" s="25"/>
@@ -7182,7 +7188,9 @@
       </c>
       <c r="AD10" s="14"/>
       <c r="AE10" s="25"/>
-      <c r="AF10" s="25"/>
+      <c r="AF10" s="25" t="s">
+        <v>249</v>
+      </c>
       <c r="AG10" s="25"/>
       <c r="AH10" s="25"/>
       <c r="AI10" s="25"/>
@@ -7195,38 +7203,36 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5</v>
+        <f t="shared" ref="A11" si="4">"Q"&amp;LEFT(B11,FIND(".",B11)-1)</f>
+        <v>Q3</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
       <c r="F11" s="31" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>257</v>
+        <v>293</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="I11" s="31"/>
       <c r="J11" s="31"/>
       <c r="K11" s="31"/>
       <c r="L11" s="31"/>
       <c r="M11" s="31"/>
-      <c r="N11" s="31"/>
+      <c r="N11" s="31" t="s">
+        <v>279</v>
+      </c>
       <c r="O11" s="25"/>
       <c r="P11" s="31"/>
-      <c r="Q11" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="R11" s="31" t="s">
-        <v>288</v>
-      </c>
+      <c r="Q11" s="31"/>
+      <c r="R11" s="31"/>
       <c r="S11" s="31"/>
       <c r="T11" s="31"/>
       <c r="U11" s="25"/>
@@ -7237,10 +7243,14 @@
       <c r="Z11" s="25"/>
       <c r="AA11" s="25"/>
       <c r="AB11" s="25"/>
-      <c r="AC11" s="25"/>
-      <c r="AD11" s="25"/>
+      <c r="AC11" s="25">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="14"/>
       <c r="AE11" s="25"/>
-      <c r="AF11" s="25"/>
+      <c r="AF11" s="25" t="s">
+        <v>249</v>
+      </c>
       <c r="AG11" s="25"/>
       <c r="AH11" s="25"/>
       <c r="AI11" s="25"/>
@@ -7253,40 +7263,42 @@
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A12" s="30" t="str">
-        <f t="shared" ref="A12" si="3">"Q"&amp;LEFT(B12,FIND(".",B12)-1)</f>
-        <v>Q5</v>
+        <f t="shared" si="3"/>
+        <v>Q4</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
       <c r="E12" s="30"/>
       <c r="F12" s="31" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>251</v>
+        <v>268</v>
       </c>
       <c r="I12" s="31"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="31"/>
+      <c r="J12" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="K12" s="31" t="s">
+        <v>286</v>
+      </c>
       <c r="L12" s="31"/>
       <c r="M12" s="31"/>
-      <c r="N12" s="31"/>
+      <c r="N12" s="31" t="s">
+        <v>287</v>
+      </c>
       <c r="O12" s="25"/>
       <c r="P12" s="31"/>
-      <c r="Q12" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="R12" s="31" t="s">
-        <v>288</v>
-      </c>
-      <c r="S12" s="25"/>
-      <c r="T12" s="25"/>
+      <c r="Q12" s="31"/>
+      <c r="R12" s="31"/>
+      <c r="S12" s="31"/>
+      <c r="T12" s="31"/>
       <c r="U12" s="25"/>
       <c r="V12" s="25"/>
       <c r="W12" s="25"/>
@@ -7295,8 +7307,10 @@
       <c r="Z12" s="25"/>
       <c r="AA12" s="25"/>
       <c r="AB12" s="25"/>
-      <c r="AC12" s="25"/>
-      <c r="AD12" s="25"/>
+      <c r="AC12" s="25">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="14"/>
       <c r="AE12" s="25"/>
       <c r="AF12" s="25"/>
       <c r="AG12" s="25"/>
@@ -7306,28 +7320,45 @@
       <c r="AK12" s="25"/>
       <c r="AL12" s="25"/>
       <c r="AM12" s="25"/>
-      <c r="AN12" s="25" t="s">
-        <v>291</v>
-      </c>
+      <c r="AN12" s="25"/>
       <c r="AO12" s="26"/>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C13" s="22"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
+      <c r="A13" s="30" t="str">
+        <f t="shared" si="0"/>
+        <v>Q5</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G13" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="H13" s="31" t="s">
+        <v>290</v>
+      </c>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
       <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="25"/>
-      <c r="R13" s="25"/>
-      <c r="S13" s="25"/>
-      <c r="T13" s="25"/>
+      <c r="P13" s="31"/>
+      <c r="Q13" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R13" s="31" t="s">
+        <v>288</v>
+      </c>
+      <c r="S13" s="31"/>
+      <c r="T13" s="31"/>
       <c r="U13" s="25"/>
       <c r="V13" s="25"/>
       <c r="W13" s="25"/>
@@ -7351,20 +7382,39 @@
       <c r="AO13" s="26"/>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C14" s="22"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
-      <c r="M14" s="25"/>
-      <c r="N14" s="25"/>
+      <c r="A14" s="30" t="str">
+        <f t="shared" ref="A14" si="5">"Q"&amp;LEFT(B14,FIND(".",B14)-1)</f>
+        <v>Q5</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>255</v>
+      </c>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="H14" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="25"/>
-      <c r="Q14" s="25"/>
-      <c r="R14" s="25"/>
+      <c r="P14" s="31"/>
+      <c r="Q14" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R14" s="31" t="s">
+        <v>288</v>
+      </c>
       <c r="S14" s="25"/>
       <c r="T14" s="25"/>
       <c r="U14" s="25"/>
@@ -7386,7 +7436,9 @@
       <c r="AK14" s="25"/>
       <c r="AL14" s="25"/>
       <c r="AM14" s="25"/>
-      <c r="AN14" s="25"/>
+      <c r="AN14" s="25" t="s">
+        <v>291</v>
+      </c>
       <c r="AO14" s="26"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.25">
@@ -33012,19 +33064,97 @@
       <c r="AN671" s="25"/>
       <c r="AO671" s="26"/>
     </row>
+    <row r="672" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C672" s="22"/>
+      <c r="F672" s="25"/>
+      <c r="G672" s="25"/>
+      <c r="H672" s="25"/>
+      <c r="I672" s="25"/>
+      <c r="J672" s="25"/>
+      <c r="K672" s="25"/>
+      <c r="L672" s="25"/>
+      <c r="M672" s="25"/>
+      <c r="N672" s="25"/>
+      <c r="O672" s="25"/>
+      <c r="P672" s="25"/>
+      <c r="Q672" s="25"/>
+      <c r="R672" s="25"/>
+      <c r="S672" s="25"/>
+      <c r="T672" s="25"/>
+      <c r="U672" s="25"/>
+      <c r="V672" s="25"/>
+      <c r="W672" s="25"/>
+      <c r="X672" s="25"/>
+      <c r="Y672" s="25"/>
+      <c r="Z672" s="25"/>
+      <c r="AA672" s="25"/>
+      <c r="AB672" s="25"/>
+      <c r="AC672" s="25"/>
+      <c r="AD672" s="25"/>
+      <c r="AE672" s="25"/>
+      <c r="AF672" s="25"/>
+      <c r="AG672" s="25"/>
+      <c r="AH672" s="25"/>
+      <c r="AI672" s="25"/>
+      <c r="AJ672" s="25"/>
+      <c r="AK672" s="25"/>
+      <c r="AL672" s="25"/>
+      <c r="AM672" s="25"/>
+      <c r="AN672" s="25"/>
+      <c r="AO672" s="26"/>
+    </row>
+    <row r="673" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C673" s="22"/>
+      <c r="F673" s="25"/>
+      <c r="G673" s="25"/>
+      <c r="H673" s="25"/>
+      <c r="I673" s="25"/>
+      <c r="J673" s="25"/>
+      <c r="K673" s="25"/>
+      <c r="L673" s="25"/>
+      <c r="M673" s="25"/>
+      <c r="N673" s="25"/>
+      <c r="O673" s="25"/>
+      <c r="P673" s="25"/>
+      <c r="Q673" s="25"/>
+      <c r="R673" s="25"/>
+      <c r="S673" s="25"/>
+      <c r="T673" s="25"/>
+      <c r="U673" s="25"/>
+      <c r="V673" s="25"/>
+      <c r="W673" s="25"/>
+      <c r="X673" s="25"/>
+      <c r="Y673" s="25"/>
+      <c r="Z673" s="25"/>
+      <c r="AA673" s="25"/>
+      <c r="AB673" s="25"/>
+      <c r="AC673" s="25"/>
+      <c r="AD673" s="25"/>
+      <c r="AE673" s="25"/>
+      <c r="AF673" s="25"/>
+      <c r="AG673" s="25"/>
+      <c r="AH673" s="25"/>
+      <c r="AI673" s="25"/>
+      <c r="AJ673" s="25"/>
+      <c r="AK673" s="25"/>
+      <c r="AL673" s="25"/>
+      <c r="AM673" s="25"/>
+      <c r="AN673" s="25"/>
+      <c r="AO673" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="5" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A9 A11:A12">
+  <conditionalFormatting sqref="A13:A14 A5:A11">
     <cfRule type="duplicateValues" dxfId="4" priority="20"/>
     <cfRule type="duplicateValues" dxfId="3" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A10">
+  <conditionalFormatting sqref="A12">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A13:A1048576 A2:A4">
+  <conditionalFormatting sqref="A15:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
- unnest RepOV qtabs - split RepOV strings and write the result into MWRec column (but MWRec is not processed yet)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6DF5433-6DE0-45D0-A1F4-FDA62E4B9B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652A058A-417B-4E07-9770-D6CEA6AB265F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="298">
   <si>
     <t>Make script</t>
   </si>
@@ -1093,6 +1093,18 @@
   <si>
     <t xml:space="preserve">q3a </t>
   </si>
+  <si>
+    <t>6. Ich nenne Ihnen gleich einige generelle Merkmale, die bei quantitativen Forschungsprojekten eine Rolle spielen. Bitte stufen Sie die Wichtigkeit ein.</t>
+  </si>
+  <si>
+    <t>q6a q6b q6c q6d q6e q6f q6g q6h</t>
+  </si>
+  <si>
+    <t>98,99,-2</t>
+  </si>
+  <si>
+    <t>TOP2:(4 THRU 5=100) (1 THRU 5=0)|TOP1:(5=100) (1 THRU 5=0)</t>
+  </si>
 </sst>
 </file>
 
@@ -1349,7 +1361,27 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2469,22 +2501,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="9" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="10" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="7" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="6" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7383,7 +7415,7 @@
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14" s="30" t="str">
-        <f t="shared" ref="A14" si="5">"Q"&amp;LEFT(B14,FIND(".",B14)-1)</f>
+        <f t="shared" ref="A14:A15" si="5">"Q"&amp;LEFT(B14,FIND(".",B14)-1)</f>
         <v>Q5</v>
       </c>
       <c r="B14" s="30" t="s">
@@ -7442,24 +7474,43 @@
       <c r="AO14" s="26"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C15" s="22"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="25"/>
-      <c r="N15" s="25"/>
+      <c r="A15" s="30" t="str">
+        <f t="shared" si="5"/>
+        <v>Q6</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>294</v>
+      </c>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G15" s="31" t="s">
+        <v>295</v>
+      </c>
+      <c r="H15" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="31"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="31"/>
       <c r="O15" s="25"/>
-      <c r="P15" s="25"/>
-      <c r="Q15" s="25"/>
-      <c r="R15" s="25"/>
-      <c r="S15" s="25"/>
-      <c r="T15" s="25"/>
-      <c r="U15" s="25"/>
-      <c r="V15" s="25"/>
+      <c r="P15" s="31"/>
+      <c r="Q15" s="31"/>
+      <c r="R15" s="31"/>
+      <c r="S15" s="31"/>
+      <c r="T15" s="31"/>
+      <c r="U15" s="31">
+        <v>0</v>
+      </c>
+      <c r="V15" s="25">
+        <v>0</v>
+      </c>
       <c r="W15" s="25"/>
       <c r="X15" s="25"/>
       <c r="Y15" s="25"/>
@@ -7475,7 +7526,9 @@
       <c r="AI15" s="25"/>
       <c r="AJ15" s="25"/>
       <c r="AK15" s="25"/>
-      <c r="AL15" s="25"/>
+      <c r="AL15" s="31" t="s">
+        <v>297</v>
+      </c>
       <c r="AM15" s="25"/>
       <c r="AN15" s="25"/>
       <c r="AO15" s="26"/>
@@ -33144,18 +33197,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A12">
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13:A14 A5:A11">
-    <cfRule type="duplicateValues" dxfId="4" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  <conditionalFormatting sqref="A16:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="2" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
+  <conditionalFormatting sqref="A15">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
- implement MWRec for stat_fun of qtab_type_cat - add test for MWRec
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652A058A-417B-4E07-9770-D6CEA6AB265F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2831EC42-DE09-412B-94C8-518930F9B017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="300">
   <si>
     <t>Make script</t>
   </si>
@@ -1103,7 +1103,13 @@
     <t>98,99,-2</t>
   </si>
   <si>
+    <t>S1E2</t>
+  </si>
+  <si>
     <t>TOP2:(4 THRU 5=100) (1 THRU 5=0)|TOP1:(5=100) (1 THRU 5=0)</t>
+  </si>
+  <si>
+    <t>(0 THRU 50 = -2)</t>
   </si>
 </sst>
 </file>
@@ -6619,7 +6625,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI673"/>
+  <dimension ref="A1:AMI674"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -6941,7 +6947,7 @@
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="str">
-        <f t="shared" ref="A6:A13" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
+        <f t="shared" ref="A6:A14" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
         <v>Q2</v>
       </c>
       <c r="B6" s="30" t="s">
@@ -7018,9 +7024,7 @@
       <c r="K7" s="31"/>
       <c r="L7" s="31"/>
       <c r="M7" s="31"/>
-      <c r="N7" s="31" t="s">
-        <v>279</v>
-      </c>
+      <c r="N7" s="31"/>
       <c r="O7" s="25"/>
       <c r="P7" s="31"/>
       <c r="Q7" s="31"/>
@@ -7123,10 +7127,10 @@
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
       <c r="F9" s="31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="H9" s="31" t="s">
         <v>268</v>
@@ -7134,9 +7138,13 @@
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
+      <c r="L9" s="31" t="s">
+        <v>299</v>
+      </c>
       <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
+      <c r="N9" s="31" t="s">
+        <v>297</v>
+      </c>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
       <c r="Q9" s="31"/>
@@ -7144,25 +7152,21 @@
       <c r="S9" s="31"/>
       <c r="T9" s="31"/>
       <c r="U9" s="25"/>
-      <c r="V9" s="25">
-        <v>0</v>
-      </c>
+      <c r="V9" s="25"/>
       <c r="W9" s="25"/>
       <c r="X9" s="25"/>
       <c r="Y9" s="25"/>
       <c r="Z9" s="25"/>
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
-      <c r="AC9" s="25"/>
-      <c r="AD9" s="14" t="s">
-        <v>281</v>
-      </c>
+      <c r="AC9" s="25">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="14"/>
       <c r="AE9" s="25"/>
       <c r="AF9" s="25"/>
       <c r="AG9" s="25"/>
-      <c r="AH9" s="25" t="s">
-        <v>282</v>
-      </c>
+      <c r="AH9" s="25"/>
       <c r="AI9" s="25"/>
       <c r="AJ9" s="25"/>
       <c r="AK9" s="25"/>
@@ -7173,7 +7177,7 @@
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A10" s="30" t="str">
-        <f t="shared" ref="A10:A12" si="3">"Q"&amp;LEFT(B10,FIND(".",B10)-1)</f>
+        <f t="shared" ref="A10" si="3">"Q"&amp;LEFT(B10,FIND(".",B10)-1)</f>
         <v>Q3</v>
       </c>
       <c r="B10" s="30" t="s">
@@ -7196,9 +7200,7 @@
       <c r="K10" s="31"/>
       <c r="L10" s="31"/>
       <c r="M10" s="31"/>
-      <c r="N10" s="31" t="s">
-        <v>279</v>
-      </c>
+      <c r="N10" s="31"/>
       <c r="O10" s="25"/>
       <c r="P10" s="31"/>
       <c r="Q10" s="31"/>
@@ -7215,16 +7217,16 @@
       <c r="Z10" s="25"/>
       <c r="AA10" s="25"/>
       <c r="AB10" s="25"/>
-      <c r="AC10" s="25">
-        <v>0</v>
-      </c>
-      <c r="AD10" s="14"/>
+      <c r="AC10" s="25"/>
+      <c r="AD10" s="14" t="s">
+        <v>281</v>
+      </c>
       <c r="AE10" s="25"/>
-      <c r="AF10" s="25" t="s">
-        <v>249</v>
-      </c>
+      <c r="AF10" s="25"/>
       <c r="AG10" s="25"/>
-      <c r="AH10" s="25"/>
+      <c r="AH10" s="25" t="s">
+        <v>282</v>
+      </c>
       <c r="AI10" s="25"/>
       <c r="AJ10" s="25"/>
       <c r="AK10" s="25"/>
@@ -7235,7 +7237,7 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="str">
-        <f t="shared" ref="A11" si="4">"Q"&amp;LEFT(B11,FIND(".",B11)-1)</f>
+        <f t="shared" ref="A11:A13" si="4">"Q"&amp;LEFT(B11,FIND(".",B11)-1)</f>
         <v>Q3</v>
       </c>
       <c r="B11" s="30" t="s">
@@ -7245,10 +7247,10 @@
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
       <c r="F11" s="31" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>268</v>
@@ -7268,7 +7270,9 @@
       <c r="S11" s="31"/>
       <c r="T11" s="31"/>
       <c r="U11" s="25"/>
-      <c r="V11" s="25"/>
+      <c r="V11" s="25">
+        <v>0</v>
+      </c>
       <c r="W11" s="25"/>
       <c r="X11" s="25"/>
       <c r="Y11" s="25"/>
@@ -7295,11 +7299,11 @@
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A12" s="30" t="str">
-        <f t="shared" si="3"/>
-        <v>Q4</v>
+        <f t="shared" ref="A12" si="5">"Q"&amp;LEFT(B12,FIND(".",B12)-1)</f>
+        <v>Q3</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>283</v>
+        <v>254</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -7308,22 +7312,18 @@
         <v>237</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="H12" s="31" t="s">
         <v>268</v>
       </c>
       <c r="I12" s="31"/>
-      <c r="J12" s="31" t="s">
-        <v>285</v>
-      </c>
-      <c r="K12" s="31" t="s">
-        <v>286</v>
-      </c>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
       <c r="L12" s="31"/>
       <c r="M12" s="31"/>
       <c r="N12" s="31" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="O12" s="25"/>
       <c r="P12" s="31"/>
@@ -7344,7 +7344,9 @@
       </c>
       <c r="AD12" s="14"/>
       <c r="AE12" s="25"/>
-      <c r="AF12" s="25"/>
+      <c r="AF12" s="25" t="s">
+        <v>249</v>
+      </c>
       <c r="AG12" s="25"/>
       <c r="AH12" s="25"/>
       <c r="AI12" s="25"/>
@@ -7357,38 +7359,40 @@
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A13" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5</v>
+        <f t="shared" si="4"/>
+        <v>Q4</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
       <c r="F13" s="31" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="I13" s="31"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
+      <c r="J13" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="K13" s="31" t="s">
+        <v>286</v>
+      </c>
       <c r="L13" s="31"/>
       <c r="M13" s="31"/>
-      <c r="N13" s="31"/>
+      <c r="N13" s="31" t="s">
+        <v>287</v>
+      </c>
       <c r="O13" s="25"/>
       <c r="P13" s="31"/>
-      <c r="Q13" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="R13" s="31" t="s">
-        <v>288</v>
-      </c>
+      <c r="Q13" s="31"/>
+      <c r="R13" s="31"/>
       <c r="S13" s="31"/>
       <c r="T13" s="31"/>
       <c r="U13" s="25"/>
@@ -7399,8 +7403,10 @@
       <c r="Z13" s="25"/>
       <c r="AA13" s="25"/>
       <c r="AB13" s="25"/>
-      <c r="AC13" s="25"/>
-      <c r="AD13" s="25"/>
+      <c r="AC13" s="25">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="14"/>
       <c r="AE13" s="25"/>
       <c r="AF13" s="25"/>
       <c r="AG13" s="25"/>
@@ -7415,7 +7421,7 @@
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14" s="30" t="str">
-        <f t="shared" ref="A14:A15" si="5">"Q"&amp;LEFT(B14,FIND(".",B14)-1)</f>
+        <f t="shared" si="0"/>
         <v>Q5</v>
       </c>
       <c r="B14" s="30" t="s">
@@ -7431,7 +7437,7 @@
         <v>257</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>251</v>
+        <v>290</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
@@ -7447,8 +7453,8 @@
       <c r="R14" s="31" t="s">
         <v>288</v>
       </c>
-      <c r="S14" s="25"/>
-      <c r="T14" s="25"/>
+      <c r="S14" s="31"/>
+      <c r="T14" s="31"/>
       <c r="U14" s="25"/>
       <c r="V14" s="25"/>
       <c r="W14" s="25"/>
@@ -7468,30 +7474,28 @@
       <c r="AK14" s="25"/>
       <c r="AL14" s="25"/>
       <c r="AM14" s="25"/>
-      <c r="AN14" s="25" t="s">
-        <v>291</v>
-      </c>
+      <c r="AN14" s="25"/>
       <c r="AO14" s="26"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="str">
-        <f t="shared" si="5"/>
-        <v>Q6</v>
+        <f t="shared" ref="A15:A16" si="6">"Q"&amp;LEFT(B15,FIND(".",B15)-1)</f>
+        <v>Q5</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>294</v>
+        <v>255</v>
       </c>
       <c r="C15" s="30"/>
       <c r="D15" s="30"/>
       <c r="E15" s="30"/>
       <c r="F15" s="31" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>295</v>
+        <v>257</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>296</v>
+        <v>251</v>
       </c>
       <c r="I15" s="31"/>
       <c r="J15" s="31"/>
@@ -7501,16 +7505,16 @@
       <c r="N15" s="31"/>
       <c r="O15" s="25"/>
       <c r="P15" s="31"/>
-      <c r="Q15" s="31"/>
-      <c r="R15" s="31"/>
-      <c r="S15" s="31"/>
-      <c r="T15" s="31"/>
-      <c r="U15" s="31">
-        <v>0</v>
-      </c>
-      <c r="V15" s="25">
-        <v>0</v>
-      </c>
+      <c r="Q15" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R15" s="31" t="s">
+        <v>288</v>
+      </c>
+      <c r="S15" s="25"/>
+      <c r="T15" s="25"/>
+      <c r="U15" s="25"/>
+      <c r="V15" s="25"/>
       <c r="W15" s="25"/>
       <c r="X15" s="25"/>
       <c r="Y15" s="25"/>
@@ -7526,32 +7530,51 @@
       <c r="AI15" s="25"/>
       <c r="AJ15" s="25"/>
       <c r="AK15" s="25"/>
-      <c r="AL15" s="31" t="s">
-        <v>297</v>
-      </c>
+      <c r="AL15" s="25"/>
       <c r="AM15" s="25"/>
-      <c r="AN15" s="25"/>
+      <c r="AN15" s="25" t="s">
+        <v>291</v>
+      </c>
       <c r="AO15" s="26"/>
     </row>
     <row r="16" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C16" s="22"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="25"/>
-      <c r="N16" s="25"/>
+      <c r="A16" s="30" t="str">
+        <f t="shared" si="6"/>
+        <v>Q6</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>294</v>
+      </c>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>295</v>
+      </c>
+      <c r="H16" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
       <c r="O16" s="25"/>
-      <c r="P16" s="25"/>
-      <c r="Q16" s="25"/>
-      <c r="R16" s="25"/>
-      <c r="S16" s="25"/>
-      <c r="T16" s="25"/>
-      <c r="U16" s="25"/>
-      <c r="V16" s="25"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="31"/>
+      <c r="S16" s="31"/>
+      <c r="T16" s="31"/>
+      <c r="U16" s="31">
+        <v>0</v>
+      </c>
+      <c r="V16" s="25">
+        <v>0</v>
+      </c>
       <c r="W16" s="25"/>
       <c r="X16" s="25"/>
       <c r="Y16" s="25"/>
@@ -7567,7 +7590,9 @@
       <c r="AI16" s="25"/>
       <c r="AJ16" s="25"/>
       <c r="AK16" s="25"/>
-      <c r="AL16" s="25"/>
+      <c r="AL16" s="31" t="s">
+        <v>298</v>
+      </c>
       <c r="AM16" s="25"/>
       <c r="AN16" s="25"/>
       <c r="AO16" s="26"/>
@@ -33195,25 +33220,64 @@
       <c r="AN673" s="25"/>
       <c r="AO673" s="26"/>
     </row>
+    <row r="674" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C674" s="22"/>
+      <c r="F674" s="25"/>
+      <c r="G674" s="25"/>
+      <c r="H674" s="25"/>
+      <c r="I674" s="25"/>
+      <c r="J674" s="25"/>
+      <c r="K674" s="25"/>
+      <c r="L674" s="25"/>
+      <c r="M674" s="25"/>
+      <c r="N674" s="25"/>
+      <c r="O674" s="25"/>
+      <c r="P674" s="25"/>
+      <c r="Q674" s="25"/>
+      <c r="R674" s="25"/>
+      <c r="S674" s="25"/>
+      <c r="T674" s="25"/>
+      <c r="U674" s="25"/>
+      <c r="V674" s="25"/>
+      <c r="W674" s="25"/>
+      <c r="X674" s="25"/>
+      <c r="Y674" s="25"/>
+      <c r="Z674" s="25"/>
+      <c r="AA674" s="25"/>
+      <c r="AB674" s="25"/>
+      <c r="AC674" s="25"/>
+      <c r="AD674" s="25"/>
+      <c r="AE674" s="25"/>
+      <c r="AF674" s="25"/>
+      <c r="AG674" s="25"/>
+      <c r="AH674" s="25"/>
+      <c r="AI674" s="25"/>
+      <c r="AJ674" s="25"/>
+      <c r="AK674" s="25"/>
+      <c r="AL674" s="25"/>
+      <c r="AM674" s="25"/>
+      <c r="AN674" s="25"/>
+      <c r="AO674" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="7" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A12">
+  <conditionalFormatting sqref="A13">
     <cfRule type="duplicateValues" dxfId="6" priority="3"/>
     <cfRule type="duplicateValues" dxfId="5" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A13:A14 A5:A11">
+  <conditionalFormatting sqref="A14:A15 A5:A12">
     <cfRule type="duplicateValues" dxfId="4" priority="22"/>
     <cfRule type="duplicateValues" dxfId="3" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A16:A1048576 A2:A4">
+  <conditionalFormatting sqref="A17:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="2" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15">
+  <conditionalFormatting sqref="A16">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A15">
+  <conditionalFormatting sqref="A16">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
- modify MdgVal to also cover ranges etc (e.g. "1 THRU 10") - added such an expression ("1 THRU 2, 4") to the first mdg in the excel file (but it doesn't change the results, as the data only contains 0s & 1s...)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2831EC42-DE09-412B-94C8-518930F9B017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A49E60F-9D54-42BC-9E97-E6FD00E55454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="301">
   <si>
     <t>Make script</t>
   </si>
@@ -1110,6 +1110,9 @@
   </si>
   <si>
     <t>(0 THRU 50 = -2)</t>
+  </si>
+  <si>
+    <t>1 THRU 2, 4</t>
   </si>
 </sst>
 </file>
@@ -6982,7 +6985,9 @@
       <c r="W6" s="25"/>
       <c r="X6" s="25"/>
       <c r="Y6" s="25"/>
-      <c r="Z6" s="25"/>
+      <c r="Z6" s="25" t="s">
+        <v>300</v>
+      </c>
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
       <c r="AC6" s="25"/>

</xml_diff>

<commit_message>
- refactor CatRec / CatLab to allow for multiple CatRec / CatLab (separated by "|") - add test to mapping
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A49E60F-9D54-42BC-9E97-E6FD00E55454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF67F94-A162-46E8-AEAA-87FB75DEB2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="304">
   <si>
     <t>Make script</t>
   </si>
@@ -1113,6 +1113,15 @@
   </si>
   <si>
     <t>1 THRU 2, 4</t>
+  </si>
+  <si>
+    <t>q6a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1 THRU 2=1) (3=2) (4 THRU 5=3)  | (1 THRU 2=1) (3=3) (4=4) (5=5) </t>
+  </si>
+  <si>
+    <t>1 '1 und 2' 2 '3' 3 '4 und 5' | 1 '1 und 2' 3 '3' 4 '4' 5 '5'</t>
   </si>
 </sst>
 </file>
@@ -7602,24 +7611,43 @@
       <c r="AN16" s="25"/>
       <c r="AO16" s="26"/>
     </row>
-    <row r="17" spans="3:41" x14ac:dyDescent="0.25">
-      <c r="C17" s="22"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="N17" s="25"/>
+    <row r="17" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="str">
+        <f t="shared" ref="A17" si="7">"Q"&amp;LEFT(B17,FIND(".",B17)-1)</f>
+        <v>Q6</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>294</v>
+      </c>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="G17" s="31" t="s">
+        <v>301</v>
+      </c>
+      <c r="H17" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31" t="s">
+        <v>302</v>
+      </c>
+      <c r="K17" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="L17" s="31"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="31"/>
       <c r="O17" s="25"/>
-      <c r="P17" s="25"/>
-      <c r="Q17" s="25"/>
-      <c r="R17" s="25"/>
-      <c r="S17" s="25"/>
-      <c r="T17" s="25"/>
-      <c r="U17" s="25"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
+      <c r="R17" s="31"/>
+      <c r="S17" s="31"/>
+      <c r="T17" s="31"/>
+      <c r="U17" s="31"/>
       <c r="V17" s="25"/>
       <c r="W17" s="25"/>
       <c r="X17" s="25"/>
@@ -7641,7 +7669,7 @@
       <c r="AN17" s="25"/>
       <c r="AO17" s="26"/>
     </row>
-    <row r="18" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C18" s="22"/>
       <c r="F18" s="25"/>
       <c r="G18" s="25"/>
@@ -7680,7 +7708,7 @@
       <c r="AN18" s="25"/>
       <c r="AO18" s="26"/>
     </row>
-    <row r="19" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C19" s="22"/>
       <c r="F19" s="25"/>
       <c r="G19" s="25"/>
@@ -7719,7 +7747,7 @@
       <c r="AN19" s="25"/>
       <c r="AO19" s="26"/>
     </row>
-    <row r="20" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C20" s="22"/>
       <c r="F20" s="25"/>
       <c r="G20" s="25"/>
@@ -7758,7 +7786,7 @@
       <c r="AN20" s="25"/>
       <c r="AO20" s="26"/>
     </row>
-    <row r="21" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C21" s="22"/>
       <c r="F21" s="25"/>
       <c r="G21" s="25"/>
@@ -7797,7 +7825,7 @@
       <c r="AN21" s="25"/>
       <c r="AO21" s="26"/>
     </row>
-    <row r="22" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C22" s="22"/>
       <c r="F22" s="25"/>
       <c r="G22" s="25"/>
@@ -7836,7 +7864,7 @@
       <c r="AN22" s="25"/>
       <c r="AO22" s="26"/>
     </row>
-    <row r="23" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C23" s="22"/>
       <c r="F23" s="25"/>
       <c r="G23" s="25"/>
@@ -7875,7 +7903,7 @@
       <c r="AN23" s="25"/>
       <c r="AO23" s="26"/>
     </row>
-    <row r="24" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C24" s="22"/>
       <c r="F24" s="25"/>
       <c r="G24" s="25"/>
@@ -7914,7 +7942,7 @@
       <c r="AN24" s="25"/>
       <c r="AO24" s="26"/>
     </row>
-    <row r="25" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C25" s="22"/>
       <c r="F25" s="25"/>
       <c r="G25" s="25"/>
@@ -7953,7 +7981,7 @@
       <c r="AN25" s="25"/>
       <c r="AO25" s="26"/>
     </row>
-    <row r="26" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C26" s="22"/>
       <c r="F26" s="25"/>
       <c r="G26" s="25"/>
@@ -7992,7 +8020,7 @@
       <c r="AN26" s="25"/>
       <c r="AO26" s="26"/>
     </row>
-    <row r="27" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C27" s="22"/>
       <c r="F27" s="25"/>
       <c r="G27" s="25"/>
@@ -8031,7 +8059,7 @@
       <c r="AN27" s="25"/>
       <c r="AO27" s="26"/>
     </row>
-    <row r="28" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C28" s="22"/>
       <c r="F28" s="25"/>
       <c r="G28" s="25"/>
@@ -8070,7 +8098,7 @@
       <c r="AN28" s="25"/>
       <c r="AO28" s="26"/>
     </row>
-    <row r="29" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C29" s="22"/>
       <c r="F29" s="25"/>
       <c r="G29" s="25"/>
@@ -8109,7 +8137,7 @@
       <c r="AN29" s="25"/>
       <c r="AO29" s="26"/>
     </row>
-    <row r="30" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C30" s="22"/>
       <c r="F30" s="25"/>
       <c r="G30" s="25"/>
@@ -8148,7 +8176,7 @@
       <c r="AN30" s="25"/>
       <c r="AO30" s="26"/>
     </row>
-    <row r="31" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C31" s="22"/>
       <c r="F31" s="25"/>
       <c r="G31" s="25"/>
@@ -8187,7 +8215,7 @@
       <c r="AN31" s="25"/>
       <c r="AO31" s="26"/>
     </row>
-    <row r="32" spans="3:41" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C32" s="22"/>
       <c r="F32" s="25"/>
       <c r="G32" s="25"/>
@@ -33276,14 +33304,12 @@
     <cfRule type="duplicateValues" dxfId="4" priority="22"/>
     <cfRule type="duplicateValues" dxfId="3" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A17:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="12"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A16">
+  <conditionalFormatting sqref="A16:A17">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A16">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A18:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
add a new test containing the {...} part in CatRec (which isn't implemented yet)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF67F94-A162-46E8-AEAA-87FB75DEB2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DDFACF-92E4-41F8-BDD1-9B786DD9B570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="308">
   <si>
     <t>Make script</t>
   </si>
@@ -1123,6 +1123,18 @@
   <si>
     <t>1 '1 und 2' 2 '3' 3 '4 und 5' | 1 '1 und 2' 3 '3' 4 '4' 5 '5'</t>
   </si>
+  <si>
+    <t>9. Würden Sie das Tabellenbandtool weiterempfehlen?' 'DC#SELVALLAB</t>
+  </si>
+  <si>
+    <t>(0 THRU 6=3) (7,8=2) (9,10=1) {[1]-[3]='NPS'}</t>
+  </si>
+  <si>
+    <t>1 'Promoters' 2 'Indifferent' 3 'Detractors'</t>
+  </si>
+  <si>
+    <t>q91</t>
+  </si>
 </sst>
 </file>
 
@@ -1379,7 +1391,27 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2519,22 +2551,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="11" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="10" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="9" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="8" priority="4">
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7613,7 +7645,7 @@
     </row>
     <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17" s="30" t="str">
-        <f t="shared" ref="A17" si="7">"Q"&amp;LEFT(B17,FIND(".",B17)-1)</f>
+        <f t="shared" ref="A17:A18" si="7">"Q"&amp;LEFT(B17,FIND(".",B17)-1)</f>
         <v>Q6</v>
       </c>
       <c r="B17" s="30" t="s">
@@ -7670,22 +7702,41 @@
       <c r="AO17" s="26"/>
     </row>
     <row r="18" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C18" s="22"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="25"/>
-      <c r="M18" s="25"/>
-      <c r="N18" s="25"/>
+      <c r="A18" s="30" t="str">
+        <f t="shared" si="7"/>
+        <v>Q9</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>304</v>
+      </c>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="G18" s="31" t="s">
+        <v>307</v>
+      </c>
+      <c r="H18" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="K18" s="31" t="s">
+        <v>306</v>
+      </c>
+      <c r="L18" s="31"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="31"/>
       <c r="O18" s="25"/>
-      <c r="P18" s="25"/>
-      <c r="Q18" s="25"/>
-      <c r="R18" s="25"/>
-      <c r="S18" s="25"/>
-      <c r="T18" s="25"/>
+      <c r="P18" s="31"/>
+      <c r="Q18" s="31"/>
+      <c r="R18" s="31"/>
+      <c r="S18" s="31"/>
+      <c r="T18" s="31"/>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
       <c r="W18" s="25"/>
@@ -33294,22 +33345,28 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:A15 A5:A12">
-    <cfRule type="duplicateValues" dxfId="4" priority="22"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A17">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A19:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="2" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A18">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A18:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="0" priority="12"/>
+  <conditionalFormatting sqref="A18">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
change test to use 2x selvar (of a single variable !) / selval
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DDFACF-92E4-41F8-BDD1-9B786DD9B570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA29840C-6AF9-4CD6-86DB-F24C174974F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="312">
   <si>
     <t>Make script</t>
   </si>
@@ -1135,6 +1135,18 @@
   <si>
     <t>q91</t>
   </si>
+  <si>
+    <t>1 2 3-6:Sonstige</t>
+  </si>
+  <si>
+    <t>sel0</t>
+  </si>
+  <si>
+    <t>q92</t>
+  </si>
+  <si>
+    <t>sel1</t>
+  </si>
 </sst>
 </file>
 
@@ -1391,7 +1403,7 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="16">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1517,6 +1529,26 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF5050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6669,7 +6701,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI674"/>
+  <dimension ref="A1:AMI673"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -7735,8 +7767,12 @@
       <c r="P18" s="31"/>
       <c r="Q18" s="31"/>
       <c r="R18" s="31"/>
-      <c r="S18" s="31"/>
-      <c r="T18" s="31"/>
+      <c r="S18" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T18" s="31" t="s">
+        <v>308</v>
+      </c>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
       <c r="W18" s="25"/>
@@ -7760,22 +7796,45 @@
       <c r="AO18" s="26"/>
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C19" s="22"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="25"/>
-      <c r="M19" s="25"/>
-      <c r="N19" s="25"/>
+      <c r="A19" s="30" t="str">
+        <f t="shared" ref="A19" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <v>Q9</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>304</v>
+      </c>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="G19" s="31" t="s">
+        <v>310</v>
+      </c>
+      <c r="H19" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="K19" s="31" t="s">
+        <v>306</v>
+      </c>
+      <c r="L19" s="31"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
       <c r="O19" s="25"/>
-      <c r="P19" s="25"/>
-      <c r="Q19" s="25"/>
-      <c r="R19" s="25"/>
-      <c r="S19" s="25"/>
-      <c r="T19" s="25"/>
+      <c r="P19" s="31"/>
+      <c r="Q19" s="31"/>
+      <c r="R19" s="31"/>
+      <c r="S19" s="31" t="s">
+        <v>311</v>
+      </c>
+      <c r="T19" s="31" t="s">
+        <v>308</v>
+      </c>
       <c r="U19" s="25"/>
       <c r="V19" s="25"/>
       <c r="W19" s="25"/>
@@ -33304,68 +33363,29 @@
       <c r="AN673" s="25"/>
       <c r="AO673" s="26"/>
     </row>
-    <row r="674" spans="3:41" x14ac:dyDescent="0.25">
-      <c r="C674" s="22"/>
-      <c r="F674" s="25"/>
-      <c r="G674" s="25"/>
-      <c r="H674" s="25"/>
-      <c r="I674" s="25"/>
-      <c r="J674" s="25"/>
-      <c r="K674" s="25"/>
-      <c r="L674" s="25"/>
-      <c r="M674" s="25"/>
-      <c r="N674" s="25"/>
-      <c r="O674" s="25"/>
-      <c r="P674" s="25"/>
-      <c r="Q674" s="25"/>
-      <c r="R674" s="25"/>
-      <c r="S674" s="25"/>
-      <c r="T674" s="25"/>
-      <c r="U674" s="25"/>
-      <c r="V674" s="25"/>
-      <c r="W674" s="25"/>
-      <c r="X674" s="25"/>
-      <c r="Y674" s="25"/>
-      <c r="Z674" s="25"/>
-      <c r="AA674" s="25"/>
-      <c r="AB674" s="25"/>
-      <c r="AC674" s="25"/>
-      <c r="AD674" s="25"/>
-      <c r="AE674" s="25"/>
-      <c r="AF674" s="25"/>
-      <c r="AG674" s="25"/>
-      <c r="AH674" s="25"/>
-      <c r="AI674" s="25"/>
-      <c r="AJ674" s="25"/>
-      <c r="AK674" s="25"/>
-      <c r="AL674" s="25"/>
-      <c r="AM674" s="25"/>
-      <c r="AN674" s="25"/>
-      <c r="AO674" s="26"/>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:A15 A5:A12">
-    <cfRule type="duplicateValues" dxfId="6" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A17">
-    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A19:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="14"/>
+  <conditionalFormatting sqref="A20:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A18">
+  <conditionalFormatting sqref="A18:A19">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A18">
+  <conditionalFormatting sqref="A18:A19">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
- refactor selvar/selval to also work with multiple `selvar`s - replace previous tests with single `selvar`s by a single test with multiple `selvar`s
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA29840C-6AF9-4CD6-86DB-F24C174974F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342C9C7C-4328-43F5-BE7C-E43FE0622D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="314">
   <si>
     <t>Make script</t>
   </si>
@@ -1136,6 +1136,12 @@
     <t>q91</t>
   </si>
   <si>
+    <t>q91 q92</t>
+  </si>
+  <si>
+    <t>sel0 sel1</t>
+  </si>
+  <si>
     <t>1 2 3-6:Sonstige</t>
   </si>
   <si>
@@ -1403,7 +1409,27 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2583,22 +2609,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="13" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="10" priority="4">
+    <cfRule type="expression" dxfId="12" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7744,9 +7770,7 @@
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
       <c r="E18" s="30"/>
-      <c r="F18" s="31" t="s">
-        <v>237</v>
-      </c>
+      <c r="F18" s="31"/>
       <c r="G18" s="31" t="s">
         <v>307</v>
       </c>
@@ -7768,10 +7792,10 @@
       <c r="Q18" s="31"/>
       <c r="R18" s="31"/>
       <c r="S18" s="31" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="T18" s="31" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
@@ -7797,7 +7821,7 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <f t="shared" ref="A19:A20" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
@@ -7806,11 +7830,9 @@
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
       <c r="E19" s="30"/>
-      <c r="F19" s="31" t="s">
-        <v>237</v>
-      </c>
+      <c r="F19" s="31"/>
       <c r="G19" s="31" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H19" s="31" t="s">
         <v>296</v>
@@ -7830,10 +7852,10 @@
       <c r="Q19" s="31"/>
       <c r="R19" s="31"/>
       <c r="S19" s="31" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="T19" s="31" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="U19" s="25"/>
       <c r="V19" s="25"/>
@@ -7858,22 +7880,45 @@
       <c r="AO19" s="26"/>
     </row>
     <row r="20" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C20" s="22"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-      <c r="M20" s="25"/>
-      <c r="N20" s="25"/>
+      <c r="A20" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>Q9</v>
+      </c>
+      <c r="B20" s="30" t="s">
+        <v>304</v>
+      </c>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="G20" s="31" t="s">
+        <v>308</v>
+      </c>
+      <c r="H20" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="K20" s="31" t="s">
+        <v>306</v>
+      </c>
+      <c r="L20" s="31"/>
+      <c r="M20" s="31"/>
+      <c r="N20" s="31"/>
       <c r="O20" s="25"/>
-      <c r="P20" s="25"/>
-      <c r="Q20" s="25"/>
-      <c r="R20" s="25"/>
-      <c r="S20" s="25"/>
-      <c r="T20" s="25"/>
+      <c r="P20" s="31"/>
+      <c r="Q20" s="31"/>
+      <c r="R20" s="31"/>
+      <c r="S20" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T20" s="31" t="s">
+        <v>310</v>
+      </c>
       <c r="U20" s="25"/>
       <c r="V20" s="25"/>
       <c r="W20" s="25"/>
@@ -33365,27 +33410,33 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:A15 A5:A12">
-    <cfRule type="duplicateValues" dxfId="6" priority="26"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A17">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A20:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
+  <conditionalFormatting sqref="A21:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="4" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:A19">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A18:A19">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A18:A19">
+  <conditionalFormatting sqref="A20">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
add SelVar/SelVal tests for mcg & mdg (not checked)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342C9C7C-4328-43F5-BE7C-E43FE0622D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995B3347-5093-45B1-BF9E-EA00E7C59C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="318">
   <si>
     <t>Make script</t>
   </si>
@@ -1153,6 +1153,18 @@
   <si>
     <t>sel1</t>
   </si>
+  <si>
+    <t xml:space="preserve">q2_01 q2_02 q2_03 q2_04 q2_05 q2_06 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">q5n1 q5n2 q5n3 q5n4 </t>
+  </si>
+  <si>
+    <t>NOT CHECKED: 2. Welche Art von Studien führen Sie mit dem Tabellenbandtool durch?' 'DC#SELVALLAB</t>
+  </si>
+  <si>
+    <t>NOT CHECKED: 5. Was lief besonders gut in den Projekten?</t>
+  </si>
 </sst>
 </file>
 
@@ -1409,7 +1421,47 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="22">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2609,22 +2661,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="15" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="19" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="13" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="12" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7821,7 +7873,7 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19:A20" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <f t="shared" ref="A19:A22" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
@@ -7942,28 +7994,47 @@
       <c r="AO20" s="26"/>
     </row>
     <row r="21" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C21" s="22"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="25"/>
-      <c r="M21" s="25"/>
-      <c r="N21" s="25"/>
+      <c r="A21" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>QNOT CHECKED: 2</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>316</v>
+      </c>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>314</v>
+      </c>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="31"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="31"/>
       <c r="O21" s="25"/>
-      <c r="P21" s="25"/>
-      <c r="Q21" s="25"/>
-      <c r="R21" s="25"/>
-      <c r="S21" s="25"/>
-      <c r="T21" s="25"/>
+      <c r="P21" s="31"/>
+      <c r="Q21" s="31"/>
+      <c r="R21" s="31"/>
+      <c r="S21" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T21" s="31" t="s">
+        <v>310</v>
+      </c>
       <c r="U21" s="25"/>
       <c r="V21" s="25"/>
       <c r="W21" s="25"/>
       <c r="X21" s="25"/>
       <c r="Y21" s="25"/>
-      <c r="Z21" s="25"/>
+      <c r="Z21" s="25" t="s">
+        <v>300</v>
+      </c>
       <c r="AA21" s="25"/>
       <c r="AB21" s="25"/>
       <c r="AC21" s="25"/>
@@ -7981,22 +8052,45 @@
       <c r="AO21" s="26"/>
     </row>
     <row r="22" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C22" s="22"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="25"/>
-      <c r="M22" s="25"/>
-      <c r="N22" s="25"/>
+      <c r="A22" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>QNOT CHECKED: 5</v>
+      </c>
+      <c r="B22" s="30" t="s">
+        <v>317</v>
+      </c>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>315</v>
+      </c>
+      <c r="H22" s="31" t="s">
+        <v>290</v>
+      </c>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="31"/>
+      <c r="M22" s="31"/>
+      <c r="N22" s="31"/>
       <c r="O22" s="25"/>
-      <c r="P22" s="25"/>
-      <c r="Q22" s="25"/>
-      <c r="R22" s="25"/>
-      <c r="S22" s="25"/>
-      <c r="T22" s="25"/>
+      <c r="P22" s="31"/>
+      <c r="Q22" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R22" s="31" t="s">
+        <v>288</v>
+      </c>
+      <c r="S22" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T22" s="31" t="s">
+        <v>310</v>
+      </c>
       <c r="U22" s="25"/>
       <c r="V22" s="25"/>
       <c r="W22" s="25"/>
@@ -33410,34 +33504,42 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:A15 A5:A12">
-    <cfRule type="duplicateValues" dxfId="8" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A17">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A21:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="4" priority="18"/>
+  <conditionalFormatting sqref="A23:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="8" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:A19">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:A19">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A21">
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A22">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
add test for multiple SelVar & type mw
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995B3347-5093-45B1-BF9E-EA00E7C59C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D837C7D-0558-4502-AFA7-019186535053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="324">
   <si>
     <t>Make script</t>
   </si>
@@ -1165,6 +1165,24 @@
   <si>
     <t>NOT CHECKED: 5. Was lief besonders gut in den Projekten?</t>
   </si>
+  <si>
+    <t>7. Für die abgefragten Studienarten: Wie zufrieden sind Sie mit dem Tabellenbandtool bezüglich der eben abgefragten Merkmale?' 'DC#SELVALLAB</t>
+  </si>
+  <si>
+    <t>(1 THRU 4=1) (5 THRU 7=2) (8 THRU 10=3)</t>
+  </si>
+  <si>
+    <t>1 '1 bis 4' 2 '5 bis 7' 3 '8 bis 10'</t>
+  </si>
+  <si>
+    <t>2 3-6:Sonstige</t>
+  </si>
+  <si>
+    <t>TOP3:(8 THRU 10=100) (1 THRU 10=0)</t>
+  </si>
+  <si>
+    <t>q7a1 q7a2 q7b1 q7b2</t>
+  </si>
 </sst>
 </file>
 
@@ -1583,6 +1601,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF7C80"/>
@@ -1607,26 +1645,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF5050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2661,22 +2679,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="19" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="20" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="19" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="16" priority="4">
+    <cfRule type="expression" dxfId="18" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7873,7 +7891,7 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19:A22" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <f t="shared" ref="A19:A23" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
@@ -8114,22 +8132,47 @@
       <c r="AO22" s="26"/>
     </row>
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C23" s="22"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
-      <c r="M23" s="25"/>
-      <c r="N23" s="25"/>
+      <c r="A23" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>Q7</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>318</v>
+      </c>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G23" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="H23" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="K23" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="L23" s="31"/>
+      <c r="M23" s="31"/>
+      <c r="N23" s="31" t="s">
+        <v>297</v>
+      </c>
       <c r="O23" s="25"/>
-      <c r="P23" s="25"/>
-      <c r="Q23" s="25"/>
-      <c r="R23" s="25"/>
-      <c r="S23" s="25"/>
-      <c r="T23" s="25"/>
+      <c r="P23" s="31"/>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="31"/>
+      <c r="S23" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T23" s="31" t="s">
+        <v>321</v>
+      </c>
       <c r="U23" s="25"/>
       <c r="V23" s="25"/>
       <c r="W23" s="25"/>
@@ -8147,7 +8190,9 @@
       <c r="AI23" s="25"/>
       <c r="AJ23" s="25"/>
       <c r="AK23" s="25"/>
-      <c r="AL23" s="25"/>
+      <c r="AL23" s="31" t="s">
+        <v>322</v>
+      </c>
       <c r="AM23" s="25"/>
       <c r="AN23" s="25"/>
       <c r="AO23" s="26"/>
@@ -33504,42 +33549,44 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="15" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="duplicateValues" dxfId="14" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:A15 A5:A12">
-    <cfRule type="duplicateValues" dxfId="12" priority="32"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A17">
-    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="12"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A23:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="8" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:A19">
+    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20">
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A18:A19">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A20">
+  <conditionalFormatting sqref="A21">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A20">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  <conditionalFormatting sqref="A22">
+    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A21">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+  <conditionalFormatting sqref="A24:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="2" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A22">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  <conditionalFormatting sqref="A23">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A23">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
allow to specify multiple cat RowVar and add test
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D837C7D-0558-4502-AFA7-019186535053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C9EF9E-AC8E-43F1-8920-D4BED3A75A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7304,7 +7304,7 @@
         <v>237</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="H9" s="31" t="s">
         <v>268</v>
@@ -33579,14 +33579,12 @@
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="24"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A23">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A24:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="0" priority="24"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
try to do multi selvar mdg with Unguelt (doesn't work)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C9EF9E-AC8E-43F1-8920-D4BED3A75A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF88102-75E1-405C-94A3-FD14BDAD0FCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="327">
   <si>
     <t>Make script</t>
   </si>
@@ -1182,6 +1182,15 @@
   </si>
   <si>
     <t>q7a1 q7a2 q7b1 q7b2</t>
+  </si>
+  <si>
+    <t>With Unguelt: 2. Welche Art von Studien führen Sie mit dem Tabellenbandtool durch?' 'DC#SELVALLAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q2_99 q2_00 q2_99 q2_00 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">q2_01 q2_02 q2_03 q2_04 </t>
   </si>
 </sst>
 </file>
@@ -6797,7 +6806,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI673"/>
+  <dimension ref="A1:AMI674"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -7891,7 +7900,7 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19:A23" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <f t="shared" ref="A19:A24" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
@@ -8071,23 +8080,23 @@
     </row>
     <row r="22" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>QNOT CHECKED: 5</v>
+        <f t="shared" ref="A22" si="9">"Q"&amp;LEFT(B22,FIND(".",B22)-1)</f>
+        <v>QWith Unguelt: 2</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
       <c r="F22" s="31" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>315</v>
+        <v>326</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>290</v>
+        <v>325</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -8097,12 +8106,8 @@
       <c r="N22" s="31"/>
       <c r="O22" s="25"/>
       <c r="P22" s="31"/>
-      <c r="Q22" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="R22" s="31" t="s">
-        <v>288</v>
-      </c>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="31"/>
       <c r="S22" s="31" t="s">
         <v>309</v>
       </c>
@@ -8114,7 +8119,9 @@
       <c r="W22" s="25"/>
       <c r="X22" s="25"/>
       <c r="Y22" s="25"/>
-      <c r="Z22" s="25"/>
+      <c r="Z22" s="25" t="s">
+        <v>300</v>
+      </c>
       <c r="AA22" s="25"/>
       <c r="AB22" s="25"/>
       <c r="AC22" s="25"/>
@@ -8134,44 +8141,42 @@
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="str">
         <f t="shared" si="8"/>
-        <v>Q7</v>
+        <v>QNOT CHECKED: 5</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="E23" s="30"/>
       <c r="F23" s="31" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="I23" s="31"/>
-      <c r="J23" s="31" t="s">
-        <v>319</v>
-      </c>
-      <c r="K23" s="31" t="s">
-        <v>320</v>
-      </c>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
       <c r="L23" s="31"/>
       <c r="M23" s="31"/>
-      <c r="N23" s="31" t="s">
-        <v>297</v>
-      </c>
+      <c r="N23" s="31"/>
       <c r="O23" s="25"/>
       <c r="P23" s="31"/>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
+      <c r="Q23" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R23" s="31" t="s">
+        <v>288</v>
+      </c>
       <c r="S23" s="31" t="s">
         <v>309</v>
       </c>
       <c r="T23" s="31" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="U23" s="25"/>
       <c r="V23" s="25"/>
@@ -8190,30 +8195,53 @@
       <c r="AI23" s="25"/>
       <c r="AJ23" s="25"/>
       <c r="AK23" s="25"/>
-      <c r="AL23" s="31" t="s">
-        <v>322</v>
-      </c>
+      <c r="AL23" s="25"/>
       <c r="AM23" s="25"/>
       <c r="AN23" s="25"/>
       <c r="AO23" s="26"/>
     </row>
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C24" s="22"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
+      <c r="A24" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>Q7</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>318</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G24" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="H24" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="K24" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="L24" s="31"/>
+      <c r="M24" s="31"/>
+      <c r="N24" s="31" t="s">
+        <v>297</v>
+      </c>
       <c r="O24" s="25"/>
-      <c r="P24" s="25"/>
-      <c r="Q24" s="25"/>
-      <c r="R24" s="25"/>
-      <c r="S24" s="25"/>
-      <c r="T24" s="25"/>
+      <c r="P24" s="31"/>
+      <c r="Q24" s="31"/>
+      <c r="R24" s="31"/>
+      <c r="S24" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T24" s="31" t="s">
+        <v>321</v>
+      </c>
       <c r="U24" s="25"/>
       <c r="V24" s="25"/>
       <c r="W24" s="25"/>
@@ -8231,7 +8259,9 @@
       <c r="AI24" s="25"/>
       <c r="AJ24" s="25"/>
       <c r="AK24" s="25"/>
-      <c r="AL24" s="25"/>
+      <c r="AL24" s="31" t="s">
+        <v>322</v>
+      </c>
       <c r="AM24" s="25"/>
       <c r="AN24" s="25"/>
       <c r="AO24" s="26"/>
@@ -33547,6 +33577,45 @@
       <c r="AN673" s="25"/>
       <c r="AO673" s="26"/>
     </row>
+    <row r="674" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C674" s="22"/>
+      <c r="F674" s="25"/>
+      <c r="G674" s="25"/>
+      <c r="H674" s="25"/>
+      <c r="I674" s="25"/>
+      <c r="J674" s="25"/>
+      <c r="K674" s="25"/>
+      <c r="L674" s="25"/>
+      <c r="M674" s="25"/>
+      <c r="N674" s="25"/>
+      <c r="O674" s="25"/>
+      <c r="P674" s="25"/>
+      <c r="Q674" s="25"/>
+      <c r="R674" s="25"/>
+      <c r="S674" s="25"/>
+      <c r="T674" s="25"/>
+      <c r="U674" s="25"/>
+      <c r="V674" s="25"/>
+      <c r="W674" s="25"/>
+      <c r="X674" s="25"/>
+      <c r="Y674" s="25"/>
+      <c r="Z674" s="25"/>
+      <c r="AA674" s="25"/>
+      <c r="AB674" s="25"/>
+      <c r="AC674" s="25"/>
+      <c r="AD674" s="25"/>
+      <c r="AE674" s="25"/>
+      <c r="AF674" s="25"/>
+      <c r="AG674" s="25"/>
+      <c r="AH674" s="25"/>
+      <c r="AI674" s="25"/>
+      <c r="AJ674" s="25"/>
+      <c r="AK674" s="25"/>
+      <c r="AL674" s="25"/>
+      <c r="AM674" s="25"/>
+      <c r="AN674" s="25"/>
+      <c r="AO674" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="17" priority="17"/>
@@ -33571,19 +33640,19 @@
     <cfRule type="duplicateValues" dxfId="8" priority="7"/>
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A21">
+  <conditionalFormatting sqref="A21:A22">
     <cfRule type="duplicateValues" dxfId="6" priority="5"/>
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A22">
+  <conditionalFormatting sqref="A23">
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23">
+  <conditionalFormatting sqref="A24">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24:A1048576 A2:A4">
+  <conditionalFormatting sqref="A25:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="24"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
2nd try to do multi selvar unguelt mdg
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C9EF9E-AC8E-43F1-8920-D4BED3A75A09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E687BF6-9B27-414B-A540-D716C648BCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="328">
   <si>
     <t>Make script</t>
   </si>
@@ -1182,6 +1182,18 @@
   </si>
   <si>
     <t>q7a1 q7a2 q7b1 q7b2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q2_01 q2_02 q2_03 q2_04 </t>
+  </si>
+  <si>
+    <t>3-6:Sonstige</t>
+  </si>
+  <si>
+    <t>multi selvar with unguelt: 2. Welche Art von Studien führen Sie mit dem Tabellenbandtool durch?' 'DC#SELVALLAB</t>
+  </si>
+  <si>
+    <t>q2_05 q2_05 q2_00 q2_00</t>
   </si>
 </sst>
 </file>
@@ -6797,7 +6809,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI673"/>
+  <dimension ref="A1:AMI674"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -7891,7 +7903,7 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19:A23" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <f t="shared" ref="A19:A24" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
@@ -8071,23 +8083,23 @@
     </row>
     <row r="22" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A22" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>QNOT CHECKED: 5</v>
+        <f t="shared" ref="A22" si="9">"Q"&amp;LEFT(B22,FIND(".",B22)-1)</f>
+        <v>Qmulti selvar with unguelt: 2</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
       <c r="F22" s="31" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -8097,17 +8109,13 @@
       <c r="N22" s="31"/>
       <c r="O22" s="25"/>
       <c r="P22" s="31"/>
-      <c r="Q22" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="R22" s="31" t="s">
-        <v>288</v>
-      </c>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="31"/>
       <c r="S22" s="31" t="s">
         <v>309</v>
       </c>
       <c r="T22" s="31" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="U22" s="25"/>
       <c r="V22" s="25"/>
@@ -8134,44 +8142,42 @@
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="str">
         <f t="shared" si="8"/>
-        <v>Q7</v>
+        <v>QNOT CHECKED: 5</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="E23" s="30"/>
       <c r="F23" s="31" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="I23" s="31"/>
-      <c r="J23" s="31" t="s">
-        <v>319</v>
-      </c>
-      <c r="K23" s="31" t="s">
-        <v>320</v>
-      </c>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
       <c r="L23" s="31"/>
       <c r="M23" s="31"/>
-      <c r="N23" s="31" t="s">
-        <v>297</v>
-      </c>
+      <c r="N23" s="31"/>
       <c r="O23" s="25"/>
       <c r="P23" s="31"/>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
+      <c r="Q23" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R23" s="31" t="s">
+        <v>288</v>
+      </c>
       <c r="S23" s="31" t="s">
         <v>309</v>
       </c>
       <c r="T23" s="31" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="U23" s="25"/>
       <c r="V23" s="25"/>
@@ -8190,30 +8196,53 @@
       <c r="AI23" s="25"/>
       <c r="AJ23" s="25"/>
       <c r="AK23" s="25"/>
-      <c r="AL23" s="31" t="s">
-        <v>322</v>
-      </c>
+      <c r="AL23" s="25"/>
       <c r="AM23" s="25"/>
       <c r="AN23" s="25"/>
       <c r="AO23" s="26"/>
     </row>
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C24" s="22"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
+      <c r="A24" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>Q7</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>318</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G24" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="H24" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="K24" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="L24" s="31"/>
+      <c r="M24" s="31"/>
+      <c r="N24" s="31" t="s">
+        <v>297</v>
+      </c>
       <c r="O24" s="25"/>
-      <c r="P24" s="25"/>
-      <c r="Q24" s="25"/>
-      <c r="R24" s="25"/>
-      <c r="S24" s="25"/>
-      <c r="T24" s="25"/>
+      <c r="P24" s="31"/>
+      <c r="Q24" s="31"/>
+      <c r="R24" s="31"/>
+      <c r="S24" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T24" s="31" t="s">
+        <v>321</v>
+      </c>
       <c r="U24" s="25"/>
       <c r="V24" s="25"/>
       <c r="W24" s="25"/>
@@ -8231,7 +8260,9 @@
       <c r="AI24" s="25"/>
       <c r="AJ24" s="25"/>
       <c r="AK24" s="25"/>
-      <c r="AL24" s="25"/>
+      <c r="AL24" s="31" t="s">
+        <v>322</v>
+      </c>
       <c r="AM24" s="25"/>
       <c r="AN24" s="25"/>
       <c r="AO24" s="26"/>
@@ -33547,6 +33578,45 @@
       <c r="AN673" s="25"/>
       <c r="AO673" s="26"/>
     </row>
+    <row r="674" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C674" s="22"/>
+      <c r="F674" s="25"/>
+      <c r="G674" s="25"/>
+      <c r="H674" s="25"/>
+      <c r="I674" s="25"/>
+      <c r="J674" s="25"/>
+      <c r="K674" s="25"/>
+      <c r="L674" s="25"/>
+      <c r="M674" s="25"/>
+      <c r="N674" s="25"/>
+      <c r="O674" s="25"/>
+      <c r="P674" s="25"/>
+      <c r="Q674" s="25"/>
+      <c r="R674" s="25"/>
+      <c r="S674" s="25"/>
+      <c r="T674" s="25"/>
+      <c r="U674" s="25"/>
+      <c r="V674" s="25"/>
+      <c r="W674" s="25"/>
+      <c r="X674" s="25"/>
+      <c r="Y674" s="25"/>
+      <c r="Z674" s="25"/>
+      <c r="AA674" s="25"/>
+      <c r="AB674" s="25"/>
+      <c r="AC674" s="25"/>
+      <c r="AD674" s="25"/>
+      <c r="AE674" s="25"/>
+      <c r="AF674" s="25"/>
+      <c r="AG674" s="25"/>
+      <c r="AH674" s="25"/>
+      <c r="AI674" s="25"/>
+      <c r="AJ674" s="25"/>
+      <c r="AK674" s="25"/>
+      <c r="AL674" s="25"/>
+      <c r="AM674" s="25"/>
+      <c r="AN674" s="25"/>
+      <c r="AO674" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="17" priority="17"/>
@@ -33571,19 +33641,19 @@
     <cfRule type="duplicateValues" dxfId="8" priority="7"/>
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A21">
+  <conditionalFormatting sqref="A21:A22">
     <cfRule type="duplicateValues" dxfId="6" priority="5"/>
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A22">
+  <conditionalFormatting sqref="A23">
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23">
+  <conditionalFormatting sqref="A24">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24:A1048576 A2:A4">
+  <conditionalFormatting sqref="A25:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="24"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
- don't count mdg cases which are invalid but where respondent also selected a valid answer - if only invalids are selected, only count the first one - add test
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E687BF6-9B27-414B-A540-D716C648BCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC38095-7901-4065-94B6-9396BD1A4B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="331">
   <si>
     <t>Make script</t>
   </si>
@@ -1194,6 +1194,15 @@
   </si>
   <si>
     <t>q2_05 q2_05 q2_00 q2_00</t>
+  </si>
+  <si>
+    <t>trigger invalid values: 2. Welche Art von Studien führen Sie mit dem Tabellenbandtool durch?</t>
+  </si>
+  <si>
+    <t>q2_06</t>
+  </si>
+  <si>
+    <t>q2_02 q2_01</t>
   </si>
 </sst>
 </file>
@@ -6809,7 +6818,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMI674"/>
+  <dimension ref="A1:AMI675"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="22" customWidth="1"/>
@@ -7903,7 +7912,7 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19:A24" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
+        <f t="shared" ref="A19:A25" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
@@ -8141,23 +8150,23 @@
     </row>
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A23" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>QNOT CHECKED: 5</v>
+        <f t="shared" ref="A23" si="10">"Q"&amp;LEFT(B23,FIND(".",B23)-1)</f>
+        <v>Qtrigger invalid values: 2</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>317</v>
+        <v>328</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="E23" s="30"/>
       <c r="F23" s="31" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>315</v>
+        <v>329</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>290</v>
+        <v>330</v>
       </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
@@ -8167,18 +8176,10 @@
       <c r="N23" s="31"/>
       <c r="O23" s="25"/>
       <c r="P23" s="31"/>
-      <c r="Q23" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="R23" s="31" t="s">
-        <v>288</v>
-      </c>
-      <c r="S23" s="31" t="s">
-        <v>309</v>
-      </c>
-      <c r="T23" s="31" t="s">
-        <v>310</v>
-      </c>
+      <c r="Q23" s="31"/>
+      <c r="R23" s="31"/>
+      <c r="S23" s="31"/>
+      <c r="T23" s="31"/>
       <c r="U23" s="25"/>
       <c r="V23" s="25"/>
       <c r="W23" s="25"/>
@@ -8204,44 +8205,42 @@
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A24" s="30" t="str">
         <f t="shared" si="8"/>
-        <v>Q7</v>
+        <v>QNOT CHECKED: 5</v>
       </c>
       <c r="B24" s="30" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
       <c r="E24" s="30"/>
       <c r="F24" s="31" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="H24" s="31" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="I24" s="31"/>
-      <c r="J24" s="31" t="s">
-        <v>319</v>
-      </c>
-      <c r="K24" s="31" t="s">
-        <v>320</v>
-      </c>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
       <c r="L24" s="31"/>
       <c r="M24" s="31"/>
-      <c r="N24" s="31" t="s">
-        <v>297</v>
-      </c>
+      <c r="N24" s="31"/>
       <c r="O24" s="25"/>
       <c r="P24" s="31"/>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
+      <c r="Q24" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="R24" s="31" t="s">
+        <v>288</v>
+      </c>
       <c r="S24" s="31" t="s">
         <v>309</v>
       </c>
       <c r="T24" s="31" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="U24" s="25"/>
       <c r="V24" s="25"/>
@@ -8260,30 +8259,53 @@
       <c r="AI24" s="25"/>
       <c r="AJ24" s="25"/>
       <c r="AK24" s="25"/>
-      <c r="AL24" s="31" t="s">
-        <v>322</v>
-      </c>
+      <c r="AL24" s="25"/>
       <c r="AM24" s="25"/>
       <c r="AN24" s="25"/>
       <c r="AO24" s="26"/>
     </row>
     <row r="25" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="C25" s="22"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="J25" s="25"/>
-      <c r="K25" s="25"/>
-      <c r="L25" s="25"/>
-      <c r="M25" s="25"/>
-      <c r="N25" s="25"/>
+      <c r="A25" s="30" t="str">
+        <f t="shared" si="8"/>
+        <v>Q7</v>
+      </c>
+      <c r="B25" s="30" t="s">
+        <v>318</v>
+      </c>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G25" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="H25" s="31" t="s">
+        <v>296</v>
+      </c>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="K25" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31" t="s">
+        <v>297</v>
+      </c>
       <c r="O25" s="25"/>
-      <c r="P25" s="25"/>
-      <c r="Q25" s="25"/>
-      <c r="R25" s="25"/>
-      <c r="S25" s="25"/>
-      <c r="T25" s="25"/>
+      <c r="P25" s="31"/>
+      <c r="Q25" s="31"/>
+      <c r="R25" s="31"/>
+      <c r="S25" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="T25" s="31" t="s">
+        <v>321</v>
+      </c>
       <c r="U25" s="25"/>
       <c r="V25" s="25"/>
       <c r="W25" s="25"/>
@@ -8301,7 +8323,9 @@
       <c r="AI25" s="25"/>
       <c r="AJ25" s="25"/>
       <c r="AK25" s="25"/>
-      <c r="AL25" s="25"/>
+      <c r="AL25" s="31" t="s">
+        <v>322</v>
+      </c>
       <c r="AM25" s="25"/>
       <c r="AN25" s="25"/>
       <c r="AO25" s="26"/>
@@ -33617,6 +33641,45 @@
       <c r="AN674" s="25"/>
       <c r="AO674" s="26"/>
     </row>
+    <row r="675" spans="3:41" x14ac:dyDescent="0.25">
+      <c r="C675" s="22"/>
+      <c r="F675" s="25"/>
+      <c r="G675" s="25"/>
+      <c r="H675" s="25"/>
+      <c r="I675" s="25"/>
+      <c r="J675" s="25"/>
+      <c r="K675" s="25"/>
+      <c r="L675" s="25"/>
+      <c r="M675" s="25"/>
+      <c r="N675" s="25"/>
+      <c r="O675" s="25"/>
+      <c r="P675" s="25"/>
+      <c r="Q675" s="25"/>
+      <c r="R675" s="25"/>
+      <c r="S675" s="25"/>
+      <c r="T675" s="25"/>
+      <c r="U675" s="25"/>
+      <c r="V675" s="25"/>
+      <c r="W675" s="25"/>
+      <c r="X675" s="25"/>
+      <c r="Y675" s="25"/>
+      <c r="Z675" s="25"/>
+      <c r="AA675" s="25"/>
+      <c r="AB675" s="25"/>
+      <c r="AC675" s="25"/>
+      <c r="AD675" s="25"/>
+      <c r="AE675" s="25"/>
+      <c r="AF675" s="25"/>
+      <c r="AG675" s="25"/>
+      <c r="AH675" s="25"/>
+      <c r="AI675" s="25"/>
+      <c r="AJ675" s="25"/>
+      <c r="AK675" s="25"/>
+      <c r="AL675" s="25"/>
+      <c r="AM675" s="25"/>
+      <c r="AN675" s="25"/>
+      <c r="AO675" s="26"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="17" priority="17"/>
@@ -33641,19 +33704,19 @@
     <cfRule type="duplicateValues" dxfId="8" priority="7"/>
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A21:A22">
+  <conditionalFormatting sqref="A21:A23">
     <cfRule type="duplicateValues" dxfId="6" priority="5"/>
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23">
+  <conditionalFormatting sqref="A24">
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24">
+  <conditionalFormatting sqref="A25">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A25:A1048576 A2:A4">
+  <conditionalFormatting sqref="A26:A1048576 A2:A4">
     <cfRule type="duplicateValues" dxfId="0" priority="24"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>

</xml_diff>

<commit_message>
- also add V_ScenName into xml file names if it's not "Standard" - add formula to generate V_ScenName into Excel file
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC38095-7901-4065-94B6-9396BD1A4B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67931BF6-9F0A-4183-8546-25BF96C6E001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
     <definedName name="V_Projektname">Config!$B$21</definedName>
     <definedName name="V_Projektverzeichnis">Config!$B$20</definedName>
     <definedName name="V_Scenario">Config!$B$16</definedName>
-    <definedName name="V_ScenDetail">#REF!</definedName>
+    <definedName name="V_ScenDetail">Macro!$E$3:$BB$44</definedName>
     <definedName name="V_ScenName">Config!$C$16</definedName>
     <definedName name="V_TemplatePath">Config!$B$27</definedName>
     <definedName name="V_Variablen">#REF!</definedName>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="331">
   <si>
     <t>Make script</t>
   </si>
@@ -2500,10 +2500,11 @@
         <v>14</v>
       </c>
       <c r="B16" s="7">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>15</v>
+        <v>2</v>
+      </c>
+      <c r="C16" s="1" t="str">
+        <f>HLOOKUP(V_Scenario,V_ScenDetail,2,FALSE)</f>
+        <v>Scenario 2</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>16</v>
@@ -4152,9 +4153,7 @@
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
       <c r="E15" s="14"/>
-      <c r="F15" s="14" t="s">
-        <v>249</v>
-      </c>
+      <c r="F15" s="14"/>
       <c r="G15" s="14"/>
       <c r="H15" s="14"/>
       <c r="I15" s="14"/>

</xml_diff>

<commit_message>
add possibility to select `RowVar`s with tidyselect selection helpers by adding the prefix "ts: " in the RowVar field (see the cell Questions!G6 in the mapping file for an example)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67931BF6-9F0A-4183-8546-25BF96C6E001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9761970-16E6-44B0-99B6-4EB18A65C5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -1007,9 +1007,6 @@
     <t xml:space="preserve">q1 </t>
   </si>
   <si>
-    <t xml:space="preserve">q2_01 q2_02 q2_03 q2_04 q2_05 q2_06 q2_07 </t>
-  </si>
-  <si>
     <t>q2_99 q2_00</t>
   </si>
   <si>
@@ -1203,6 +1200,9 @@
   </si>
   <si>
     <t>q2_02 q2_01</t>
+  </si>
+  <si>
+    <t>ts: dplyr::matches("q2_\\d+$") &amp; -c(q2_00, q2_99) &amp; where(\(x) length(unique(x)) &gt; 1)</t>
   </si>
 </sst>
 </file>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="33" t="s">
+        <v>275</v>
+      </c>
+      <c r="B23" s="33" t="s">
         <v>276</v>
-      </c>
-      <c r="B23" s="33" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2641,7 +2641,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B35" s="34">
         <v>-2</v>
@@ -3216,7 +3216,7 @@
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>149</v>
@@ -3228,7 +3228,7 @@
         <v>151</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F5" s="29" t="str">
         <f>E5</f>
@@ -6848,13 +6848,13 @@
         <v>223</v>
       </c>
       <c r="C1" s="28" t="s">
+        <v>268</v>
+      </c>
+      <c r="D1" s="28" t="s">
         <v>269</v>
       </c>
-      <c r="D1" s="28" t="s">
+      <c r="E1" s="28" t="s">
         <v>270</v>
-      </c>
-      <c r="E1" s="28" t="s">
-        <v>271</v>
       </c>
       <c r="F1" s="28" t="s">
         <v>224</v>
@@ -6884,10 +6884,10 @@
         <v>244</v>
       </c>
       <c r="O1" s="28" t="s">
+        <v>271</v>
+      </c>
+      <c r="P1" s="28" t="s">
         <v>272</v>
-      </c>
-      <c r="P1" s="28" t="s">
-        <v>273</v>
       </c>
       <c r="Q1" s="28" t="s">
         <v>245</v>
@@ -6914,7 +6914,7 @@
         <v>202</v>
       </c>
       <c r="Y1" s="28" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="Z1" s="28" t="s">
         <v>232</v>
@@ -7152,10 +7152,10 @@
         <v>253</v>
       </c>
       <c r="G6" s="31" t="s">
+        <v>330</v>
+      </c>
+      <c r="H6" s="31" t="s">
         <v>265</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>266</v>
       </c>
       <c r="I6" s="31"/>
       <c r="J6" s="31"/>
@@ -7175,7 +7175,7 @@
       <c r="X6" s="25"/>
       <c r="Y6" s="25"/>
       <c r="Z6" s="25" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
@@ -7208,10 +7208,10 @@
         <v>238</v>
       </c>
       <c r="G7" s="31" t="s">
+        <v>266</v>
+      </c>
+      <c r="H7" s="31" t="s">
         <v>267</v>
-      </c>
-      <c r="H7" s="31" t="s">
-        <v>268</v>
       </c>
       <c r="I7" s="31"/>
       <c r="J7" s="31"/>
@@ -7266,10 +7266,10 @@
         <v>237</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H8" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I8" s="31"/>
       <c r="J8" s="31"/>
@@ -7277,7 +7277,7 @@
       <c r="L8" s="31"/>
       <c r="M8" s="31"/>
       <c r="N8" s="31" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O8" s="25"/>
       <c r="P8" s="31"/>
@@ -7324,20 +7324,20 @@
         <v>237</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
       <c r="L9" s="31" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="M9" s="31"/>
       <c r="N9" s="31" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
@@ -7384,10 +7384,10 @@
         <v>238</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H10" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="31"/>
@@ -7413,13 +7413,13 @@
       <c r="AB10" s="25"/>
       <c r="AC10" s="25"/>
       <c r="AD10" s="14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="AE10" s="25"/>
       <c r="AF10" s="25"/>
       <c r="AG10" s="25"/>
       <c r="AH10" s="25" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AI10" s="25"/>
       <c r="AJ10" s="25"/>
@@ -7444,10 +7444,10 @@
         <v>238</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I11" s="31"/>
       <c r="J11" s="31"/>
@@ -7455,7 +7455,7 @@
       <c r="L11" s="31"/>
       <c r="M11" s="31"/>
       <c r="N11" s="31" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O11" s="25"/>
       <c r="P11" s="31"/>
@@ -7506,10 +7506,10 @@
         <v>237</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I12" s="31"/>
       <c r="J12" s="31"/>
@@ -7517,7 +7517,7 @@
       <c r="L12" s="31"/>
       <c r="M12" s="31"/>
       <c r="N12" s="31" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O12" s="25"/>
       <c r="P12" s="31"/>
@@ -7557,7 +7557,7 @@
         <v>Q4</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
@@ -7566,22 +7566,22 @@
         <v>237</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I13" s="31"/>
       <c r="J13" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="K13" s="31" t="s">
         <v>285</v>
-      </c>
-      <c r="K13" s="31" t="s">
-        <v>286</v>
       </c>
       <c r="L13" s="31"/>
       <c r="M13" s="31"/>
       <c r="N13" s="31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O13" s="25"/>
       <c r="P13" s="31"/>
@@ -7631,7 +7631,7 @@
         <v>257</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
@@ -7645,7 +7645,7 @@
         <v>258</v>
       </c>
       <c r="R14" s="31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="S14" s="31"/>
       <c r="T14" s="31"/>
@@ -7703,7 +7703,7 @@
         <v>258</v>
       </c>
       <c r="R15" s="31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="S15" s="25"/>
       <c r="T15" s="25"/>
@@ -7727,7 +7727,7 @@
       <c r="AL15" s="25"/>
       <c r="AM15" s="25"/>
       <c r="AN15" s="25" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AO15" s="26"/>
     </row>
@@ -7737,7 +7737,7 @@
         <v>Q6</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="30"/>
@@ -7746,10 +7746,10 @@
         <v>238</v>
       </c>
       <c r="G16" s="31" t="s">
+        <v>294</v>
+      </c>
+      <c r="H16" s="31" t="s">
         <v>295</v>
-      </c>
-      <c r="H16" s="31" t="s">
-        <v>296</v>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
@@ -7785,7 +7785,7 @@
       <c r="AJ16" s="25"/>
       <c r="AK16" s="25"/>
       <c r="AL16" s="31" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="AM16" s="25"/>
       <c r="AN16" s="25"/>
@@ -7797,7 +7797,7 @@
         <v>Q6</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -7806,17 +7806,17 @@
         <v>237</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I17" s="31"/>
       <c r="J17" s="31" t="s">
+        <v>301</v>
+      </c>
+      <c r="K17" s="31" t="s">
         <v>302</v>
-      </c>
-      <c r="K17" s="31" t="s">
-        <v>303</v>
       </c>
       <c r="L17" s="31"/>
       <c r="M17" s="31"/>
@@ -7855,24 +7855,24 @@
         <v>Q9</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
       <c r="E18" s="30"/>
       <c r="F18" s="31"/>
       <c r="G18" s="31" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I18" s="31"/>
       <c r="J18" s="31" t="s">
+        <v>304</v>
+      </c>
+      <c r="K18" s="31" t="s">
         <v>305</v>
-      </c>
-      <c r="K18" s="31" t="s">
-        <v>306</v>
       </c>
       <c r="L18" s="31"/>
       <c r="M18" s="31"/>
@@ -7882,10 +7882,10 @@
       <c r="Q18" s="31"/>
       <c r="R18" s="31"/>
       <c r="S18" s="31" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="T18" s="31" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
@@ -7915,24 +7915,24 @@
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
       <c r="E19" s="30"/>
       <c r="F19" s="31"/>
       <c r="G19" s="31" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I19" s="31"/>
       <c r="J19" s="31" t="s">
+        <v>304</v>
+      </c>
+      <c r="K19" s="31" t="s">
         <v>305</v>
-      </c>
-      <c r="K19" s="31" t="s">
-        <v>306</v>
       </c>
       <c r="L19" s="31"/>
       <c r="M19" s="31"/>
@@ -7942,10 +7942,10 @@
       <c r="Q19" s="31"/>
       <c r="R19" s="31"/>
       <c r="S19" s="31" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="T19" s="31" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="U19" s="25"/>
       <c r="V19" s="25"/>
@@ -7975,7 +7975,7 @@
         <v>Q9</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -7984,17 +7984,17 @@
         <v>237</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I20" s="31"/>
       <c r="J20" s="31" t="s">
+        <v>304</v>
+      </c>
+      <c r="K20" s="31" t="s">
         <v>305</v>
-      </c>
-      <c r="K20" s="31" t="s">
-        <v>306</v>
       </c>
       <c r="L20" s="31"/>
       <c r="M20" s="31"/>
@@ -8004,10 +8004,10 @@
       <c r="Q20" s="31"/>
       <c r="R20" s="31"/>
       <c r="S20" s="31" t="s">
+        <v>308</v>
+      </c>
+      <c r="T20" s="31" t="s">
         <v>309</v>
-      </c>
-      <c r="T20" s="31" t="s">
-        <v>310</v>
       </c>
       <c r="U20" s="25"/>
       <c r="V20" s="25"/>
@@ -8037,7 +8037,7 @@
         <v>QNOT CHECKED: 2</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
@@ -8046,7 +8046,7 @@
         <v>253</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H21" s="31"/>
       <c r="I21" s="31"/>
@@ -8060,10 +8060,10 @@
       <c r="Q21" s="31"/>
       <c r="R21" s="31"/>
       <c r="S21" s="31" t="s">
+        <v>308</v>
+      </c>
+      <c r="T21" s="31" t="s">
         <v>309</v>
-      </c>
-      <c r="T21" s="31" t="s">
-        <v>310</v>
       </c>
       <c r="U21" s="25"/>
       <c r="V21" s="25"/>
@@ -8071,7 +8071,7 @@
       <c r="X21" s="25"/>
       <c r="Y21" s="25"/>
       <c r="Z21" s="25" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AA21" s="25"/>
       <c r="AB21" s="25"/>
@@ -8095,7 +8095,7 @@
         <v>Qmulti selvar with unguelt: 2</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -8104,10 +8104,10 @@
         <v>253</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -8120,10 +8120,10 @@
       <c r="Q22" s="31"/>
       <c r="R22" s="31"/>
       <c r="S22" s="31" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="T22" s="31" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U22" s="25"/>
       <c r="V22" s="25"/>
@@ -8153,7 +8153,7 @@
         <v>Qtrigger invalid values: 2</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
@@ -8162,10 +8162,10 @@
         <v>253</v>
       </c>
       <c r="G23" s="31" t="s">
+        <v>328</v>
+      </c>
+      <c r="H23" s="31" t="s">
         <v>329</v>
-      </c>
-      <c r="H23" s="31" t="s">
-        <v>330</v>
       </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
@@ -8207,7 +8207,7 @@
         <v>QNOT CHECKED: 5</v>
       </c>
       <c r="B24" s="30" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -8216,10 +8216,10 @@
         <v>256</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H24" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I24" s="31"/>
       <c r="J24" s="31"/>
@@ -8233,13 +8233,13 @@
         <v>258</v>
       </c>
       <c r="R24" s="31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="S24" s="31" t="s">
+        <v>308</v>
+      </c>
+      <c r="T24" s="31" t="s">
         <v>309</v>
-      </c>
-      <c r="T24" s="31" t="s">
-        <v>310</v>
       </c>
       <c r="U24" s="25"/>
       <c r="V24" s="25"/>
@@ -8269,7 +8269,7 @@
         <v>Q7</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C25" s="30"/>
       <c r="D25" s="30"/>
@@ -8278,32 +8278,32 @@
         <v>238</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I25" s="31"/>
       <c r="J25" s="31" t="s">
+        <v>318</v>
+      </c>
+      <c r="K25" s="31" t="s">
         <v>319</v>
-      </c>
-      <c r="K25" s="31" t="s">
-        <v>320</v>
       </c>
       <c r="L25" s="31"/>
       <c r="M25" s="31"/>
       <c r="N25" s="31" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="O25" s="25"/>
       <c r="P25" s="31"/>
       <c r="Q25" s="31"/>
       <c r="R25" s="31"/>
       <c r="S25" s="31" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="T25" s="31" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="U25" s="25"/>
       <c r="V25" s="25"/>
@@ -8323,7 +8323,7 @@
       <c r="AJ25" s="25"/>
       <c r="AK25" s="25"/>
       <c r="AL25" s="31" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AM25" s="25"/>
       <c r="AN25" s="25"/>

</xml_diff>

<commit_message>
check if the sum of all mw variables = 100 %, if: - In a column "Checks" in the Questions sheet, there is the attribute "100percent" in the respective row - if the check passes, a column "TabDetails" with the value "100percent" is added to the Tab table - a warning is printed, if there are cases where the sum is not equal to 100 (except cases which are = -2 in all variables)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9761970-16E6-44B0-99B6-4EB18A65C5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892C7EDA-DF54-4FA8-A20E-8773434778D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="333">
   <si>
     <t>Make script</t>
   </si>
@@ -1203,6 +1203,12 @@
   </si>
   <si>
     <t>ts: dplyr::matches("q2_\\d+$") &amp; -c(q2_00, q2_99) &amp; where(\(x) length(unique(x)) &gt; 1)</t>
+  </si>
+  <si>
+    <t>Checks</t>
+  </si>
+  <si>
+    <t>100percent</t>
   </si>
 </sst>
 </file>
@@ -6961,6 +6967,9 @@
       <c r="AN1" s="28" t="s">
         <v>262</v>
       </c>
+      <c r="AO1" s="24" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A2" s="19"/>
@@ -7249,7 +7258,9 @@
       <c r="AL7" s="25"/>
       <c r="AM7" s="25"/>
       <c r="AN7" s="25"/>
-      <c r="AO7" s="26"/>
+      <c r="AO7" s="26" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="str">

</xml_diff>

<commit_message>
put NA (instead of 0) in crosstab cells where (M)Statistics are calculated for rowvar & Colvar/colval combinations not occurring in the data
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892C7EDA-DF54-4FA8-A20E-8773434778D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B600E8-C344-43CD-A6EC-960EEF235A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,8 +50,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -210,7 +208,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="334">
   <si>
     <t>Make script</t>
   </si>
@@ -1210,6 +1208,9 @@
   <si>
     <t>100percent</t>
   </si>
+  <si>
+    <t>q3a_NA q3b</t>
+  </si>
 </sst>
 </file>
 
@@ -2003,11 +2004,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Hinweis"/>
       <sheetName val="R"/>
@@ -7395,7 +7393,7 @@
         <v>238</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>279</v>
+        <v>333</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>267</v>

</xml_diff>

<commit_message>
use new format in mapping macro sheet: invalid values in row "Invalid" (TODO: no ranges allowed yet)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B600E8-C344-43CD-A6EC-960EEF235A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207905FF-BB92-4BF3-B824-80175ED26BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
     <definedName name="V_Projektname">Config!$B$21</definedName>
     <definedName name="V_Projektverzeichnis">Config!$B$20</definedName>
     <definedName name="V_Scenario">Config!$B$16</definedName>
-    <definedName name="V_ScenDetail">Macro!$E$3:$BB$44</definedName>
+    <definedName name="V_ScenDetail">Macro!$E$3:$BB$42</definedName>
     <definedName name="V_ScenName">Config!$C$16</definedName>
     <definedName name="V_TemplatePath">Config!$B$27</definedName>
     <definedName name="V_Variablen">#REF!</definedName>
@@ -208,7 +208,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="331">
   <si>
     <t>Make script</t>
   </si>
@@ -675,19 +675,7 @@
     <t>-1,-2,-999/-199</t>
   </si>
   <si>
-    <t>Miss2</t>
-  </si>
-  <si>
-    <t>Invalid value 2</t>
-  </si>
-  <si>
     <t>x</t>
-  </si>
-  <si>
-    <t>Miss3</t>
-  </si>
-  <si>
-    <t>Invalid value 3</t>
   </si>
   <si>
     <t>Overall filter</t>
@@ -925,9 +913,6 @@
   </si>
   <si>
     <t>mw</t>
-  </si>
-  <si>
-    <t>Miss1</t>
   </si>
   <si>
     <t>RowVar</t>
@@ -1211,6 +1196,12 @@
   <si>
     <t>q3a_NA q3b</t>
   </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>-1,-3,-2</t>
+  </si>
 </sst>
 </file>
 
@@ -1412,7 +1403,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1462,6 +1453,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1767,13 +1759,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>390600</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>132945</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>117000</xdr:colOff>
-      <xdr:row>36</xdr:row>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2495,7 +2487,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="E15" s="10"/>
     </row>
@@ -2559,10 +2551,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="33" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2645,7 +2637,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B35" s="34">
         <v>-2</v>
@@ -2732,7 +2724,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AMJ44"/>
+  <dimension ref="A1:AMJ42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="15" customWidth="1"/>
@@ -3220,7 +3212,7 @@
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B5" s="20" t="s">
         <v>149</v>
@@ -3232,7 +3224,7 @@
         <v>151</v>
       </c>
       <c r="E5" s="29" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="F5" s="29" t="str">
         <f>E5</f>
@@ -3290,7 +3282,7 @@
     </row>
     <row r="6" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>239</v>
+        <v>329</v>
       </c>
       <c r="B6" s="20" t="s">
         <v>152</v>
@@ -3301,161 +3293,161 @@
       <c r="D6" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="E6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="F6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="G6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="H6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="I6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="J6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="K6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="L6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="M6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="N6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="O6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="P6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="Q6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="R6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="S6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="T6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="U6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="V6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="W6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="X6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="Y6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="Z6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AA6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AB6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AC6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AD6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AE6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AF6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AG6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AH6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AI6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AJ6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AK6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AL6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AM6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AN6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AO6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AP6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AQ6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AR6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AS6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AT6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AU6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AV6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AW6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AX6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AY6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="AZ6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="BA6" s="14">
-        <v>-1</v>
-      </c>
-      <c r="BB6" s="14">
-        <v>-1</v>
+      <c r="E6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="F6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="G6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="H6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="I6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="J6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="K6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="L6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="M6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="N6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="O6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="P6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="Q6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="R6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="S6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="T6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="U6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="V6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="W6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="X6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="Y6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="Z6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AA6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AB6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AC6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AD6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AE6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AF6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AG6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AH6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AI6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AJ6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AK6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AL6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AM6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AN6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AO6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AP6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AQ6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AR6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AS6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AT6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AU6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AV6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AW6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AX6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AY6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="AZ6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="BA6" s="37" t="s">
+        <v>330</v>
+      </c>
+      <c r="BB6" s="37" t="s">
+        <v>330</v>
       </c>
       <c r="BD6" s="19"/>
     </row>
     <row r="7" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
-        <v>155</v>
+        <v>221</v>
       </c>
       <c r="B7" s="20" t="s">
         <v>156</v>
@@ -3463,334 +3455,128 @@
       <c r="C7" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="D7" s="20"/>
-      <c r="E7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="F7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="G7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="H7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="I7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="J7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="K7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="L7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="M7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="N7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="O7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="P7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="Q7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="R7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="S7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="T7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="U7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="V7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="W7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="X7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="Y7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="Z7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AA7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AB7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AC7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AD7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AE7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AF7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AG7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AH7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AI7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AJ7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AK7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AL7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AM7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AN7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AO7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AP7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AQ7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AR7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AS7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AT7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AU7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AV7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AW7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AX7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AY7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="AZ7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="BA7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="BB7" s="14">
-        <v>-3</v>
-      </c>
+      <c r="D7" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="14"/>
+      <c r="AA7" s="14"/>
+      <c r="AB7" s="14"/>
+      <c r="AC7" s="14"/>
+      <c r="AD7" s="14"/>
+      <c r="AE7" s="14"/>
+      <c r="AF7" s="14"/>
+      <c r="AG7" s="14"/>
+      <c r="AH7" s="14"/>
+      <c r="AI7" s="14"/>
+      <c r="AJ7" s="14"/>
+      <c r="AK7" s="14"/>
+      <c r="AL7" s="14"/>
+      <c r="AM7" s="14"/>
+      <c r="AN7" s="14"/>
+      <c r="AO7" s="14"/>
+      <c r="AP7" s="14"/>
+      <c r="AQ7" s="14"/>
+      <c r="AR7" s="14"/>
+      <c r="AS7" s="14"/>
+      <c r="AT7" s="14"/>
+      <c r="AU7" s="14"/>
+      <c r="AV7" s="14"/>
+      <c r="AW7" s="14"/>
+      <c r="AX7" s="14"/>
+      <c r="AY7" s="14"/>
+      <c r="AZ7" s="14"/>
+      <c r="BA7" s="14"/>
+      <c r="BB7" s="14"/>
       <c r="BD7" s="19"/>
     </row>
     <row r="8" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>158</v>
-      </c>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="14"/>
+      <c r="S8" s="14"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14"/>
+      <c r="X8" s="14"/>
+      <c r="Y8" s="14"/>
+      <c r="Z8" s="14"/>
+      <c r="AA8" s="14"/>
+      <c r="AB8" s="14"/>
+      <c r="AC8" s="14"/>
+      <c r="AD8" s="14"/>
+      <c r="AE8" s="14"/>
+      <c r="AF8" s="14"/>
+      <c r="AG8" s="14"/>
+      <c r="AH8" s="14"/>
+      <c r="AI8" s="14"/>
+      <c r="AJ8" s="14"/>
+      <c r="AK8" s="14"/>
+      <c r="AL8" s="14"/>
+      <c r="AM8" s="14"/>
+      <c r="AN8" s="14"/>
+      <c r="AO8" s="14"/>
+      <c r="AP8" s="14"/>
+      <c r="AQ8" s="14"/>
+      <c r="AR8" s="14"/>
+      <c r="AS8" s="14"/>
+      <c r="AT8" s="14"/>
+      <c r="AU8" s="14"/>
+      <c r="AV8" s="14"/>
+      <c r="AW8" s="14"/>
+      <c r="AX8" s="14"/>
+      <c r="AY8" s="14"/>
+      <c r="AZ8" s="14"/>
+      <c r="BA8" s="14"/>
+      <c r="BB8" s="14"/>
+      <c r="BD8" s="19"/>
+    </row>
+    <row r="9" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
         <v>159</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" s="20"/>
-      <c r="E8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="F8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="G8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="H8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="I8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="J8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="K8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="L8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="M8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="N8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="O8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="P8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="Q8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="R8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="S8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="T8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="U8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="V8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="W8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="X8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="Y8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="Z8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AA8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AB8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AC8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AD8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AE8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AF8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AG8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AH8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AI8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AJ8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AK8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AL8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AM8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AN8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AO8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AP8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AQ8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AR8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AS8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AT8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AU8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AV8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AW8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AX8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AY8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="AZ8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="BA8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="BB8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="BD8" s="19"/>
-    </row>
-    <row r="9" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>225</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="20"/>
+      <c r="D9" s="20" t="s">
         <v>161</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>162</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
@@ -3845,9 +3631,13 @@
       <c r="BD9" s="19"/>
     </row>
     <row r="10" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A10" s="20"/>
+      <c r="A10" s="20" t="s">
+        <v>162</v>
+      </c>
       <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="C10" s="20" t="s">
+        <v>155</v>
+      </c>
       <c r="D10" s="20"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
@@ -3902,16 +3692,14 @@
       <c r="BD10" s="19"/>
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="21" t="s">
         <v>163</v>
       </c>
       <c r="B11" s="20" t="s">
         <v>164</v>
       </c>
       <c r="C11" s="20"/>
-      <c r="D11" s="20" t="s">
-        <v>165</v>
-      </c>
+      <c r="D11" s="20"/>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="14"/>
@@ -3966,11 +3754,11 @@
     </row>
     <row r="12" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="14"/>
@@ -4026,11 +3814,11 @@
       <c r="BD12" s="19"/>
     </row>
     <row r="13" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>167</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>168</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="20"/>
@@ -4088,13 +3876,15 @@
     </row>
     <row r="14" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D14" s="20"/>
+        <v>155</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>169</v>
+      </c>
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
       <c r="G14" s="14"/>
@@ -4148,7 +3938,7 @@
       <c r="BD14" s="19"/>
     </row>
     <row r="15" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="21" t="s">
         <v>170</v>
       </c>
       <c r="B15" s="20" t="s">
@@ -4209,300 +3999,398 @@
       <c r="BD15" s="19"/>
     </row>
     <row r="16" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="B16" s="20"/>
+      <c r="B16" s="20" t="s">
+        <v>173</v>
+      </c>
       <c r="C16" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D16" s="20" t="s">
-        <v>173</v>
-      </c>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="14"/>
-      <c r="R16" s="14"/>
-      <c r="S16" s="14"/>
-      <c r="T16" s="14"/>
-      <c r="U16" s="14"/>
-      <c r="V16" s="14"/>
-      <c r="W16" s="14"/>
-      <c r="X16" s="14"/>
-      <c r="Y16" s="14"/>
-      <c r="Z16" s="14"/>
-      <c r="AA16" s="14"/>
-      <c r="AB16" s="14"/>
-      <c r="AC16" s="14"/>
-      <c r="AD16" s="14"/>
-      <c r="AE16" s="14"/>
-      <c r="AF16" s="14"/>
-      <c r="AG16" s="14"/>
-      <c r="AH16" s="14"/>
-      <c r="AI16" s="14"/>
-      <c r="AJ16" s="14"/>
-      <c r="AK16" s="14"/>
-      <c r="AL16" s="14"/>
-      <c r="AM16" s="14"/>
-      <c r="AN16" s="14"/>
-      <c r="AO16" s="14"/>
-      <c r="AP16" s="14"/>
-      <c r="AQ16" s="14"/>
-      <c r="AR16" s="14"/>
-      <c r="AS16" s="14"/>
-      <c r="AT16" s="14"/>
-      <c r="AU16" s="14"/>
-      <c r="AV16" s="14"/>
-      <c r="AW16" s="14"/>
-      <c r="AX16" s="14"/>
-      <c r="AY16" s="14"/>
-      <c r="AZ16" s="14"/>
-      <c r="BA16" s="14"/>
-      <c r="BB16" s="14"/>
+        <v>174</v>
+      </c>
+      <c r="D16" s="20"/>
+      <c r="E16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="L16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="M16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="N16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="O16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="P16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="R16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="S16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="T16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="U16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="V16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="W16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="X16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="Y16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="Z16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AA16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AB16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AC16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AD16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AE16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AF16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AG16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AH16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AI16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AJ16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AK16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AL16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AM16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AN16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AO16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AP16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AQ16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AR16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AS16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AT16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AU16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AV16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AW16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AX16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AY16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="AZ16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="BA16" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="BB16" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="BD16" s="19"/>
     </row>
     <row r="17" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="C17" s="20"/>
+      <c r="A17" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20" t="s">
+        <v>155</v>
+      </c>
       <c r="D17" s="20"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="14"/>
-      <c r="R17" s="14"/>
-      <c r="S17" s="14"/>
-      <c r="T17" s="14"/>
-      <c r="U17" s="14"/>
-      <c r="V17" s="14"/>
-      <c r="W17" s="14"/>
-      <c r="X17" s="14"/>
-      <c r="Y17" s="14"/>
-      <c r="Z17" s="14"/>
-      <c r="AA17" s="14"/>
-      <c r="AB17" s="14"/>
-      <c r="AC17" s="14"/>
-      <c r="AD17" s="14"/>
-      <c r="AE17" s="14"/>
-      <c r="AF17" s="14"/>
-      <c r="AG17" s="14"/>
-      <c r="AH17" s="14"/>
-      <c r="AI17" s="14"/>
-      <c r="AJ17" s="14"/>
-      <c r="AK17" s="14"/>
-      <c r="AL17" s="14"/>
-      <c r="AM17" s="14"/>
-      <c r="AN17" s="14"/>
-      <c r="AO17" s="14"/>
-      <c r="AP17" s="14"/>
-      <c r="AQ17" s="14"/>
-      <c r="AR17" s="14"/>
-      <c r="AS17" s="14"/>
-      <c r="AT17" s="14"/>
-      <c r="AU17" s="14"/>
-      <c r="AV17" s="14"/>
-      <c r="AW17" s="14"/>
-      <c r="AX17" s="14"/>
-      <c r="AY17" s="14"/>
-      <c r="AZ17" s="14"/>
-      <c r="BA17" s="14"/>
-      <c r="BB17" s="14"/>
+      <c r="E17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="G17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="M17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="O17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="P17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="R17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="S17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="T17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="U17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="V17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="W17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="X17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="Y17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AA17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AD17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AE17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AG17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AH17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AI17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AJ17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AK17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AM17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AN17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AP17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AQ17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AS17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AT17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AU17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AV17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AW17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AX17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AY17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="AZ17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="BA17" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="BB17" s="14" t="s">
+        <v>177</v>
+      </c>
       <c r="BD17" s="19"/>
     </row>
     <row r="18" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>177</v>
-      </c>
+      <c r="A18" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="B18" s="20"/>
       <c r="C18" s="20" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="D18" s="20"/>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+      <c r="S18" s="14"/>
+      <c r="T18" s="14"/>
+      <c r="U18" s="14"/>
+      <c r="V18" s="14"/>
+      <c r="W18" s="14"/>
+      <c r="X18" s="14"/>
+      <c r="Y18" s="14"/>
+      <c r="Z18" s="14"/>
+      <c r="AA18" s="14"/>
+      <c r="AB18" s="14"/>
+      <c r="AC18" s="14"/>
+      <c r="AD18" s="14"/>
+      <c r="AE18" s="14"/>
+      <c r="AF18" s="14"/>
+      <c r="AG18" s="14"/>
+      <c r="AH18" s="14"/>
+      <c r="AI18" s="14"/>
+      <c r="AJ18" s="14"/>
+      <c r="AK18" s="14"/>
+      <c r="AL18" s="14"/>
+      <c r="AM18" s="14"/>
+      <c r="AN18" s="14"/>
+      <c r="AO18" s="14"/>
+      <c r="AP18" s="14"/>
+      <c r="AQ18" s="14"/>
+      <c r="AR18" s="14"/>
+      <c r="AS18" s="14"/>
+      <c r="AT18" s="14"/>
+      <c r="AU18" s="14"/>
+      <c r="AV18" s="14"/>
+      <c r="AW18" s="14"/>
+      <c r="AX18" s="14"/>
+      <c r="AY18" s="14"/>
+      <c r="AZ18" s="14"/>
+      <c r="BA18" s="14"/>
+      <c r="BB18" s="14"/>
+      <c r="BD18" s="19"/>
+    </row>
+    <row r="19" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A19" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="F18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="J18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="K18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="L18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="M18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="N18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="O18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="P18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="Q18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="R18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="S18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="T18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="U18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="V18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="W18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="X18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="Z18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AA18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AB18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AC18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AD18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AE18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AF18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AG18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AI18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AJ18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AK18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AL18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AM18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AN18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AO18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AP18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AQ18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AR18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AS18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AT18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AU18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AV18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AW18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AX18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AY18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="AZ18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="BA18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="BB18" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="BD18" s="19"/>
-    </row>
-    <row r="19" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A19" s="20" t="s">
+      <c r="B19" s="20" t="s">
         <v>180</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20" t="s">
-        <v>157</v>
-      </c>
+      <c r="C19" s="20"/>
       <c r="D19" s="20"/>
       <c r="E19" s="14" t="s">
         <v>181</v>
@@ -4660,11 +4548,13 @@
       <c r="A20" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D20" s="20"/>
+      <c r="B20" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20" t="s">
+        <v>184</v>
+      </c>
       <c r="E20" s="14"/>
       <c r="F20" s="14"/>
       <c r="G20" s="14"/>
@@ -4718,177 +4608,75 @@
       <c r="BD20" s="19"/>
     </row>
     <row r="21" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
-        <v>183</v>
-      </c>
-      <c r="B21" s="20" t="s">
-        <v>184</v>
-      </c>
-      <c r="C21" s="20"/>
+      <c r="A21" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20" t="s">
+        <v>155</v>
+      </c>
       <c r="D21" s="20"/>
-      <c r="E21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="K21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="L21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="M21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="N21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="O21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="P21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="R21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="S21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="T21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="U21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="V21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="W21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="X21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="Y21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="Z21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AA21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AB21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AC21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AD21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AE21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AF21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AG21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AH21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AI21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AJ21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AK21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AL21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AM21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AN21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AO21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AP21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AQ21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AR21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AS21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AT21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AU21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AV21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AW21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AX21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AY21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="AZ21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="BA21" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="BB21" s="14" t="s">
-        <v>185</v>
-      </c>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="14"/>
+      <c r="S21" s="14"/>
+      <c r="T21" s="14"/>
+      <c r="U21" s="14"/>
+      <c r="V21" s="14"/>
+      <c r="W21" s="14"/>
+      <c r="X21" s="14"/>
+      <c r="Y21" s="14"/>
+      <c r="Z21" s="14"/>
+      <c r="AA21" s="14"/>
+      <c r="AB21" s="14"/>
+      <c r="AC21" s="14"/>
+      <c r="AD21" s="14"/>
+      <c r="AE21" s="14"/>
+      <c r="AF21" s="14"/>
+      <c r="AG21" s="14"/>
+      <c r="AH21" s="14"/>
+      <c r="AI21" s="14"/>
+      <c r="AJ21" s="14"/>
+      <c r="AK21" s="14"/>
+      <c r="AL21" s="14"/>
+      <c r="AM21" s="14"/>
+      <c r="AN21" s="14"/>
+      <c r="AO21" s="14"/>
+      <c r="AP21" s="14"/>
+      <c r="AQ21" s="14"/>
+      <c r="AR21" s="14"/>
+      <c r="AS21" s="14"/>
+      <c r="AT21" s="14"/>
+      <c r="AU21" s="14"/>
+      <c r="AV21" s="14"/>
+      <c r="AW21" s="14"/>
+      <c r="AX21" s="14"/>
+      <c r="AY21" s="14"/>
+      <c r="AZ21" s="14"/>
+      <c r="BA21" s="14"/>
+      <c r="BB21" s="14"/>
       <c r="BD21" s="19"/>
     </row>
     <row r="22" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="B22" s="20" t="s">
-        <v>187</v>
-      </c>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20" t="s">
-        <v>188</v>
-      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="D22" s="20"/>
       <c r="E22" s="14"/>
       <c r="F22" s="14"/>
       <c r="G22" s="14"/>
@@ -4943,11 +4731,11 @@
     </row>
     <row r="23" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B23" s="20"/>
       <c r="C23" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D23" s="20"/>
       <c r="E23" s="14"/>
@@ -5004,11 +4792,11 @@
     </row>
     <row r="24" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B24" s="20"/>
       <c r="C24" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D24" s="20"/>
       <c r="E24" s="14"/>
@@ -5065,459 +4853,561 @@
     </row>
     <row r="25" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B25" s="20"/>
       <c r="C25" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D25" s="20"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="14"/>
-      <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
-      <c r="R25" s="14"/>
-      <c r="S25" s="14"/>
-      <c r="T25" s="14"/>
-      <c r="U25" s="14"/>
-      <c r="V25" s="14"/>
-      <c r="W25" s="14"/>
-      <c r="X25" s="14"/>
-      <c r="Y25" s="14"/>
-      <c r="Z25" s="14"/>
-      <c r="AA25" s="14"/>
-      <c r="AB25" s="14"/>
-      <c r="AC25" s="14"/>
-      <c r="AD25" s="14"/>
-      <c r="AE25" s="14"/>
-      <c r="AF25" s="14"/>
-      <c r="AG25" s="14"/>
-      <c r="AH25" s="14"/>
-      <c r="AI25" s="14"/>
-      <c r="AJ25" s="14"/>
-      <c r="AK25" s="14"/>
-      <c r="AL25" s="14"/>
-      <c r="AM25" s="14"/>
-      <c r="AN25" s="14"/>
-      <c r="AO25" s="14"/>
-      <c r="AP25" s="14"/>
-      <c r="AQ25" s="14"/>
-      <c r="AR25" s="14"/>
-      <c r="AS25" s="14"/>
-      <c r="AT25" s="14"/>
-      <c r="AU25" s="14"/>
-      <c r="AV25" s="14"/>
-      <c r="AW25" s="14"/>
-      <c r="AX25" s="14"/>
-      <c r="AY25" s="14"/>
-      <c r="AZ25" s="14"/>
-      <c r="BA25" s="14"/>
-      <c r="BB25" s="14"/>
+      <c r="E25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="J25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="K25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="L25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="M25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="N25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="O25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="P25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="R25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="S25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="T25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="U25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="V25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="W25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="X25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="Z25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AA25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AB25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AC25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AD25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AE25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AF25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AG25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AH25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AI25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AJ25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AK25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AL25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AM25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AN25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AO25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AP25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AQ25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AR25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AS25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AT25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AU25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AV25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AW25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AX25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AY25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="AZ25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="BA25" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="BB25" s="14" t="s">
+        <v>190</v>
+      </c>
       <c r="BD25" s="19"/>
     </row>
     <row r="26" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="21" t="s">
+        <v>191</v>
+      </c>
+      <c r="B26" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="B26" s="20"/>
       <c r="C26" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="14"/>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="14"/>
-      <c r="R26" s="14"/>
-      <c r="S26" s="14"/>
-      <c r="T26" s="14"/>
-      <c r="U26" s="14"/>
-      <c r="V26" s="14"/>
-      <c r="W26" s="14"/>
-      <c r="X26" s="14"/>
-      <c r="Y26" s="14"/>
-      <c r="Z26" s="14"/>
-      <c r="AA26" s="14"/>
-      <c r="AB26" s="14"/>
-      <c r="AC26" s="14"/>
-      <c r="AD26" s="14"/>
-      <c r="AE26" s="14"/>
-      <c r="AF26" s="14"/>
-      <c r="AG26" s="14"/>
-      <c r="AH26" s="14"/>
-      <c r="AI26" s="14"/>
-      <c r="AJ26" s="14"/>
-      <c r="AK26" s="14"/>
-      <c r="AL26" s="14"/>
-      <c r="AM26" s="14"/>
-      <c r="AN26" s="14"/>
-      <c r="AO26" s="14"/>
-      <c r="AP26" s="14"/>
-      <c r="AQ26" s="14"/>
-      <c r="AR26" s="14"/>
-      <c r="AS26" s="14"/>
-      <c r="AT26" s="14"/>
-      <c r="AU26" s="14"/>
-      <c r="AV26" s="14"/>
-      <c r="AW26" s="14"/>
-      <c r="AX26" s="14"/>
-      <c r="AY26" s="14"/>
-      <c r="AZ26" s="14"/>
-      <c r="BA26" s="14"/>
-      <c r="BB26" s="14"/>
+        <v>193</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="L26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="M26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="N26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="O26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="P26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="R26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="S26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="T26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="U26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="V26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="W26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="X26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="Y26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="Z26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AA26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AB26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AC26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AD26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AE26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AF26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AG26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AH26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AI26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AJ26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AK26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AL26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AM26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AN26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AO26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AP26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AQ26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AR26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AS26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AT26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AU26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AV26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AW26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AX26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AY26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="AZ26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="BA26" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="BB26" s="14" t="s">
+        <v>195</v>
+      </c>
       <c r="BD26" s="19"/>
     </row>
     <row r="27" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B27" s="20"/>
       <c r="C27" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D27" s="20"/>
       <c r="E27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="K27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="L27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="M27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="N27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="O27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="P27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Q27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="R27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="S27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="T27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="U27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="V27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="W27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="X27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Y27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Z27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AA27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AB27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AC27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AD27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AE27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AF27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AG27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AH27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AI27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AJ27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AK27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AL27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AM27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AN27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AO27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AP27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AQ27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AR27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AS27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AT27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AU27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AV27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AW27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AX27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AY27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="AZ27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="BA27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="BB27" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="BD27" s="19"/>
     </row>
     <row r="28" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A28" s="21" t="s">
-        <v>195</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>196</v>
-      </c>
+      <c r="A28" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="B28" s="20"/>
       <c r="C28" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>198</v>
-      </c>
-      <c r="E28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="I28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="J28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="K28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="L28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="M28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="N28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="O28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="P28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="Q28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="R28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="S28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="T28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="U28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="V28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="W28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="X28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="Y28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="Z28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AA28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AB28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AC28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AD28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AE28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AF28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AG28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AH28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AI28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AJ28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AK28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AL28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AM28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AN28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AO28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AP28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AQ28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AR28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AS28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AT28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AU28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AV28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AW28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AX28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AY28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="AZ28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="BA28" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="BB28" s="14" t="s">
-        <v>199</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="D28" s="20"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="14"/>
+      <c r="N28" s="14"/>
+      <c r="O28" s="14"/>
+      <c r="P28" s="14"/>
+      <c r="Q28" s="14"/>
+      <c r="R28" s="14"/>
+      <c r="S28" s="14"/>
+      <c r="T28" s="14"/>
+      <c r="U28" s="14"/>
+      <c r="V28" s="14"/>
+      <c r="W28" s="14"/>
+      <c r="X28" s="14"/>
+      <c r="Y28" s="14"/>
+      <c r="Z28" s="14"/>
+      <c r="AA28" s="14"/>
+      <c r="AB28" s="14"/>
+      <c r="AC28" s="14"/>
+      <c r="AD28" s="14"/>
+      <c r="AE28" s="14"/>
+      <c r="AF28" s="14"/>
+      <c r="AG28" s="14"/>
+      <c r="AH28" s="14"/>
+      <c r="AI28" s="14"/>
+      <c r="AJ28" s="14"/>
+      <c r="AK28" s="14"/>
+      <c r="AL28" s="14"/>
+      <c r="AM28" s="14"/>
+      <c r="AN28" s="14"/>
+      <c r="AO28" s="14"/>
+      <c r="AP28" s="14"/>
+      <c r="AQ28" s="14"/>
+      <c r="AR28" s="14"/>
+      <c r="AS28" s="14"/>
+      <c r="AT28" s="14"/>
+      <c r="AU28" s="14"/>
+      <c r="AV28" s="14"/>
+      <c r="AW28" s="14"/>
+      <c r="AX28" s="14"/>
+      <c r="AY28" s="14"/>
+      <c r="AZ28" s="14"/>
+      <c r="BA28" s="14"/>
+      <c r="BB28" s="14"/>
       <c r="BD28" s="19"/>
     </row>
     <row r="29" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="B29" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="B29" s="20"/>
       <c r="C29" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D29" s="20"/>
       <c r="E29" s="14" t="s">
@@ -5676,9 +5566,11 @@
       <c r="A30" s="20" t="s">
         <v>202</v>
       </c>
-      <c r="B30" s="20"/>
+      <c r="B30" s="20" t="s">
+        <v>203</v>
+      </c>
       <c r="C30" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D30" s="20"/>
       <c r="E30" s="14"/>
@@ -5735,165 +5627,65 @@
     </row>
     <row r="31" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D31" s="20"/>
-      <c r="E31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="G31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="H31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="I31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="J31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="K31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="L31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="M31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="N31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="O31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="P31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="R31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="S31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="T31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="U31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="V31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="W31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="X31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="Y31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="Z31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AA31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AB31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AC31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AD31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AE31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AF31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AG31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AH31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AI31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AJ31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AK31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AL31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AM31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AN31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AO31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AP31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AQ31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AR31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AS31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AT31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AU31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AV31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AW31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AX31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AY31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="AZ31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="BA31" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="BB31" s="14" t="s">
-        <v>205</v>
-      </c>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
+      <c r="N31" s="14"/>
+      <c r="O31" s="14"/>
+      <c r="P31" s="14"/>
+      <c r="Q31" s="14"/>
+      <c r="R31" s="14"/>
+      <c r="S31" s="14"/>
+      <c r="T31" s="14"/>
+      <c r="U31" s="14"/>
+      <c r="V31" s="14"/>
+      <c r="W31" s="14"/>
+      <c r="X31" s="14"/>
+      <c r="Y31" s="14"/>
+      <c r="Z31" s="14"/>
+      <c r="AA31" s="14"/>
+      <c r="AB31" s="14"/>
+      <c r="AC31" s="14"/>
+      <c r="AD31" s="14"/>
+      <c r="AE31" s="14"/>
+      <c r="AF31" s="14"/>
+      <c r="AG31" s="14"/>
+      <c r="AH31" s="14"/>
+      <c r="AI31" s="14"/>
+      <c r="AJ31" s="14"/>
+      <c r="AK31" s="14"/>
+      <c r="AL31" s="14"/>
+      <c r="AM31" s="14"/>
+      <c r="AN31" s="14"/>
+      <c r="AO31" s="14"/>
+      <c r="AP31" s="14"/>
+      <c r="AQ31" s="14"/>
+      <c r="AR31" s="14"/>
+      <c r="AS31" s="14"/>
+      <c r="AT31" s="14"/>
+      <c r="AU31" s="14"/>
+      <c r="AV31" s="14"/>
+      <c r="AW31" s="14"/>
+      <c r="AX31" s="14"/>
+      <c r="AY31" s="14"/>
+      <c r="AZ31" s="14"/>
+      <c r="BA31" s="14"/>
+      <c r="BB31" s="14"/>
       <c r="BD31" s="19"/>
     </row>
     <row r="32" spans="1:56" x14ac:dyDescent="0.25">
@@ -5901,10 +5693,10 @@
         <v>206</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D32" s="20"/>
       <c r="E32" s="14"/>
@@ -5961,13 +5753,13 @@
     </row>
     <row r="33" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D33" s="20"/>
       <c r="E33" s="14"/>
@@ -6024,13 +5816,13 @@
     </row>
     <row r="34" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D34" s="20"/>
       <c r="E34" s="14"/>
@@ -6087,13 +5879,13 @@
     </row>
     <row r="35" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D35" s="20"/>
       <c r="E35" s="14"/>
@@ -6150,13 +5942,13 @@
     </row>
     <row r="36" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D36" s="20"/>
       <c r="E36" s="14"/>
@@ -6213,13 +6005,13 @@
     </row>
     <row r="37" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A37" s="20" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C37" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D37" s="20"/>
       <c r="E37" s="14"/>
@@ -6276,13 +6068,13 @@
     </row>
     <row r="38" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A38" s="20" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D38" s="20"/>
       <c r="E38" s="14"/>
@@ -6339,13 +6131,13 @@
     </row>
     <row r="39" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D39" s="20"/>
       <c r="E39" s="14"/>
@@ -6402,13 +6194,13 @@
     </row>
     <row r="40" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D40" s="20"/>
       <c r="E40" s="14"/>
@@ -6464,16 +6256,14 @@
       <c r="BD40" s="19"/>
     </row>
     <row r="41" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A41" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="B41" s="20" t="s">
-        <v>209</v>
-      </c>
+      <c r="A41" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="B41" s="14"/>
       <c r="C41" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D41" s="20"/>
+        <v>155</v>
+      </c>
+      <c r="D41" s="14"/>
       <c r="E41" s="14"/>
       <c r="F41" s="14"/>
       <c r="G41" s="14"/>
@@ -6527,285 +6317,161 @@
       <c r="BD41" s="19"/>
     </row>
     <row r="42" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A42" s="20" t="s">
-        <v>218</v>
-      </c>
-      <c r="B42" s="20" t="s">
-        <v>209</v>
+      <c r="A42" s="15" t="s">
+        <v>216</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D42" s="20"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="14"/>
-      <c r="K42" s="14"/>
-      <c r="L42" s="14"/>
-      <c r="M42" s="14"/>
-      <c r="N42" s="14"/>
-      <c r="O42" s="14"/>
-      <c r="P42" s="14"/>
-      <c r="Q42" s="14"/>
-      <c r="R42" s="14"/>
-      <c r="S42" s="14"/>
-      <c r="T42" s="14"/>
-      <c r="U42" s="14"/>
-      <c r="V42" s="14"/>
-      <c r="W42" s="14"/>
-      <c r="X42" s="14"/>
-      <c r="Y42" s="14"/>
-      <c r="Z42" s="14"/>
-      <c r="AA42" s="14"/>
-      <c r="AB42" s="14"/>
-      <c r="AC42" s="14"/>
-      <c r="AD42" s="14"/>
-      <c r="AE42" s="14"/>
-      <c r="AF42" s="14"/>
-      <c r="AG42" s="14"/>
-      <c r="AH42" s="14"/>
-      <c r="AI42" s="14"/>
-      <c r="AJ42" s="14"/>
-      <c r="AK42" s="14"/>
-      <c r="AL42" s="14"/>
-      <c r="AM42" s="14"/>
-      <c r="AN42" s="14"/>
-      <c r="AO42" s="14"/>
-      <c r="AP42" s="14"/>
-      <c r="AQ42" s="14"/>
-      <c r="AR42" s="14"/>
-      <c r="AS42" s="14"/>
-      <c r="AT42" s="14"/>
-      <c r="AU42" s="14"/>
-      <c r="AV42" s="14"/>
-      <c r="AW42" s="14"/>
-      <c r="AX42" s="14"/>
-      <c r="AY42" s="14"/>
-      <c r="AZ42" s="14"/>
-      <c r="BA42" s="14"/>
-      <c r="BB42" s="14"/>
-      <c r="BD42" s="19"/>
-    </row>
-    <row r="43" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>219</v>
-      </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
-      <c r="L43" s="14"/>
-      <c r="M43" s="14"/>
-      <c r="N43" s="14"/>
-      <c r="O43" s="14"/>
-      <c r="P43" s="14"/>
-      <c r="Q43" s="14"/>
-      <c r="R43" s="14"/>
-      <c r="S43" s="14"/>
-      <c r="T43" s="14"/>
-      <c r="U43" s="14"/>
-      <c r="V43" s="14"/>
-      <c r="W43" s="14"/>
-      <c r="X43" s="14"/>
-      <c r="Y43" s="14"/>
-      <c r="Z43" s="14"/>
-      <c r="AA43" s="14"/>
-      <c r="AB43" s="14"/>
-      <c r="AC43" s="14"/>
-      <c r="AD43" s="14"/>
-      <c r="AE43" s="14"/>
-      <c r="AF43" s="14"/>
-      <c r="AG43" s="14"/>
-      <c r="AH43" s="14"/>
-      <c r="AI43" s="14"/>
-      <c r="AJ43" s="14"/>
-      <c r="AK43" s="14"/>
-      <c r="AL43" s="14"/>
-      <c r="AM43" s="14"/>
-      <c r="AN43" s="14"/>
-      <c r="AO43" s="14"/>
-      <c r="AP43" s="14"/>
-      <c r="AQ43" s="14"/>
-      <c r="AR43" s="14"/>
-      <c r="AS43" s="14"/>
-      <c r="AT43" s="14"/>
-      <c r="AU43" s="14"/>
-      <c r="AV43" s="14"/>
-      <c r="AW43" s="14"/>
-      <c r="AX43" s="14"/>
-      <c r="AY43" s="14"/>
-      <c r="AZ43" s="14"/>
-      <c r="BA43" s="14"/>
-      <c r="BB43" s="14"/>
-      <c r="BD43" s="19"/>
-    </row>
-    <row r="44" spans="1:56" x14ac:dyDescent="0.25">
-      <c r="A44" s="15" t="s">
-        <v>220</v>
-      </c>
-      <c r="C44" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="E44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="F44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="G44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="H44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="I44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="J44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="K44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="L44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="M44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="N44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="O44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="P44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="Q44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="R44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="S44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="T44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="U44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="V44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="W44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="X44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="Y44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="Z44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AA44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AB44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AC44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AD44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AE44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AF44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AG44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AH44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AI44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AJ44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AK44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AL44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AM44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AN44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AO44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AP44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AQ44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AR44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AS44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AT44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AU44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AV44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AW44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AX44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AY44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="AZ44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="BA44" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="BB44" s="15" t="s">
-        <v>221</v>
+        <v>155</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="G42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="H42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="I42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="J42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="K42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="L42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="M42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="N42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="O42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="P42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="Q42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="R42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="S42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="T42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="U42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="V42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="W42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="X42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="Y42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="Z42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AA42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AB42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AC42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AD42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AE42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AF42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AG42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AH42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AI42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AJ42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AK42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AL42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AM42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AN42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AO42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AP42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AQ42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AR42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AS42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AT42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AU42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AV42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AW42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AX42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AY42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="AZ42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="BA42" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="BB42" s="15" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -6846,127 +6512,127 @@
   <sheetData>
     <row r="1" spans="1:41" s="24" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="28" t="s">
+        <v>218</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="D1" s="28" t="s">
+        <v>264</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="F1" s="28" t="s">
+        <v>220</v>
+      </c>
+      <c r="G1" s="32" t="s">
+        <v>235</v>
+      </c>
+      <c r="H1" s="28" t="s">
+        <v>236</v>
+      </c>
+      <c r="I1" s="28" t="s">
+        <v>221</v>
+      </c>
+      <c r="J1" s="28" t="s">
         <v>222</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="K1" s="28" t="s">
         <v>223</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="L1" s="28" t="s">
+        <v>237</v>
+      </c>
+      <c r="M1" s="28" t="s">
+        <v>238</v>
+      </c>
+      <c r="N1" s="28" t="s">
+        <v>239</v>
+      </c>
+      <c r="O1" s="28" t="s">
+        <v>266</v>
+      </c>
+      <c r="P1" s="28" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q1" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="R1" s="28" t="s">
+        <v>224</v>
+      </c>
+      <c r="S1" s="28" t="s">
+        <v>225</v>
+      </c>
+      <c r="T1" s="28" t="s">
+        <v>226</v>
+      </c>
+      <c r="U1" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="V1" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="W1" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="X1" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="Y1" s="28" t="s">
         <v>268</v>
       </c>
-      <c r="D1" s="28" t="s">
-        <v>269</v>
-      </c>
-      <c r="E1" s="28" t="s">
-        <v>270</v>
-      </c>
-      <c r="F1" s="28" t="s">
-        <v>224</v>
-      </c>
-      <c r="G1" s="32" t="s">
-        <v>240</v>
-      </c>
-      <c r="H1" s="28" t="s">
+      <c r="Z1" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="AA1" s="28" t="s">
+        <v>229</v>
+      </c>
+      <c r="AB1" s="28" t="s">
+        <v>230</v>
+      </c>
+      <c r="AC1" s="28" t="s">
+        <v>254</v>
+      </c>
+      <c r="AD1" s="28" t="s">
+        <v>243</v>
+      </c>
+      <c r="AE1" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="AF1" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="AG1" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="AH1" s="28" t="s">
         <v>241</v>
       </c>
-      <c r="I1" s="28" t="s">
-        <v>225</v>
-      </c>
-      <c r="J1" s="28" t="s">
-        <v>226</v>
-      </c>
-      <c r="K1" s="28" t="s">
-        <v>227</v>
-      </c>
-      <c r="L1" s="28" t="s">
+      <c r="AI1" s="28" t="s">
+        <v>231</v>
+      </c>
+      <c r="AJ1" s="28" t="s">
         <v>242</v>
       </c>
-      <c r="M1" s="28" t="s">
-        <v>243</v>
-      </c>
-      <c r="N1" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="O1" s="28" t="s">
-        <v>271</v>
-      </c>
-      <c r="P1" s="28" t="s">
-        <v>272</v>
-      </c>
-      <c r="Q1" s="28" t="s">
-        <v>245</v>
-      </c>
-      <c r="R1" s="28" t="s">
-        <v>228</v>
-      </c>
-      <c r="S1" s="28" t="s">
-        <v>229</v>
-      </c>
-      <c r="T1" s="28" t="s">
-        <v>230</v>
-      </c>
-      <c r="U1" s="28" t="s">
-        <v>231</v>
-      </c>
-      <c r="V1" s="28" t="s">
-        <v>186</v>
-      </c>
-      <c r="W1" s="28" t="s">
-        <v>193</v>
-      </c>
-      <c r="X1" s="28" t="s">
-        <v>202</v>
-      </c>
-      <c r="Y1" s="28" t="s">
-        <v>273</v>
-      </c>
-      <c r="Z1" s="28" t="s">
+      <c r="AK1" s="28" t="s">
         <v>232</v>
       </c>
-      <c r="AA1" s="28" t="s">
-        <v>233</v>
-      </c>
-      <c r="AB1" s="28" t="s">
-        <v>234</v>
-      </c>
-      <c r="AC1" s="28" t="s">
-        <v>259</v>
-      </c>
-      <c r="AD1" s="28" t="s">
-        <v>248</v>
-      </c>
-      <c r="AE1" s="28" t="s">
-        <v>200</v>
-      </c>
-      <c r="AF1" s="28" t="s">
-        <v>170</v>
-      </c>
-      <c r="AG1" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="AH1" s="28" t="s">
-        <v>246</v>
-      </c>
-      <c r="AI1" s="28" t="s">
-        <v>235</v>
-      </c>
-      <c r="AJ1" s="28" t="s">
-        <v>247</v>
-      </c>
-      <c r="AK1" s="28" t="s">
-        <v>236</v>
-      </c>
       <c r="AL1" s="28" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AM1" s="28" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AN1" s="28" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="AO1" s="24" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
@@ -7096,19 +6762,19 @@
         <v>Q1</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C5" s="30"/>
       <c r="D5" s="30"/>
       <c r="E5" s="30"/>
       <c r="F5" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G5" s="31" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="H5" s="31" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="I5" s="31"/>
       <c r="J5" s="31"/>
@@ -7150,19 +6816,19 @@
         <v>Q2</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C6" s="30"/>
       <c r="D6" s="30"/>
       <c r="E6" s="30"/>
       <c r="F6" s="31" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="I6" s="31"/>
       <c r="J6" s="31"/>
@@ -7182,7 +6848,7 @@
       <c r="X6" s="25"/>
       <c r="Y6" s="25"/>
       <c r="Z6" s="25" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
@@ -7206,19 +6872,19 @@
         <v>Q3</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C7" s="30"/>
       <c r="D7" s="30"/>
       <c r="E7" s="30"/>
       <c r="F7" s="31" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="H7" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I7" s="31"/>
       <c r="J7" s="31"/>
@@ -7257,7 +6923,7 @@
       <c r="AM7" s="25"/>
       <c r="AN7" s="25"/>
       <c r="AO7" s="26" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.25">
@@ -7266,19 +6932,19 @@
         <v>Q3</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
       <c r="F8" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="H8" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I8" s="31"/>
       <c r="J8" s="31"/>
@@ -7286,7 +6952,7 @@
       <c r="L8" s="31"/>
       <c r="M8" s="31"/>
       <c r="N8" s="31" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="O8" s="25"/>
       <c r="P8" s="31"/>
@@ -7324,29 +6990,29 @@
         <v>Q3</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
       <c r="F9" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
       <c r="L9" s="31" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="M9" s="31"/>
       <c r="N9" s="31" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
@@ -7384,19 +7050,19 @@
         <v>Q3</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
       <c r="F10" s="31" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="H10" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="31"/>
@@ -7422,13 +7088,13 @@
       <c r="AB10" s="25"/>
       <c r="AC10" s="25"/>
       <c r="AD10" s="14" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="AE10" s="25"/>
       <c r="AF10" s="25"/>
       <c r="AG10" s="25"/>
       <c r="AH10" s="25" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="AI10" s="25"/>
       <c r="AJ10" s="25"/>
@@ -7444,19 +7110,19 @@
         <v>Q3</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
       <c r="F11" s="31" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="H11" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I11" s="31"/>
       <c r="J11" s="31"/>
@@ -7464,7 +7130,7 @@
       <c r="L11" s="31"/>
       <c r="M11" s="31"/>
       <c r="N11" s="31" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="O11" s="25"/>
       <c r="P11" s="31"/>
@@ -7488,7 +7154,7 @@
       <c r="AD11" s="14"/>
       <c r="AE11" s="25"/>
       <c r="AF11" s="25" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="AG11" s="25"/>
       <c r="AH11" s="25"/>
@@ -7506,19 +7172,19 @@
         <v>Q3</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
       <c r="E12" s="30"/>
       <c r="F12" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I12" s="31"/>
       <c r="J12" s="31"/>
@@ -7526,7 +7192,7 @@
       <c r="L12" s="31"/>
       <c r="M12" s="31"/>
       <c r="N12" s="31" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="O12" s="25"/>
       <c r="P12" s="31"/>
@@ -7548,7 +7214,7 @@
       <c r="AD12" s="14"/>
       <c r="AE12" s="25"/>
       <c r="AF12" s="25" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="AG12" s="25"/>
       <c r="AH12" s="25"/>
@@ -7566,31 +7232,31 @@
         <v>Q4</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
       <c r="F13" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I13" s="31"/>
       <c r="J13" s="31" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="K13" s="31" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="L13" s="31"/>
       <c r="M13" s="31"/>
       <c r="N13" s="31" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="O13" s="25"/>
       <c r="P13" s="31"/>
@@ -7628,19 +7294,19 @@
         <v>Q5</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="30"/>
       <c r="E14" s="30"/>
       <c r="F14" s="31" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
@@ -7651,10 +7317,10 @@
       <c r="O14" s="25"/>
       <c r="P14" s="31"/>
       <c r="Q14" s="31" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="R14" s="31" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="S14" s="31"/>
       <c r="T14" s="31"/>
@@ -7686,19 +7352,19 @@
         <v>Q5</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="C15" s="30"/>
       <c r="D15" s="30"/>
       <c r="E15" s="30"/>
       <c r="F15" s="31" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="I15" s="31"/>
       <c r="J15" s="31"/>
@@ -7709,10 +7375,10 @@
       <c r="O15" s="25"/>
       <c r="P15" s="31"/>
       <c r="Q15" s="31" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="R15" s="31" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="S15" s="25"/>
       <c r="T15" s="25"/>
@@ -7736,7 +7402,7 @@
       <c r="AL15" s="25"/>
       <c r="AM15" s="25"/>
       <c r="AN15" s="25" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="AO15" s="26"/>
     </row>
@@ -7746,19 +7412,19 @@
         <v>Q6</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="30"/>
       <c r="E16" s="30"/>
       <c r="F16" s="31" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="H16" s="31" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
@@ -7794,7 +7460,7 @@
       <c r="AJ16" s="25"/>
       <c r="AK16" s="25"/>
       <c r="AL16" s="31" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="AM16" s="25"/>
       <c r="AN16" s="25"/>
@@ -7806,26 +7472,26 @@
         <v>Q6</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
       <c r="E17" s="30"/>
       <c r="F17" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="I17" s="31"/>
       <c r="J17" s="31" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="K17" s="31" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="L17" s="31"/>
       <c r="M17" s="31"/>
@@ -7864,24 +7530,24 @@
         <v>Q9</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
       <c r="E18" s="30"/>
       <c r="F18" s="31"/>
       <c r="G18" s="31" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="I18" s="31"/>
       <c r="J18" s="31" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="K18" s="31" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="L18" s="31"/>
       <c r="M18" s="31"/>
@@ -7891,10 +7557,10 @@
       <c r="Q18" s="31"/>
       <c r="R18" s="31"/>
       <c r="S18" s="31" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="T18" s="31" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
@@ -7924,24 +7590,24 @@
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
       <c r="E19" s="30"/>
       <c r="F19" s="31"/>
       <c r="G19" s="31" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="I19" s="31"/>
       <c r="J19" s="31" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="K19" s="31" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="L19" s="31"/>
       <c r="M19" s="31"/>
@@ -7951,10 +7617,10 @@
       <c r="Q19" s="31"/>
       <c r="R19" s="31"/>
       <c r="S19" s="31" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="T19" s="31" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="U19" s="25"/>
       <c r="V19" s="25"/>
@@ -7984,26 +7650,26 @@
         <v>Q9</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
       <c r="E20" s="30"/>
       <c r="F20" s="31" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="I20" s="31"/>
       <c r="J20" s="31" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="K20" s="31" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="L20" s="31"/>
       <c r="M20" s="31"/>
@@ -8013,10 +7679,10 @@
       <c r="Q20" s="31"/>
       <c r="R20" s="31"/>
       <c r="S20" s="31" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="T20" s="31" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="U20" s="25"/>
       <c r="V20" s="25"/>
@@ -8046,16 +7712,16 @@
         <v>QNOT CHECKED: 2</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
       <c r="E21" s="30"/>
       <c r="F21" s="31" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="H21" s="31"/>
       <c r="I21" s="31"/>
@@ -8069,10 +7735,10 @@
       <c r="Q21" s="31"/>
       <c r="R21" s="31"/>
       <c r="S21" s="31" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="T21" s="31" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="U21" s="25"/>
       <c r="V21" s="25"/>
@@ -8080,7 +7746,7 @@
       <c r="X21" s="25"/>
       <c r="Y21" s="25"/>
       <c r="Z21" s="25" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="AA21" s="25"/>
       <c r="AB21" s="25"/>
@@ -8104,19 +7770,19 @@
         <v>Qmulti selvar with unguelt: 2</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
       <c r="F22" s="31" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -8129,10 +7795,10 @@
       <c r="Q22" s="31"/>
       <c r="R22" s="31"/>
       <c r="S22" s="31" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="T22" s="31" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="U22" s="25"/>
       <c r="V22" s="25"/>
@@ -8162,19 +7828,19 @@
         <v>Qtrigger invalid values: 2</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="E23" s="30"/>
       <c r="F23" s="31" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
@@ -8216,19 +7882,19 @@
         <v>QNOT CHECKED: 5</v>
       </c>
       <c r="B24" s="30" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
       <c r="E24" s="30"/>
       <c r="F24" s="31" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="H24" s="31" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="I24" s="31"/>
       <c r="J24" s="31"/>
@@ -8239,16 +7905,16 @@
       <c r="O24" s="25"/>
       <c r="P24" s="31"/>
       <c r="Q24" s="31" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="R24" s="31" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="S24" s="31" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="T24" s="31" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="U24" s="25"/>
       <c r="V24" s="25"/>
@@ -8278,41 +7944,41 @@
         <v>Q7</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="C25" s="30"/>
       <c r="D25" s="30"/>
       <c r="E25" s="30"/>
       <c r="F25" s="31" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="I25" s="31"/>
       <c r="J25" s="31" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="K25" s="31" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="L25" s="31"/>
       <c r="M25" s="31"/>
       <c r="N25" s="31" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="O25" s="25"/>
       <c r="P25" s="31"/>
       <c r="Q25" s="31"/>
       <c r="R25" s="31"/>
       <c r="S25" s="31" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="T25" s="31" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="U25" s="25"/>
       <c r="V25" s="25"/>
@@ -8332,7 +7998,7 @@
       <c r="AJ25" s="25"/>
       <c r="AK25" s="25"/>
       <c r="AL25" s="31" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="AM25" s="25"/>
       <c r="AN25" s="25"/>

</xml_diff>

<commit_message>
also allow the label strings in CatLab to be within double quotes instead of single quotes
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{207905FF-BB92-4BF3-B824-80175ED26BAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D69A94-9A0E-4A88-8BBE-7B257CE4E9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -1050,9 +1050,6 @@
     <t xml:space="preserve">(1 THRU 2 = 1) (3 THRU 5 = 2) (6 THRU HI = 3) </t>
   </si>
   <si>
-    <t xml:space="preserve">1 '1-2mal' 2 '3-5mal' 3 '&gt;5mal' </t>
-  </si>
-  <si>
     <t>S1E2M0</t>
   </si>
   <si>
@@ -1201,6 +1198,9 @@
   </si>
   <si>
     <t>-1,-3,-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 "1-2mal" 2 '3-5mal' 3 '&gt;5mal' </t>
   </si>
 </sst>
 </file>
@@ -2637,7 +2637,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B35" s="34">
         <v>-2</v>
@@ -3282,7 +3282,7 @@
     </row>
     <row r="6" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B6" s="20" t="s">
         <v>152</v>
@@ -3294,154 +3294,154 @@
         <v>154</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="M6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="N6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="O6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="P6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="Q6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="R6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="S6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="T6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="U6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="V6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="W6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="X6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="Y6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="Z6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AA6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AB6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AC6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AD6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AE6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AF6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AG6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AH6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AI6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AJ6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AK6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AL6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AM6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AN6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AO6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AP6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AQ6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AR6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AS6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AT6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AU6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AV6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AW6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AX6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AY6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AZ6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="BA6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="BB6" s="37" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="BD6" s="19"/>
     </row>
@@ -6632,7 +6632,7 @@
         <v>257</v>
       </c>
       <c r="AO1" s="24" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
@@ -6825,7 +6825,7 @@
         <v>248</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H6" s="31" t="s">
         <v>260</v>
@@ -6848,7 +6848,7 @@
       <c r="X6" s="25"/>
       <c r="Y6" s="25"/>
       <c r="Z6" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
@@ -6923,7 +6923,7 @@
       <c r="AM7" s="25"/>
       <c r="AN7" s="25"/>
       <c r="AO7" s="26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.25">
@@ -6941,7 +6941,7 @@
         <v>233</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H8" s="31" t="s">
         <v>262</v>
@@ -7008,11 +7008,11 @@
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
       <c r="L9" s="31" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="M9" s="31"/>
       <c r="N9" s="31" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O9" s="25"/>
       <c r="P9" s="31"/>
@@ -7059,7 +7059,7 @@
         <v>234</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="H10" s="31" t="s">
         <v>262</v>
@@ -7181,7 +7181,7 @@
         <v>233</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H12" s="31" t="s">
         <v>262</v>
@@ -7251,12 +7251,12 @@
         <v>279</v>
       </c>
       <c r="K13" s="31" t="s">
-        <v>280</v>
+        <v>330</v>
       </c>
       <c r="L13" s="31"/>
       <c r="M13" s="31"/>
       <c r="N13" s="31" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="O13" s="25"/>
       <c r="P13" s="31"/>
@@ -7306,7 +7306,7 @@
         <v>252</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
@@ -7320,7 +7320,7 @@
         <v>253</v>
       </c>
       <c r="R14" s="31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="S14" s="31"/>
       <c r="T14" s="31"/>
@@ -7378,7 +7378,7 @@
         <v>253</v>
       </c>
       <c r="R15" s="31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="S15" s="25"/>
       <c r="T15" s="25"/>
@@ -7402,7 +7402,7 @@
       <c r="AL15" s="25"/>
       <c r="AM15" s="25"/>
       <c r="AN15" s="25" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AO15" s="26"/>
     </row>
@@ -7412,7 +7412,7 @@
         <v>Q6</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="30"/>
@@ -7421,10 +7421,10 @@
         <v>234</v>
       </c>
       <c r="G16" s="31" t="s">
+        <v>288</v>
+      </c>
+      <c r="H16" s="31" t="s">
         <v>289</v>
-      </c>
-      <c r="H16" s="31" t="s">
-        <v>290</v>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
@@ -7460,7 +7460,7 @@
       <c r="AJ16" s="25"/>
       <c r="AK16" s="25"/>
       <c r="AL16" s="31" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AM16" s="25"/>
       <c r="AN16" s="25"/>
@@ -7472,7 +7472,7 @@
         <v>Q6</v>
       </c>
       <c r="B17" s="30" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -7481,17 +7481,17 @@
         <v>233</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I17" s="31"/>
       <c r="J17" s="31" t="s">
+        <v>295</v>
+      </c>
+      <c r="K17" s="31" t="s">
         <v>296</v>
-      </c>
-      <c r="K17" s="31" t="s">
-        <v>297</v>
       </c>
       <c r="L17" s="31"/>
       <c r="M17" s="31"/>
@@ -7530,24 +7530,24 @@
         <v>Q9</v>
       </c>
       <c r="B18" s="30" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
       <c r="E18" s="30"/>
       <c r="F18" s="31"/>
       <c r="G18" s="31" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H18" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I18" s="31"/>
       <c r="J18" s="31" t="s">
+        <v>298</v>
+      </c>
+      <c r="K18" s="31" t="s">
         <v>299</v>
-      </c>
-      <c r="K18" s="31" t="s">
-        <v>300</v>
       </c>
       <c r="L18" s="31"/>
       <c r="M18" s="31"/>
@@ -7557,10 +7557,10 @@
       <c r="Q18" s="31"/>
       <c r="R18" s="31"/>
       <c r="S18" s="31" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="T18" s="31" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="U18" s="25"/>
       <c r="V18" s="25"/>
@@ -7590,24 +7590,24 @@
         <v>Q9</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
       <c r="E19" s="30"/>
       <c r="F19" s="31"/>
       <c r="G19" s="31" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I19" s="31"/>
       <c r="J19" s="31" t="s">
+        <v>298</v>
+      </c>
+      <c r="K19" s="31" t="s">
         <v>299</v>
-      </c>
-      <c r="K19" s="31" t="s">
-        <v>300</v>
       </c>
       <c r="L19" s="31"/>
       <c r="M19" s="31"/>
@@ -7617,10 +7617,10 @@
       <c r="Q19" s="31"/>
       <c r="R19" s="31"/>
       <c r="S19" s="31" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="T19" s="31" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="U19" s="25"/>
       <c r="V19" s="25"/>
@@ -7650,7 +7650,7 @@
         <v>Q9</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -7659,17 +7659,17 @@
         <v>233</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I20" s="31"/>
       <c r="J20" s="31" t="s">
+        <v>298</v>
+      </c>
+      <c r="K20" s="31" t="s">
         <v>299</v>
-      </c>
-      <c r="K20" s="31" t="s">
-        <v>300</v>
       </c>
       <c r="L20" s="31"/>
       <c r="M20" s="31"/>
@@ -7679,10 +7679,10 @@
       <c r="Q20" s="31"/>
       <c r="R20" s="31"/>
       <c r="S20" s="31" t="s">
+        <v>302</v>
+      </c>
+      <c r="T20" s="31" t="s">
         <v>303</v>
-      </c>
-      <c r="T20" s="31" t="s">
-        <v>304</v>
       </c>
       <c r="U20" s="25"/>
       <c r="V20" s="25"/>
@@ -7712,7 +7712,7 @@
         <v>QNOT CHECKED: 2</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
@@ -7721,7 +7721,7 @@
         <v>248</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H21" s="31"/>
       <c r="I21" s="31"/>
@@ -7735,10 +7735,10 @@
       <c r="Q21" s="31"/>
       <c r="R21" s="31"/>
       <c r="S21" s="31" t="s">
+        <v>302</v>
+      </c>
+      <c r="T21" s="31" t="s">
         <v>303</v>
-      </c>
-      <c r="T21" s="31" t="s">
-        <v>304</v>
       </c>
       <c r="U21" s="25"/>
       <c r="V21" s="25"/>
@@ -7746,7 +7746,7 @@
       <c r="X21" s="25"/>
       <c r="Y21" s="25"/>
       <c r="Z21" s="25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AA21" s="25"/>
       <c r="AB21" s="25"/>
@@ -7770,7 +7770,7 @@
         <v>Qmulti selvar with unguelt: 2</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
@@ -7779,10 +7779,10 @@
         <v>248</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -7795,10 +7795,10 @@
       <c r="Q22" s="31"/>
       <c r="R22" s="31"/>
       <c r="S22" s="31" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="T22" s="31" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="U22" s="25"/>
       <c r="V22" s="25"/>
@@ -7828,7 +7828,7 @@
         <v>Qtrigger invalid values: 2</v>
       </c>
       <c r="B23" s="30" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
@@ -7837,10 +7837,10 @@
         <v>248</v>
       </c>
       <c r="G23" s="31" t="s">
+        <v>322</v>
+      </c>
+      <c r="H23" s="31" t="s">
         <v>323</v>
-      </c>
-      <c r="H23" s="31" t="s">
-        <v>324</v>
       </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
@@ -7882,7 +7882,7 @@
         <v>QNOT CHECKED: 5</v>
       </c>
       <c r="B24" s="30" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -7891,10 +7891,10 @@
         <v>251</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H24" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I24" s="31"/>
       <c r="J24" s="31"/>
@@ -7908,13 +7908,13 @@
         <v>253</v>
       </c>
       <c r="R24" s="31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="S24" s="31" t="s">
+        <v>302</v>
+      </c>
+      <c r="T24" s="31" t="s">
         <v>303</v>
-      </c>
-      <c r="T24" s="31" t="s">
-        <v>304</v>
       </c>
       <c r="U24" s="25"/>
       <c r="V24" s="25"/>
@@ -7944,7 +7944,7 @@
         <v>Q7</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C25" s="30"/>
       <c r="D25" s="30"/>
@@ -7953,32 +7953,32 @@
         <v>234</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I25" s="31"/>
       <c r="J25" s="31" t="s">
+        <v>312</v>
+      </c>
+      <c r="K25" s="31" t="s">
         <v>313</v>
-      </c>
-      <c r="K25" s="31" t="s">
-        <v>314</v>
       </c>
       <c r="L25" s="31"/>
       <c r="M25" s="31"/>
       <c r="N25" s="31" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O25" s="25"/>
       <c r="P25" s="31"/>
       <c r="Q25" s="31"/>
       <c r="R25" s="31"/>
       <c r="S25" s="31" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="T25" s="31" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="U25" s="25"/>
       <c r="V25" s="25"/>
@@ -7998,7 +7998,7 @@
       <c r="AJ25" s="25"/>
       <c r="AK25" s="25"/>
       <c r="AL25" s="31" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AM25" s="25"/>
       <c r="AN25" s="25"/>

</xml_diff>

<commit_message>
import content of named region cell V_BookNo from mapping
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88D69A94-9A0E-4A88-8BBE-7B257CE4E9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F5FDF6-9C0D-41B3-B591-1018A3404B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="R_miss_rec_val">Config!$B$35</definedName>
+    <definedName name="V_BookNo">Config!$B$11</definedName>
     <definedName name="V_Datum">Config!$B$18</definedName>
     <definedName name="V_ErrCountLog10">#REF!</definedName>
     <definedName name="V_ErrCountLog20">#REF!</definedName>
@@ -208,7 +209,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="332">
   <si>
     <t>Make script</t>
   </si>
@@ -1202,6 +1203,9 @@
   <si>
     <t xml:space="preserve">1 "1-2mal" 2 '3-5mal' 3 '&gt;5mal' </t>
   </si>
+  <si>
+    <t>V_BookNo</t>
+  </si>
 </sst>
 </file>
 
@@ -1447,13 +1451,13 @@
     <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="1" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2469,7 +2473,12 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B11" s="10"/>
+      <c r="A11" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B11" s="10">
+        <v>999999999</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
@@ -2901,8 +2910,8 @@
     </row>
     <row r="2" spans="1:56" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A3" s="35"/>
-      <c r="B3" s="36"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="37"/>
       <c r="E3" s="18">
         <v>1</v>
       </c>
@@ -3056,8 +3065,8 @@
       <c r="BD3" s="19"/>
     </row>
     <row r="4" spans="1:56" s="18" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="35"/>
-      <c r="B4" s="36"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="37"/>
       <c r="E4" s="18" t="s">
         <v>15</v>
       </c>
@@ -3293,154 +3302,154 @@
       <c r="D6" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="E6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="F6" s="37" t="s">
+      <c r="F6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="G6" s="37" t="s">
+      <c r="G6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="H6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="I6" s="37" t="s">
+      <c r="I6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="J6" s="37" t="s">
+      <c r="J6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="K6" s="37" t="s">
+      <c r="K6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="L6" s="37" t="s">
+      <c r="L6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="M6" s="37" t="s">
+      <c r="M6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="N6" s="37" t="s">
+      <c r="N6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="O6" s="37" t="s">
+      <c r="O6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="P6" s="37" t="s">
+      <c r="P6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="Q6" s="37" t="s">
+      <c r="Q6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="R6" s="37" t="s">
+      <c r="R6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="S6" s="37" t="s">
+      <c r="S6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="T6" s="37" t="s">
+      <c r="T6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="U6" s="37" t="s">
+      <c r="U6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="V6" s="37" t="s">
+      <c r="V6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="W6" s="37" t="s">
+      <c r="W6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="X6" s="37" t="s">
+      <c r="X6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="Y6" s="37" t="s">
+      <c r="Y6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="Z6" s="37" t="s">
+      <c r="Z6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AA6" s="37" t="s">
+      <c r="AA6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AB6" s="37" t="s">
+      <c r="AB6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AC6" s="37" t="s">
+      <c r="AC6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AD6" s="37" t="s">
+      <c r="AD6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AE6" s="37" t="s">
+      <c r="AE6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AF6" s="37" t="s">
+      <c r="AF6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AG6" s="37" t="s">
+      <c r="AG6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AH6" s="37" t="s">
+      <c r="AH6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AI6" s="37" t="s">
+      <c r="AI6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AJ6" s="37" t="s">
+      <c r="AJ6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AK6" s="37" t="s">
+      <c r="AK6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AL6" s="37" t="s">
+      <c r="AL6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AM6" s="37" t="s">
+      <c r="AM6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AN6" s="37" t="s">
+      <c r="AN6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AO6" s="37" t="s">
+      <c r="AO6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AP6" s="37" t="s">
+      <c r="AP6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AQ6" s="37" t="s">
+      <c r="AQ6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AR6" s="37" t="s">
+      <c r="AR6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AS6" s="37" t="s">
+      <c r="AS6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AT6" s="37" t="s">
+      <c r="AT6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AU6" s="37" t="s">
+      <c r="AU6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AV6" s="37" t="s">
+      <c r="AV6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AW6" s="37" t="s">
+      <c r="AW6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AX6" s="37" t="s">
+      <c r="AX6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AY6" s="37" t="s">
+      <c r="AY6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="AZ6" s="37" t="s">
+      <c r="AZ6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="BA6" s="37" t="s">
+      <c r="BA6" s="35" t="s">
         <v>329</v>
       </c>
-      <c r="BB6" s="37" t="s">
+      <c r="BB6" s="35" t="s">
         <v>329</v>
       </c>
       <c r="BD6" s="19"/>

</xml_diff>

<commit_message>
add TabCount to tab_table
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F5FDF6-9C0D-41B3-B591-1018A3404B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D983D936-FB90-46DD-945F-15ACF4CAC77F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -209,7 +209,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="353">
   <si>
     <t>Make script</t>
   </si>
@@ -1205,6 +1205,69 @@
   </si>
   <si>
     <t>V_BookNo</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3_1</t>
+  </si>
+  <si>
+    <t>Q3_2</t>
+  </si>
+  <si>
+    <t>Q3_3</t>
+  </si>
+  <si>
+    <t>Q3_4</t>
+  </si>
+  <si>
+    <t>Q3_5</t>
+  </si>
+  <si>
+    <t>Q3_6</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Q5_1</t>
+  </si>
+  <si>
+    <t>Q5_2</t>
+  </si>
+  <si>
+    <t>Q6_1</t>
+  </si>
+  <si>
+    <t>Q6_2</t>
+  </si>
+  <si>
+    <t>Q9_1</t>
+  </si>
+  <si>
+    <t>Q9_2</t>
+  </si>
+  <si>
+    <t>Q9_3</t>
+  </si>
+  <si>
+    <t>QNOT CHECKED: 2</t>
+  </si>
+  <si>
+    <t>Qmulti selvar with unguelt: 2</t>
+  </si>
+  <si>
+    <t>Qtrigger invalid values: 2</t>
+  </si>
+  <si>
+    <t>QNOT CHECKED: 5</t>
+  </si>
+  <si>
+    <t>Q7</t>
   </si>
 </sst>
 </file>
@@ -6766,9 +6829,8 @@
       <c r="AO4" s="26"/>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="str">
-        <f>"Q"&amp;LEFT(B5,FIND(".",B5)-1)</f>
-        <v>Q1</v>
+      <c r="A5" s="30" t="s">
+        <v>332</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>245</v>
@@ -6820,9 +6882,8 @@
       <c r="AO5" s="26"/>
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="str">
-        <f t="shared" ref="A6:A14" si="0">"Q"&amp;LEFT(B6,FIND(".",B6)-1)</f>
-        <v>Q2</v>
+      <c r="A6" s="30" t="s">
+        <v>333</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>247</v>
@@ -6876,9 +6937,8 @@
       <c r="AO6" s="26"/>
     </row>
     <row r="7" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q3</v>
+      <c r="A7" s="30" t="s">
+        <v>334</v>
       </c>
       <c r="B7" s="30" t="s">
         <v>249</v>
@@ -6936,9 +6996,8 @@
       </c>
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="str">
-        <f t="shared" ref="A8" si="1">"Q"&amp;LEFT(B8,FIND(".",B8)-1)</f>
-        <v>Q3</v>
+      <c r="A8" s="30" t="s">
+        <v>335</v>
       </c>
       <c r="B8" s="30" t="s">
         <v>249</v>
@@ -6994,9 +7053,8 @@
       <c r="AO8" s="26"/>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A9" s="30" t="str">
-        <f t="shared" ref="A9" si="2">"Q"&amp;LEFT(B9,FIND(".",B9)-1)</f>
-        <v>Q3</v>
+      <c r="A9" s="30" t="s">
+        <v>336</v>
       </c>
       <c r="B9" s="30" t="s">
         <v>249</v>
@@ -7054,9 +7112,8 @@
       <c r="AO9" s="26"/>
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A10" s="30" t="str">
-        <f t="shared" ref="A10" si="3">"Q"&amp;LEFT(B10,FIND(".",B10)-1)</f>
-        <v>Q3</v>
+      <c r="A10" s="30" t="s">
+        <v>337</v>
       </c>
       <c r="B10" s="30" t="s">
         <v>249</v>
@@ -7114,9 +7171,8 @@
       <c r="AO10" s="26"/>
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A11" s="30" t="str">
-        <f t="shared" ref="A11:A13" si="4">"Q"&amp;LEFT(B11,FIND(".",B11)-1)</f>
-        <v>Q3</v>
+      <c r="A11" s="30" t="s">
+        <v>338</v>
       </c>
       <c r="B11" s="30" t="s">
         <v>249</v>
@@ -7176,9 +7232,8 @@
       <c r="AO11" s="26"/>
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A12" s="30" t="str">
-        <f t="shared" ref="A12" si="5">"Q"&amp;LEFT(B12,FIND(".",B12)-1)</f>
-        <v>Q3</v>
+      <c r="A12" s="30" t="s">
+        <v>339</v>
       </c>
       <c r="B12" s="30" t="s">
         <v>249</v>
@@ -7236,9 +7291,8 @@
       <c r="AO12" s="26"/>
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A13" s="30" t="str">
-        <f t="shared" si="4"/>
-        <v>Q4</v>
+      <c r="A13" s="30" t="s">
+        <v>340</v>
       </c>
       <c r="B13" s="30" t="s">
         <v>277</v>
@@ -7298,9 +7352,8 @@
       <c r="AO13" s="26"/>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v>Q5</v>
+      <c r="A14" s="30" t="s">
+        <v>341</v>
       </c>
       <c r="B14" s="30" t="s">
         <v>250</v>
@@ -7356,9 +7409,8 @@
       <c r="AO14" s="26"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A15" s="30" t="str">
-        <f t="shared" ref="A15:A16" si="6">"Q"&amp;LEFT(B15,FIND(".",B15)-1)</f>
-        <v>Q5</v>
+      <c r="A15" s="30" t="s">
+        <v>342</v>
       </c>
       <c r="B15" s="30" t="s">
         <v>250</v>
@@ -7416,9 +7468,8 @@
       <c r="AO15" s="26"/>
     </row>
     <row r="16" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A16" s="30" t="str">
-        <f t="shared" si="6"/>
-        <v>Q6</v>
+      <c r="A16" s="30" t="s">
+        <v>343</v>
       </c>
       <c r="B16" s="30" t="s">
         <v>287</v>
@@ -7476,9 +7527,8 @@
       <c r="AO16" s="26"/>
     </row>
     <row r="17" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A17" s="30" t="str">
-        <f t="shared" ref="A17:A18" si="7">"Q"&amp;LEFT(B17,FIND(".",B17)-1)</f>
-        <v>Q6</v>
+      <c r="A17" s="30" t="s">
+        <v>344</v>
       </c>
       <c r="B17" s="30" t="s">
         <v>287</v>
@@ -7534,9 +7584,8 @@
       <c r="AO17" s="26"/>
     </row>
     <row r="18" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="str">
-        <f t="shared" si="7"/>
-        <v>Q9</v>
+      <c r="A18" s="30" t="s">
+        <v>345</v>
       </c>
       <c r="B18" s="30" t="s">
         <v>297</v>
@@ -7594,9 +7643,8 @@
       <c r="AO18" s="26"/>
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="str">
-        <f t="shared" ref="A19:A25" si="8">"Q"&amp;LEFT(B19,FIND(".",B19)-1)</f>
-        <v>Q9</v>
+      <c r="A19" s="30" t="s">
+        <v>346</v>
       </c>
       <c r="B19" s="30" t="s">
         <v>297</v>
@@ -7654,9 +7702,8 @@
       <c r="AO19" s="26"/>
     </row>
     <row r="20" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A20" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>Q9</v>
+      <c r="A20" s="30" t="s">
+        <v>347</v>
       </c>
       <c r="B20" s="30" t="s">
         <v>297</v>
@@ -7716,9 +7763,8 @@
       <c r="AO20" s="26"/>
     </row>
     <row r="21" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>QNOT CHECKED: 2</v>
+      <c r="A21" s="30" t="s">
+        <v>348</v>
       </c>
       <c r="B21" s="30" t="s">
         <v>309</v>
@@ -7774,9 +7820,8 @@
       <c r="AO21" s="26"/>
     </row>
     <row r="22" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A22" s="30" t="str">
-        <f t="shared" ref="A22" si="9">"Q"&amp;LEFT(B22,FIND(".",B22)-1)</f>
-        <v>Qmulti selvar with unguelt: 2</v>
+      <c r="A22" s="30" t="s">
+        <v>349</v>
       </c>
       <c r="B22" s="30" t="s">
         <v>319</v>
@@ -7832,9 +7877,8 @@
       <c r="AO22" s="26"/>
     </row>
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A23" s="30" t="str">
-        <f t="shared" ref="A23" si="10">"Q"&amp;LEFT(B23,FIND(".",B23)-1)</f>
-        <v>Qtrigger invalid values: 2</v>
+      <c r="A23" s="30" t="s">
+        <v>350</v>
       </c>
       <c r="B23" s="30" t="s">
         <v>321</v>
@@ -7886,9 +7930,8 @@
       <c r="AO23" s="26"/>
     </row>
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>QNOT CHECKED: 5</v>
+      <c r="A24" s="30" t="s">
+        <v>351</v>
       </c>
       <c r="B24" s="30" t="s">
         <v>310</v>
@@ -7948,9 +7991,8 @@
       <c r="AO24" s="26"/>
     </row>
     <row r="25" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="str">
-        <f t="shared" si="8"/>
-        <v>Q7</v>
+      <c r="A25" s="30" t="s">
+        <v>352</v>
       </c>
       <c r="B25" s="30" t="s">
         <v>311</v>

</xml_diff>

<commit_message>
only use 3 invalid values
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B372EDB-FDEF-4E6C-802E-3759EE851670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B7A5E8-E325-431A-B78F-9A17CE0F49FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="353">
   <si>
     <t>Make script</t>
   </si>
@@ -1254,6 +1254,9 @@
   </si>
   <si>
     <t>(0 THRU 50 = -2) (ELSE=COPY)</t>
+  </si>
+  <si>
+    <t>5, 99,-2</t>
   </si>
 </sst>
 </file>
@@ -7097,7 +7100,7 @@
         <v>300</v>
       </c>
       <c r="H14" s="29" t="s">
-        <v>301</v>
+        <v>352</v>
       </c>
       <c r="I14" s="29"/>
       <c r="J14" s="29"/>

</xml_diff>

<commit_message>
refactor calculation of Qtab$p$df_stat_fun: - also allow to specify `fun` instead of `shortcut` from df_metr_mac - allow to omit the precision and use the new column `decimals` in df_metr_mac if not specified - allow to pass multiple new columns, e.g. S1[label=hello][another column in df_stat_funs=value of the column in this row]
For the moment only one option is used:
- optionally change the label RowTitle1/2/3 stat_fun label of a function in a cat table by e.g. changingMetrMac = "S1" to S1[label=hallo] to use "hallo" here
- every name passed ("label" in the example above) will be available as a new column in Qtab$p$df_stat_funs
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B7A5E8-E325-431A-B78F-9A17CE0F49FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B312986-3756-41B7-99C5-1BD3F002C78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="354">
   <si>
     <t>Make script</t>
   </si>
@@ -1257,6 +1257,9 @@
   </si>
   <si>
     <t>5, 99,-2</t>
+  </si>
+  <si>
+    <t>S1[label=hello]E2M0P250T0I0A0</t>
   </si>
 </sst>
 </file>
@@ -6776,7 +6779,7 @@
       <c r="L8" s="29"/>
       <c r="M8" s="29"/>
       <c r="N8" s="29" t="s">
-        <v>279</v>
+        <v>353</v>
       </c>
       <c r="O8" s="29"/>
       <c r="P8" s="29"/>

</xml_diff>

<commit_message>
Allow to also use the notation of MetrMac in ZsfgMW. This adds the (optional) possibilities to: - alter the default RowDecimals (see df_metr_mac) of the MStatistics Rows with the number after the fun name/shortcut - change RowTitle3 of MStatistics rows with: ...[label=<put the label replacement here>] - change RowTitle3 of MValid rows with: ...[ValidN=<put the label replacement here>] - change RowDecimals of MValid rows with: ...[ValidDec=<put the label replacement here>]
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B312986-3756-41B7-99C5-1BD3F002C78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8CC780-8670-4043-B8EF-1A029DDEC846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1055,9 +1055,6 @@
     <t>q3a_NA q3b</t>
   </si>
   <si>
-    <t>median</t>
-  </si>
-  <si>
     <t>Summary of Medians</t>
   </si>
   <si>
@@ -1260,6 +1257,9 @@
   </si>
   <si>
     <t>S1[label=hello]E2M0P250T0I0A0</t>
+  </si>
+  <si>
+    <t>median3[label=hi][ValidN=how are you][ValidDec=2]</t>
   </si>
 </sst>
 </file>
@@ -3536,7 +3536,7 @@
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A11" s="24" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>173</v>
@@ -6779,7 +6779,7 @@
       <c r="L8" s="29"/>
       <c r="M8" s="29"/>
       <c r="N8" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="O8" s="29"/>
       <c r="P8" s="29"/>
@@ -6830,7 +6830,7 @@
       <c r="J9" s="29"/>
       <c r="K9" s="29"/>
       <c r="L9" s="29" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="M9" s="29"/>
       <c r="N9" s="29" t="s">
@@ -6903,13 +6903,13 @@
       <c r="AB10" s="29"/>
       <c r="AC10" s="29"/>
       <c r="AD10" s="17" t="s">
-        <v>285</v>
+        <v>353</v>
       </c>
       <c r="AE10" s="29"/>
       <c r="AF10" s="29"/>
       <c r="AG10" s="29"/>
       <c r="AH10" s="29" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AI10" s="29"/>
       <c r="AJ10" s="29"/>
@@ -6921,7 +6921,7 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B11" s="25" t="s">
         <v>273</v>
@@ -6964,7 +6964,7 @@
       <c r="AD11" s="17"/>
       <c r="AE11" s="29"/>
       <c r="AF11" s="29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AG11" s="29"/>
       <c r="AH11" s="29"/>
@@ -6978,7 +6978,7 @@
     </row>
     <row r="12" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B12" s="25" t="s">
         <v>273</v>
@@ -6988,7 +6988,7 @@
         <v>263</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H12" s="29"/>
       <c r="I12" s="29"/>
@@ -7019,7 +7019,7 @@
       <c r="AD12" s="17"/>
       <c r="AE12" s="29"/>
       <c r="AF12" s="29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="AG12" s="29"/>
       <c r="AH12" s="29"/>
@@ -7033,30 +7033,30 @@
     </row>
     <row r="13" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="B13" s="25" t="s">
         <v>291</v>
-      </c>
-      <c r="B13" s="25" t="s">
-        <v>292</v>
       </c>
       <c r="C13" s="25"/>
       <c r="F13" s="29" t="s">
         <v>263</v>
       </c>
       <c r="G13" s="29" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H13" s="29"/>
       <c r="I13" s="29"/>
       <c r="J13" s="29" t="s">
+        <v>293</v>
+      </c>
+      <c r="K13" s="29" t="s">
         <v>294</v>
-      </c>
-      <c r="K13" s="29" t="s">
-        <v>295</v>
       </c>
       <c r="L13" s="29"/>
       <c r="M13" s="29"/>
       <c r="N13" s="29" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="O13" s="29"/>
       <c r="P13" s="29"/>
@@ -7090,20 +7090,20 @@
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="B14" s="25" t="s">
         <v>297</v>
-      </c>
-      <c r="B14" s="25" t="s">
-        <v>298</v>
       </c>
       <c r="C14" s="25"/>
       <c r="F14" s="29" t="s">
+        <v>298</v>
+      </c>
+      <c r="G14" s="29" t="s">
         <v>299</v>
       </c>
-      <c r="G14" s="29" t="s">
-        <v>300</v>
-      </c>
       <c r="H14" s="29" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I14" s="29"/>
       <c r="J14" s="29"/>
@@ -7114,10 +7114,10 @@
       <c r="O14" s="29"/>
       <c r="P14" s="29"/>
       <c r="Q14" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="R14" s="29" t="s">
         <v>302</v>
-      </c>
-      <c r="R14" s="29" t="s">
-        <v>303</v>
       </c>
       <c r="S14" s="29"/>
       <c r="T14" s="29"/>
@@ -7145,17 +7145,17 @@
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C15" s="25"/>
       <c r="F15" s="29" t="s">
+        <v>298</v>
+      </c>
+      <c r="G15" s="29" t="s">
         <v>299</v>
-      </c>
-      <c r="G15" s="29" t="s">
-        <v>300</v>
       </c>
       <c r="H15" s="29" t="s">
         <v>265</v>
@@ -7169,10 +7169,10 @@
       <c r="O15" s="29"/>
       <c r="P15" s="29"/>
       <c r="Q15" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="R15" s="29" t="s">
         <v>302</v>
-      </c>
-      <c r="R15" s="29" t="s">
-        <v>303</v>
       </c>
       <c r="S15" s="29"/>
       <c r="T15" s="29"/>
@@ -7196,26 +7196,26 @@
       <c r="AL15" s="29"/>
       <c r="AM15" s="29"/>
       <c r="AN15" s="29" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="AO15" s="30"/>
     </row>
     <row r="16" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
+        <v>305</v>
+      </c>
+      <c r="B16" s="25" t="s">
         <v>306</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>307</v>
       </c>
       <c r="C16" s="25"/>
       <c r="F16" s="29" t="s">
         <v>274</v>
       </c>
       <c r="G16" s="29" t="s">
+        <v>307</v>
+      </c>
+      <c r="H16" s="29" t="s">
         <v>308</v>
-      </c>
-      <c r="H16" s="29" t="s">
-        <v>309</v>
       </c>
       <c r="I16" s="29"/>
       <c r="J16" s="29"/>
@@ -7251,7 +7251,7 @@
       <c r="AJ16" s="29"/>
       <c r="AK16" s="29"/>
       <c r="AL16" s="29" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="AM16" s="29"/>
       <c r="AN16" s="29"/>
@@ -7259,27 +7259,27 @@
     </row>
     <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C17" s="25"/>
       <c r="F17" s="29" t="s">
         <v>263</v>
       </c>
       <c r="G17" s="29" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H17" s="29" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I17" s="29"/>
       <c r="J17" s="29" t="s">
+        <v>312</v>
+      </c>
+      <c r="K17" s="29" t="s">
         <v>313</v>
-      </c>
-      <c r="K17" s="29" t="s">
-        <v>314</v>
       </c>
       <c r="L17" s="29"/>
       <c r="M17" s="29"/>
@@ -7314,25 +7314,25 @@
     </row>
     <row r="18" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="B18" s="25" t="s">
         <v>315</v>
-      </c>
-      <c r="B18" s="25" t="s">
-        <v>316</v>
       </c>
       <c r="C18" s="25"/>
       <c r="F18" s="29"/>
       <c r="G18" s="29" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H18" s="29" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I18" s="29"/>
       <c r="J18" s="29" t="s">
+        <v>317</v>
+      </c>
+      <c r="K18" s="29" t="s">
         <v>318</v>
-      </c>
-      <c r="K18" s="29" t="s">
-        <v>319</v>
       </c>
       <c r="L18" s="29"/>
       <c r="M18" s="29"/>
@@ -7342,10 +7342,10 @@
       <c r="Q18" s="29"/>
       <c r="R18" s="29"/>
       <c r="S18" s="29" t="s">
+        <v>319</v>
+      </c>
+      <c r="T18" s="29" t="s">
         <v>320</v>
-      </c>
-      <c r="T18" s="29" t="s">
-        <v>321</v>
       </c>
       <c r="U18" s="29"/>
       <c r="V18" s="29"/>
@@ -7371,25 +7371,25 @@
     </row>
     <row r="19" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C19" s="25"/>
       <c r="F19" s="29"/>
       <c r="G19" s="29" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H19" s="29" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I19" s="29"/>
       <c r="J19" s="29" t="s">
+        <v>317</v>
+      </c>
+      <c r="K19" s="29" t="s">
         <v>318</v>
-      </c>
-      <c r="K19" s="29" t="s">
-        <v>319</v>
       </c>
       <c r="L19" s="29"/>
       <c r="M19" s="29"/>
@@ -7399,10 +7399,10 @@
       <c r="Q19" s="29"/>
       <c r="R19" s="29"/>
       <c r="S19" s="29" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="T19" s="29" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="U19" s="29"/>
       <c r="V19" s="29"/>
@@ -7428,27 +7428,27 @@
     </row>
     <row r="20" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C20" s="25"/>
       <c r="F20" s="29" t="s">
         <v>263</v>
       </c>
       <c r="G20" s="29" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="H20" s="29" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I20" s="29"/>
       <c r="J20" s="29" t="s">
+        <v>317</v>
+      </c>
+      <c r="K20" s="29" t="s">
         <v>318</v>
-      </c>
-      <c r="K20" s="29" t="s">
-        <v>319</v>
       </c>
       <c r="L20" s="29"/>
       <c r="M20" s="29"/>
@@ -7458,10 +7458,10 @@
       <c r="Q20" s="29"/>
       <c r="R20" s="29"/>
       <c r="S20" s="29" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T20" s="29" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="U20" s="29"/>
       <c r="V20" s="29"/>
@@ -7487,17 +7487,17 @@
     </row>
     <row r="21" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A21" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="B21" s="25" t="s">
         <v>328</v>
-      </c>
-      <c r="B21" s="25" t="s">
-        <v>329</v>
       </c>
       <c r="C21" s="25"/>
       <c r="F21" s="29" t="s">
         <v>268</v>
       </c>
       <c r="G21" s="29" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="H21" s="29"/>
       <c r="I21" s="29"/>
@@ -7511,10 +7511,10 @@
       <c r="Q21" s="29"/>
       <c r="R21" s="29"/>
       <c r="S21" s="29" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T21" s="29" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="U21" s="29"/>
       <c r="V21" s="29"/>
@@ -7542,20 +7542,20 @@
     </row>
     <row r="22" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="B22" s="25" t="s">
         <v>331</v>
-      </c>
-      <c r="B22" s="25" t="s">
-        <v>332</v>
       </c>
       <c r="C22" s="25"/>
       <c r="F22" s="29" t="s">
         <v>268</v>
       </c>
       <c r="G22" s="29" t="s">
+        <v>332</v>
+      </c>
+      <c r="H22" s="29" t="s">
         <v>333</v>
-      </c>
-      <c r="H22" s="29" t="s">
-        <v>334</v>
       </c>
       <c r="I22" s="29"/>
       <c r="J22" s="29"/>
@@ -7568,10 +7568,10 @@
       <c r="Q22" s="29"/>
       <c r="R22" s="29"/>
       <c r="S22" s="29" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T22" s="29" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="U22" s="29"/>
       <c r="V22" s="29"/>
@@ -7597,20 +7597,20 @@
     </row>
     <row r="23" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="B23" s="25" t="s">
         <v>336</v>
-      </c>
-      <c r="B23" s="25" t="s">
-        <v>337</v>
       </c>
       <c r="C23" s="25"/>
       <c r="F23" s="29" t="s">
         <v>268</v>
       </c>
       <c r="G23" s="29" t="s">
+        <v>337</v>
+      </c>
+      <c r="H23" s="29" t="s">
         <v>338</v>
-      </c>
-      <c r="H23" s="29" t="s">
-        <v>339</v>
       </c>
       <c r="I23" s="29"/>
       <c r="J23" s="29"/>
@@ -7648,20 +7648,20 @@
     </row>
     <row r="24" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A24" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="B24" s="25" t="s">
         <v>340</v>
-      </c>
-      <c r="B24" s="25" t="s">
-        <v>341</v>
       </c>
       <c r="C24" s="25"/>
       <c r="F24" s="29" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G24" s="29" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H24" s="29" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I24" s="29"/>
       <c r="J24" s="29"/>
@@ -7672,16 +7672,16 @@
       <c r="O24" s="29"/>
       <c r="P24" s="29"/>
       <c r="Q24" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="R24" s="29" t="s">
         <v>302</v>
       </c>
-      <c r="R24" s="29" t="s">
-        <v>303</v>
-      </c>
       <c r="S24" s="29" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T24" s="29" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="U24" s="29"/>
       <c r="V24" s="29"/>
@@ -7707,27 +7707,27 @@
     </row>
     <row r="25" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="B25" s="25" t="s">
         <v>343</v>
-      </c>
-      <c r="B25" s="25" t="s">
-        <v>344</v>
       </c>
       <c r="C25" s="25"/>
       <c r="F25" s="29" t="s">
         <v>274</v>
       </c>
       <c r="G25" s="29" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H25" s="29" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I25" s="29"/>
       <c r="J25" s="29" t="s">
+        <v>345</v>
+      </c>
+      <c r="K25" s="29" t="s">
         <v>346</v>
-      </c>
-      <c r="K25" s="29" t="s">
-        <v>347</v>
       </c>
       <c r="L25" s="29"/>
       <c r="M25" s="29"/>
@@ -7739,10 +7739,10 @@
       <c r="Q25" s="29"/>
       <c r="R25" s="29"/>
       <c r="S25" s="29" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="T25" s="29" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="U25" s="29"/>
       <c r="V25" s="29"/>
@@ -7762,7 +7762,7 @@
       <c r="AJ25" s="29"/>
       <c r="AK25" s="29"/>
       <c r="AL25" s="29" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AM25" s="29"/>
       <c r="AN25" s="29"/>

</xml_diff>

<commit_message>
also use catrec Syntax to allow to specify sets of intervals/values in SelVal (in contrast to the other CatRec we must not use spaces in the SelVal intervals to make it work with the traditional SelVal syntax)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8CC780-8670-4043-B8EF-1A029DDEC846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52E252B-8DB4-4B95-9B9F-F260701B4F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="355">
   <si>
     <t>Make script</t>
   </si>
@@ -1260,6 +1260,9 @@
   </si>
   <si>
     <t>median3[label=hi][ValidN=how are you][ValidDec=2]</t>
+  </si>
+  <si>
+    <t>1 2 3-4,5,6:Sonstige</t>
   </si>
 </sst>
 </file>
@@ -7681,7 +7684,7 @@
         <v>326</v>
       </c>
       <c r="T24" s="29" t="s">
-        <v>320</v>
+        <v>354</v>
       </c>
       <c r="U24" s="29"/>
       <c r="V24" s="29"/>

</xml_diff>

<commit_message>
refactor filtering: - the global filter is now applied to filter Tabula$dat_mod to generate the new Tabula$dat_tab field which will be used instead of dat_mod - add a new row to the Questions sheet with a filtered question
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_neu_reduced.xlsx
+++ b/tests/testthat/excel/mapping_neu_reduced.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\crosstabser\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52E252B-8DB4-4B95-9B9F-F260701B4F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45459D3B-5B4A-47A3-B2A3-25A5D5597687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -198,7 +198,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="357">
   <si>
     <t>Make script</t>
   </si>
@@ -1263,6 +1263,12 @@
   </si>
   <si>
     <t>1 2 3-4,5,6:Sonstige</t>
+  </si>
+  <si>
+    <t>q2_01 != 1 &amp; q2_03 != 1</t>
+  </si>
+  <si>
+    <t>1 (mit Filter). Wie viele Mitarbeiter beschäftigt Ihr Unternehmen?</t>
   </si>
 </sst>
 </file>
@@ -1483,7 +1489,27 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="24">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2543,22 +2569,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H5">
-    <cfRule type="expression" dxfId="21" priority="2">
+    <cfRule type="expression" dxfId="23" priority="2">
       <formula>H5&lt;H3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="20" priority="3">
+    <cfRule type="expression" dxfId="22" priority="3">
       <formula>H7&lt;H5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9">
-    <cfRule type="expression" dxfId="19" priority="4">
+    <cfRule type="expression" dxfId="21" priority="4">
       <formula>H9&lt;H7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G8">
-    <cfRule type="cellIs" dxfId="18" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7772,11 +7798,25 @@
       <c r="AO25" s="30"/>
     </row>
     <row r="26" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A26" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>356</v>
+      </c>
       <c r="C26" s="25"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="29"/>
+      <c r="F26" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="G26" s="29" t="s">
+        <v>264</v>
+      </c>
+      <c r="H26" s="29" t="s">
+        <v>265</v>
+      </c>
+      <c r="I26" s="29" t="s">
+        <v>355</v>
+      </c>
       <c r="J26" s="29"/>
       <c r="K26" s="29"/>
       <c r="L26" s="29"/>
@@ -33123,42 +33163,46 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A25">
-    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24">
-    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A23">
-    <cfRule type="duplicateValues" dxfId="13" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20">
-    <cfRule type="duplicateValues" dxfId="11" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A18:A19">
-    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A17">
-    <cfRule type="duplicateValues" dxfId="7" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
-    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="3" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="18"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A26:A1048576 A2:A4">
-    <cfRule type="duplicateValues" dxfId="2" priority="17"/>
+  <conditionalFormatting sqref="A27:A1048576 A2:A4">
+    <cfRule type="duplicateValues" dxfId="4" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A14:A15 A5:A12">
-    <cfRule type="duplicateValues" dxfId="1" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="21"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A26">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>